<commit_message>
Corregge ticker Yahoo Finance per altri 49 ETF trovati per ISIN
Ricerca automatica tramite Yahoo Finance search API per ISIN.
Molti ETF Amundi su .MI rimappati verso .PA (Euronext Paris),
.DE (XETRA), .L (LSE), .AS (Amsterdam), .SW (Zurigo).

Rimangono 13 ETF senza ticker valido (probabilmente delistati):
SCIT, WSRE, EMUP(x2), ITAP, ABCK, EXMU, D50E, X1GA(1), CPBD,
SMRT, AIIA, IEUS.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -584,7 +584,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -642,7 +642,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -874,7 +874,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -932,7 +932,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ENRJ.MI</t>
+          <t>ENRG.PA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1063,7 +1063,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CECE.MI</t>
+          <t>CEC.PA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1232,8 +1232,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
-        <v>1</v>
+      <c r="A14" s="5" t="n">
+        <v>3</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1256,31 +1256,31 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>104.78</v>
+        <v>257.975</v>
       </c>
       <c r="H14" t="n">
-        <v>104.042</v>
+        <v>253.3442</v>
       </c>
       <c r="I14" t="n">
-        <v>102.4304</v>
+        <v>230.3964</v>
       </c>
       <c r="J14" t="n">
-        <v>57.2</v>
+        <v>53.4</v>
       </c>
       <c r="K14" t="n">
-        <v>25.6</v>
+        <v>7.3</v>
       </c>
       <c r="L14" t="n">
-        <v>0.1625</v>
-      </c>
-      <c r="M14" s="1" t="inlineStr">
-        <is>
-          <t>L1 BUY (5/5)</t>
+        <v>-2.4656</v>
+      </c>
+      <c r="M14" s="6" t="inlineStr">
+        <is>
+          <t>L3</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -1411,7 +1411,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PAFR.MI</t>
+          <t>LAFRI.MI</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -1570,7 +1570,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -1604,22 +1604,22 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>6.79</v>
+        <v>7.419</v>
       </c>
       <c r="H20" t="n">
-        <v>6.6095</v>
+        <v>7.3129</v>
       </c>
       <c r="I20" t="n">
-        <v>6.6312</v>
+        <v>6.9057</v>
       </c>
       <c r="J20" t="n">
-        <v>62.4</v>
+        <v>57.1</v>
       </c>
       <c r="K20" t="n">
-        <v>18.2</v>
+        <v>30.5</v>
       </c>
       <c r="L20" t="n">
-        <v>0.0515</v>
+        <v>-0.0317</v>
       </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
@@ -1628,7 +1628,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -1686,7 +1686,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>EMQA.MI</t>
+          <t>EGEE.DE</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -1836,22 +1836,22 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>65.33</v>
+        <v>5963.5</v>
       </c>
       <c r="H24" t="n">
-        <v>63.9134</v>
+        <v>5799.7546</v>
       </c>
       <c r="I24" t="n">
-        <v>63.9156</v>
+        <v>4758.1534</v>
       </c>
       <c r="J24" t="n">
-        <v>61.7</v>
+        <v>54.4</v>
       </c>
       <c r="K24" t="n">
-        <v>18.8</v>
+        <v>10.3</v>
       </c>
       <c r="L24" t="n">
-        <v>0.4318</v>
+        <v>-97.5719</v>
       </c>
       <c r="M24" s="4" t="inlineStr">
         <is>
@@ -1860,7 +1860,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>AMJP.MI</t>
+          <t>CJ1.PA</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1918,7 +1918,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -1928,8 +1928,8 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="n">
-        <v>3</v>
+      <c r="A26" s="1" t="n">
+        <v>2</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1969,14 +1969,14 @@
       <c r="L26" t="n">
         <v>0.2534</v>
       </c>
-      <c r="M26" s="6" t="inlineStr">
-        <is>
-          <t>L3</t>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t>L2 WATCH</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
@@ -2092,7 +2092,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
@@ -2107,7 +2107,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>AAUS.MI</t>
+          <t>LYPU.DE</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2150,7 +2150,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
@@ -2184,22 +2184,22 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>436.16</v>
+        <v>2479.5</v>
       </c>
       <c r="H30" t="n">
-        <v>423.9476</v>
+        <v>2398.2214</v>
       </c>
       <c r="I30" t="n">
-        <v>423.7632</v>
+        <v>2081.951</v>
       </c>
       <c r="J30" t="n">
-        <v>71</v>
+        <v>57.1</v>
       </c>
       <c r="K30" t="n">
-        <v>24.9</v>
+        <v>11.9</v>
       </c>
       <c r="L30" t="n">
-        <v>2.3344</v>
+        <v>-19.8327</v>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -2281,7 +2281,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>SD3E.MI</t>
+          <t>SEL.PA</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
@@ -2382,7 +2382,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -2397,7 +2397,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>EAEJ.MI</t>
+          <t>AZEH.DE</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2440,7 +2440,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>AWAT.MI</t>
+          <t>WATC.SW</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2498,7 +2498,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
@@ -2513,7 +2513,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>AWAT.MI</t>
+          <t>WAT.PA</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
@@ -2706,22 +2706,22 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>63.76</v>
+        <v>2161.75</v>
       </c>
       <c r="H39" t="n">
-        <v>62.3375</v>
+        <v>2070.7854</v>
       </c>
       <c r="I39" t="n">
-        <v>62.345</v>
+        <v>1663.2564</v>
       </c>
       <c r="J39" t="n">
-        <v>62.1</v>
+        <v>55.8</v>
       </c>
       <c r="K39" t="n">
-        <v>19</v>
+        <v>12.3</v>
       </c>
       <c r="L39" t="n">
-        <v>0.426</v>
+        <v>-34.4316</v>
       </c>
       <c r="M39" s="4" t="inlineStr">
         <is>
@@ -2730,7 +2730,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
@@ -2740,8 +2740,8 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
-        <v>2</v>
+      <c r="A40" s="5" t="n">
+        <v>3</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -2764,31 +2764,31 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>66.59999999999999</v>
+        <v>4.318</v>
       </c>
       <c r="H40" t="n">
-        <v>65.20740000000001</v>
+        <v>6.0109</v>
       </c>
       <c r="I40" t="n">
-        <v>65.3232</v>
+        <v>15.1466</v>
       </c>
       <c r="J40" t="n">
-        <v>61.3</v>
+        <v>45.4</v>
       </c>
       <c r="K40" t="n">
-        <v>18.7</v>
+        <v>9.5</v>
       </c>
       <c r="L40" t="n">
-        <v>0.442</v>
-      </c>
-      <c r="M40" s="4" t="inlineStr">
-        <is>
-          <t>L2 WATCH</t>
+        <v>0.7793</v>
+      </c>
+      <c r="M40" s="6" t="inlineStr">
+        <is>
+          <t>L3</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
@@ -2846,7 +2846,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
@@ -2904,7 +2904,7 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
@@ -2962,7 +2962,7 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
@@ -2996,22 +2996,22 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>176.74</v>
+        <v>442.4755</v>
       </c>
       <c r="H44" t="n">
-        <v>172.7139</v>
+        <v>427.4077</v>
       </c>
       <c r="I44" t="n">
-        <v>170.5344</v>
+        <v>378.4935</v>
       </c>
       <c r="J44" t="n">
-        <v>70.8</v>
+        <v>55.7</v>
       </c>
       <c r="K44" t="n">
-        <v>30.2</v>
+        <v>9.6</v>
       </c>
       <c r="L44" t="n">
-        <v>0.8333</v>
+        <v>-3.0072</v>
       </c>
       <c r="M44" s="4" t="inlineStr">
         <is>
@@ -3020,7 +3020,7 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
@@ -3146,8 +3146,8 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="n">
-        <v>3</v>
+      <c r="A47" s="1" t="n">
+        <v>2</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -3187,14 +3187,14 @@
       <c r="L47" t="n">
         <v>-0.955</v>
       </c>
-      <c r="M47" s="6" t="inlineStr">
-        <is>
-          <t>L3</t>
+      <c r="M47" s="4" t="inlineStr">
+        <is>
+          <t>L2 WATCH</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
@@ -3209,7 +3209,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PREU.MI</t>
+          <t>LWCE.PA</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3252,7 +3252,7 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
@@ -3310,7 +3310,7 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
@@ -3368,7 +3368,7 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
@@ -3426,7 +3426,7 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>EAEU.MI</t>
+          <t>EUEE.DE</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3484,7 +3484,7 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
@@ -3542,7 +3542,7 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
@@ -3658,7 +3658,7 @@
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
@@ -3673,7 +3673,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>UIMU.MI</t>
+          <t>MFDD.MI</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -3716,7 +3716,7 @@
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
@@ -3731,7 +3731,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>QFEU.MI</t>
+          <t>QCEU.PA</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3774,7 +3774,7 @@
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O57" t="inlineStr">
@@ -3832,7 +3832,7 @@
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O58" t="inlineStr">
@@ -3847,7 +3847,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>MBES.MI</t>
+          <t>FMI.MI</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3890,7 +3890,7 @@
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
@@ -3948,7 +3948,7 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O60" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
@@ -4021,7 +4021,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>PAZE.MI</t>
+          <t>EPAB.PA</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O62" t="inlineStr">
@@ -4079,7 +4079,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MEMU.MI</t>
+          <t>CMU.PA</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -4122,7 +4122,7 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O63" t="inlineStr">
@@ -4132,8 +4132,8 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
-        <v>2</v>
+      <c r="A64" s="5" t="n">
+        <v>3</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -4156,31 +4156,31 @@
         </is>
       </c>
       <c r="G64" t="n">
-        <v>411.58</v>
+        <v>237.2</v>
       </c>
       <c r="H64" t="n">
-        <v>409.1595</v>
+        <v>238.5414</v>
       </c>
       <c r="I64" t="n">
-        <v>410.6092</v>
+        <v>266.4454</v>
       </c>
       <c r="J64" t="n">
-        <v>55.1</v>
+        <v>47.7</v>
       </c>
       <c r="K64" t="n">
-        <v>17.9</v>
+        <v>8.4</v>
       </c>
       <c r="L64" t="n">
-        <v>1.2223</v>
-      </c>
-      <c r="M64" s="4" t="inlineStr">
-        <is>
-          <t>L2 WATCH</t>
+        <v>2.8977</v>
+      </c>
+      <c r="M64" s="6" t="inlineStr">
+        <is>
+          <t>L3</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
@@ -4238,7 +4238,7 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
@@ -4248,8 +4248,8 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
-        <v>1</v>
+      <c r="A66" s="5" t="n">
+        <v>3</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -4272,31 +4272,31 @@
         </is>
       </c>
       <c r="G66" t="n">
-        <v>4.85</v>
+        <v>4.3305</v>
       </c>
       <c r="H66" t="n">
-        <v>4.8027</v>
+        <v>4.2799</v>
       </c>
       <c r="I66" t="n">
-        <v>4.8002</v>
+        <v>4.2752</v>
       </c>
       <c r="J66" t="n">
-        <v>64.59999999999999</v>
+        <v>54.5</v>
       </c>
       <c r="K66" t="n">
-        <v>24.5</v>
+        <v>6.1</v>
       </c>
       <c r="L66" t="n">
-        <v>0.0124</v>
-      </c>
-      <c r="M66" s="1" t="inlineStr">
-        <is>
-          <t>L1 BUY (5/5)</t>
+        <v>0.0139</v>
+      </c>
+      <c r="M66" s="6" t="inlineStr">
+        <is>
+          <t>L3</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O66" t="inlineStr">
@@ -4330,22 +4330,22 @@
         </is>
       </c>
       <c r="G67" t="n">
-        <v>203.58</v>
+        <v>354.35</v>
       </c>
       <c r="H67" t="n">
-        <v>198.4826</v>
+        <v>343.7271</v>
       </c>
       <c r="I67" t="n">
-        <v>199.0398</v>
+        <v>313.427</v>
       </c>
       <c r="J67" t="n">
-        <v>63.7</v>
+        <v>55.7</v>
       </c>
       <c r="K67" t="n">
-        <v>23.3</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="L67" t="n">
-        <v>1.3773</v>
+        <v>-1.9145</v>
       </c>
       <c r="M67" s="4" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O67" t="inlineStr">
@@ -4412,7 +4412,7 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O68" t="inlineStr">
@@ -4470,7 +4470,7 @@
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
@@ -4528,7 +4528,7 @@
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O70" t="inlineStr">
@@ -4586,7 +4586,7 @@
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O71" t="inlineStr">
@@ -4644,7 +4644,7 @@
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O72" t="inlineStr">
@@ -4702,7 +4702,7 @@
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O73" t="inlineStr">
@@ -4760,7 +4760,7 @@
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O74" t="inlineStr">
@@ -4818,7 +4818,7 @@
       </c>
       <c r="N75" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O75" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O76" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
@@ -4968,22 +4968,22 @@
         </is>
       </c>
       <c r="G78" t="n">
-        <v>5.15</v>
+        <v>12</v>
       </c>
       <c r="H78" t="n">
-        <v>5.1391</v>
+        <v>12.1352</v>
       </c>
       <c r="I78" t="n">
-        <v>5.1558</v>
+        <v>11.0472</v>
       </c>
       <c r="J78" t="n">
-        <v>53.8</v>
+        <v>50.2</v>
       </c>
       <c r="K78" t="n">
-        <v>22</v>
+        <v>6.8</v>
       </c>
       <c r="L78" t="n">
-        <v>0.0051</v>
+        <v>-0.0963</v>
       </c>
       <c r="M78" s="4" t="inlineStr">
         <is>
@@ -4992,7 +4992,7 @@
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O78" t="inlineStr">
@@ -5026,22 +5026,22 @@
         </is>
       </c>
       <c r="G79" t="n">
-        <v>5.47</v>
+        <v>2828</v>
       </c>
       <c r="H79" t="n">
-        <v>5.4141</v>
+        <v>2753.1811</v>
       </c>
       <c r="I79" t="n">
-        <v>5.4432</v>
+        <v>2352.7483</v>
       </c>
       <c r="J79" t="n">
-        <v>59</v>
+        <v>55.4</v>
       </c>
       <c r="K79" t="n">
-        <v>18</v>
+        <v>10.3</v>
       </c>
       <c r="L79" t="n">
-        <v>0.0193</v>
+        <v>-31.1544</v>
       </c>
       <c r="M79" s="4" t="inlineStr">
         <is>
@@ -5050,7 +5050,7 @@
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O79" t="inlineStr">
@@ -5108,7 +5108,7 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>WENA.MI</t>
+          <t>WOEE.AS</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -5166,7 +5166,7 @@
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O81" t="inlineStr">
@@ -5200,22 +5200,22 @@
         </is>
       </c>
       <c r="G82" t="n">
-        <v>0.77</v>
+        <v>3.11</v>
       </c>
       <c r="H82" t="n">
-        <v>0.8127</v>
+        <v>2.8871</v>
       </c>
       <c r="I82" t="n">
-        <v>0.8102</v>
+        <v>2.2077</v>
       </c>
       <c r="J82" t="n">
-        <v>36.3</v>
+        <v>56.5</v>
       </c>
       <c r="K82" t="n">
-        <v>18</v>
+        <v>16.8</v>
       </c>
       <c r="L82" t="n">
-        <v>-0.0109</v>
+        <v>-0.0269</v>
       </c>
       <c r="M82" s="4" t="inlineStr">
         <is>
@@ -5224,7 +5224,7 @@
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O82" t="inlineStr">
@@ -5282,7 +5282,7 @@
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O83" t="inlineStr">
@@ -5340,7 +5340,7 @@
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O84" t="inlineStr">
@@ -5398,7 +5398,7 @@
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O85" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="N86" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O86" t="inlineStr">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O87" t="inlineStr">
@@ -5529,7 +5529,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>EXEM.MI</t>
+          <t>WEXU.DE</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -5572,7 +5572,7 @@
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O88" t="inlineStr">
@@ -5630,7 +5630,7 @@
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O89" t="inlineStr">
@@ -5688,7 +5688,7 @@
       </c>
       <c r="N90" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O90" t="inlineStr">
@@ -5746,7 +5746,7 @@
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O91" t="inlineStr">
@@ -5804,7 +5804,7 @@
       </c>
       <c r="N92" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O92" t="inlineStr">
@@ -5862,7 +5862,7 @@
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O93" t="inlineStr">
@@ -5920,7 +5920,7 @@
       </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O94" t="inlineStr">
@@ -5978,7 +5978,7 @@
       </c>
       <c r="N95" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O95" t="inlineStr">
@@ -5993,7 +5993,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>EAEG.MI</t>
+          <t>EGRI.PA</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -6036,7 +6036,7 @@
       </c>
       <c r="N96" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O96" t="inlineStr">
@@ -6094,7 +6094,7 @@
       </c>
       <c r="N97" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O97" t="inlineStr">
@@ -6152,7 +6152,7 @@
       </c>
       <c r="N98" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O98" t="inlineStr">
@@ -6210,7 +6210,7 @@
       </c>
       <c r="N99" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O99" t="inlineStr">
@@ -6225,7 +6225,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>AFHY.MI</t>
+          <t>AHYE.PA</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -6268,7 +6268,7 @@
       </c>
       <c r="N100" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O100" t="inlineStr">
@@ -6326,7 +6326,7 @@
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O101" t="inlineStr">
@@ -6384,7 +6384,7 @@
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O102" t="inlineStr">
@@ -6442,7 +6442,7 @@
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O103" t="inlineStr">
@@ -6457,7 +6457,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>GGRN.MI</t>
+          <t>CB3.PA</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -6500,7 +6500,7 @@
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O104" t="inlineStr">
@@ -6558,7 +6558,7 @@
       </c>
       <c r="N105" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O105" t="inlineStr">
@@ -6616,7 +6616,7 @@
       </c>
       <c r="N106" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O106" t="inlineStr">
@@ -6631,7 +6631,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>ECBX.MI</t>
+          <t>CBEF.MI</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -6674,7 +6674,7 @@
       </c>
       <c r="N107" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O107" t="inlineStr">
@@ -6708,22 +6708,22 @@
         </is>
       </c>
       <c r="G108" t="n">
-        <v>21.15</v>
+        <v>5.0855</v>
       </c>
       <c r="H108" t="n">
-        <v>21.1723</v>
+        <v>5.5709</v>
       </c>
       <c r="I108" t="n">
-        <v>21.1848</v>
+        <v>8.2729</v>
       </c>
       <c r="J108" t="n">
-        <v>47.6</v>
+        <v>45.5</v>
       </c>
       <c r="K108" t="n">
-        <v>14.4</v>
+        <v>9.4</v>
       </c>
       <c r="L108" t="n">
-        <v>-0.0016</v>
+        <v>0.2116</v>
       </c>
       <c r="M108" s="6" t="inlineStr">
         <is>
@@ -6732,7 +6732,7 @@
       </c>
       <c r="N108" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O108" t="inlineStr">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="N109" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O109" t="inlineStr">
@@ -6848,7 +6848,7 @@
       </c>
       <c r="N110" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O110" t="inlineStr">
@@ -6906,7 +6906,7 @@
       </c>
       <c r="N111" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O111" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="N112" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O112" t="inlineStr">
@@ -7022,7 +7022,7 @@
       </c>
       <c r="N113" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O113" t="inlineStr">
@@ -7037,7 +7037,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>WENA.MI</t>
+          <t>WOEH.MI</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -7080,7 +7080,7 @@
       </c>
       <c r="N114" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O114" t="inlineStr">
@@ -7138,7 +7138,7 @@
       </c>
       <c r="N115" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O115" t="inlineStr">
@@ -7153,7 +7153,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>BTP1.MI</t>
+          <t>BTP13.MI</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -7196,7 +7196,7 @@
       </c>
       <c r="N116" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O116" t="inlineStr">
@@ -7211,7 +7211,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>X1GA.MI</t>
+          <t>MA35.PA</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -7254,7 +7254,7 @@
       </c>
       <c r="N117" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O117" t="inlineStr">
@@ -7269,7 +7269,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>X1GA.MI</t>
+          <t>AM3A.PA</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="N118" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O118" t="inlineStr">
@@ -7327,7 +7327,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>UFRH.MI</t>
+          <t>AFRN.PA</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -7370,7 +7370,7 @@
       </c>
       <c r="N119" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O119" t="inlineStr">
@@ -7380,8 +7380,8 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="1" t="n">
-        <v>2</v>
+      <c r="A120" s="5" t="n">
+        <v>3</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -7404,31 +7404,31 @@
         </is>
       </c>
       <c r="G120" t="n">
-        <v>5.07</v>
+        <v>5.0283</v>
       </c>
       <c r="H120" t="n">
-        <v>5.0675</v>
+        <v>5.0295</v>
       </c>
       <c r="I120" t="n">
-        <v>5.0628</v>
+        <v>5.0358</v>
       </c>
       <c r="J120" t="n">
-        <v>99.8</v>
+        <v>45.3</v>
       </c>
       <c r="K120" t="n">
-        <v>95.8</v>
+        <v>9.9</v>
       </c>
       <c r="L120" t="n">
-        <v>0</v>
-      </c>
-      <c r="M120" s="4" t="inlineStr">
-        <is>
-          <t>L2 WATCH</t>
+        <v>0.0005</v>
+      </c>
+      <c r="M120" s="6" t="inlineStr">
+        <is>
+          <t>L3</t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O120" t="inlineStr">
@@ -7438,8 +7438,8 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="5" t="n">
-        <v>3</v>
+      <c r="A121" s="1" t="n">
+        <v>2</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -7479,14 +7479,14 @@
       <c r="L121" t="n">
         <v>-0.0759</v>
       </c>
-      <c r="M121" s="6" t="inlineStr">
-        <is>
-          <t>L3</t>
+      <c r="M121" s="4" t="inlineStr">
+        <is>
+          <t>L2 WATCH</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O121" t="inlineStr">
@@ -7544,7 +7544,7 @@
       </c>
       <c r="N122" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O122" t="inlineStr">
@@ -7602,7 +7602,7 @@
       </c>
       <c r="N123" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O123" t="inlineStr">
@@ -7660,7 +7660,7 @@
       </c>
       <c r="N124" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O124" t="inlineStr">
@@ -7675,7 +7675,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>X1GA.MI</t>
+          <t>MA13.PA</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -7718,7 +7718,7 @@
       </c>
       <c r="N125" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O125" t="inlineStr">
@@ -7776,7 +7776,7 @@
       </c>
       <c r="N126" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O126" t="inlineStr">
@@ -7834,7 +7834,7 @@
       </c>
       <c r="N127" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O127" t="inlineStr">
@@ -7892,7 +7892,7 @@
       </c>
       <c r="N128" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O128" t="inlineStr">
@@ -7907,7 +7907,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>LFIN.MI</t>
+          <t>FINSW.MI</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -7950,7 +7950,7 @@
       </c>
       <c r="N129" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O129" t="inlineStr">
@@ -8008,7 +8008,7 @@
       </c>
       <c r="N130" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O130" t="inlineStr">
@@ -8066,7 +8066,7 @@
       </c>
       <c r="N131" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O131" t="inlineStr">
@@ -8124,7 +8124,7 @@
       </c>
       <c r="N132" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O132" t="inlineStr">
@@ -8139,7 +8139,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>UFRH.MI</t>
+          <t>AFLT.PA</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -8182,7 +8182,7 @@
       </c>
       <c r="N133" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O133" t="inlineStr">
@@ -8192,8 +8192,8 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="1" t="n">
-        <v>2</v>
+      <c r="A134" s="5" t="n">
+        <v>3</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
@@ -8216,31 +8216,31 @@
         </is>
       </c>
       <c r="G134" t="n">
-        <v>15.47</v>
+        <v>6.354</v>
       </c>
       <c r="H134" t="n">
-        <v>15.4573</v>
+        <v>6.5967</v>
       </c>
       <c r="I134" t="n">
-        <v>15.4462</v>
+        <v>7.977</v>
       </c>
       <c r="J134" t="n">
-        <v>100</v>
+        <v>45.6</v>
       </c>
       <c r="K134" t="n">
-        <v>100</v>
+        <v>9.4</v>
       </c>
       <c r="L134" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="M134" s="4" t="inlineStr">
-        <is>
-          <t>L2 WATCH</t>
+        <v>0.1191</v>
+      </c>
+      <c r="M134" s="6" t="inlineStr">
+        <is>
+          <t>L3</t>
         </is>
       </c>
       <c r="N134" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O134" t="inlineStr">
@@ -8298,7 +8298,7 @@
       </c>
       <c r="N135" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O135" t="inlineStr">
@@ -8313,7 +8313,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>X006.MI</t>
+          <t>C3M.PA</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -8356,7 +8356,7 @@
       </c>
       <c r="N136" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O136" t="inlineStr">
@@ -8371,7 +8371,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>EONA.MI</t>
+          <t>CSH.PA</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="N137" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O137" t="inlineStr">
@@ -8448,22 +8448,22 @@
         </is>
       </c>
       <c r="G138" t="n">
-        <v>20.73</v>
+        <v>19.194</v>
       </c>
       <c r="H138" t="n">
-        <v>20.7477</v>
+        <v>19.7582</v>
       </c>
       <c r="I138" t="n">
-        <v>21.141</v>
+        <v>20.2935</v>
       </c>
       <c r="J138" t="n">
-        <v>47.7</v>
+        <v>32.3</v>
       </c>
       <c r="K138" t="n">
-        <v>17.7</v>
+        <v>27.4</v>
       </c>
       <c r="L138" t="n">
-        <v>0.0601</v>
+        <v>-0.0717</v>
       </c>
       <c r="M138" s="6" t="inlineStr">
         <is>
@@ -8472,7 +8472,7 @@
       </c>
       <c r="N138" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O138" t="inlineStr">
@@ -8530,7 +8530,7 @@
       </c>
       <c r="N139" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O139" t="inlineStr">
@@ -8588,7 +8588,7 @@
       </c>
       <c r="N140" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O140" t="inlineStr">
@@ -8603,7 +8603,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>DAXE.MI</t>
+          <t>LYY7.DE</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -8646,7 +8646,7 @@
       </c>
       <c r="N141" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O141" t="inlineStr">
@@ -8704,7 +8704,7 @@
       </c>
       <c r="N142" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O142" t="inlineStr">
@@ -8714,8 +8714,8 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="5" t="n">
-        <v>3</v>
+      <c r="A143" s="1" t="n">
+        <v>2</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
@@ -8755,14 +8755,14 @@
       <c r="L143" t="n">
         <v>0.074</v>
       </c>
-      <c r="M143" s="6" t="inlineStr">
-        <is>
-          <t>L3</t>
+      <c r="M143" s="4" t="inlineStr">
+        <is>
+          <t>L2 WATCH</t>
         </is>
       </c>
       <c r="N143" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O143" t="inlineStr">
@@ -8820,7 +8820,7 @@
       </c>
       <c r="N144" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O144" t="inlineStr">
@@ -8835,7 +8835,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>EMGB.MI</t>
+          <t>EMBHI.MI</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -8878,7 +8878,7 @@
       </c>
       <c r="N145" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O145" t="inlineStr">
@@ -8893,7 +8893,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>EMGB.MI</t>
+          <t>AGEB.PA</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -8936,7 +8936,7 @@
       </c>
       <c r="N146" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O146" t="inlineStr">
@@ -8951,7 +8951,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>USEA.MI</t>
+          <t>USEH.MI</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -8994,7 +8994,7 @@
       </c>
       <c r="N147" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O147" t="inlineStr">
@@ -9028,22 +9028,22 @@
         </is>
       </c>
       <c r="G148" t="n">
-        <v>149.33</v>
+        <v>148.37</v>
       </c>
       <c r="H148" t="n">
-        <v>150.4255</v>
+        <v>148.6929</v>
       </c>
       <c r="I148" t="n">
-        <v>151.2204</v>
+        <v>149.6427</v>
       </c>
       <c r="J148" t="n">
-        <v>37.6</v>
+        <v>43.6</v>
       </c>
       <c r="K148" t="n">
-        <v>17.6</v>
+        <v>22.4</v>
       </c>
       <c r="L148" t="n">
-        <v>-0.2021</v>
+        <v>-0.001</v>
       </c>
       <c r="M148" s="6" t="inlineStr">
         <is>
@@ -9052,7 +9052,7 @@
       </c>
       <c r="N148" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O148" t="inlineStr">
@@ -9110,7 +9110,7 @@
       </c>
       <c r="N149" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O149" t="inlineStr">
@@ -9125,7 +9125,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>EMGB.MI</t>
+          <t>LEMB.L</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="N150" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O150" t="inlineStr">
@@ -9226,7 +9226,7 @@
       </c>
       <c r="N151" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O151" t="inlineStr">
@@ -9241,7 +9241,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>UCBP.MI</t>
+          <t>USIH.PA</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -9284,7 +9284,7 @@
       </c>
       <c r="N152" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O152" t="inlineStr">
@@ -9299,7 +9299,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>UCBE.MI</t>
+          <t>PRAP.SW</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -9342,7 +9342,7 @@
       </c>
       <c r="N153" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O153" t="inlineStr">
@@ -9400,7 +9400,7 @@
       </c>
       <c r="N154" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O154" t="inlineStr">
@@ -9415,7 +9415,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>UCBP.MI</t>
+          <t>USIG.L</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -9458,7 +9458,7 @@
       </c>
       <c r="N155" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O155" t="inlineStr">
@@ -9516,7 +9516,7 @@
       </c>
       <c r="N156" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O156" t="inlineStr">
@@ -9531,7 +9531,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>UCBP.MI</t>
+          <t>USIC.L</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -9574,7 +9574,7 @@
       </c>
       <c r="N157" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O157" t="inlineStr">
@@ -9589,7 +9589,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>USCP.MI</t>
+          <t>USRIH.MI</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -9632,7 +9632,7 @@
       </c>
       <c r="N158" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O158" t="inlineStr">
@@ -9647,7 +9647,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>USCP.MI</t>
+          <t>WEBD.DE</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -9690,7 +9690,7 @@
       </c>
       <c r="N159" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O159" t="inlineStr">
@@ -9748,7 +9748,7 @@
       </c>
       <c r="N160" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O160" t="inlineStr">
@@ -9806,7 +9806,7 @@
       </c>
       <c r="N161" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O161" t="inlineStr">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="N162" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O162" t="inlineStr">
@@ -9879,7 +9879,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>USEX.MI</t>
+          <t>LESA.DE</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -9922,7 +9922,7 @@
       </c>
       <c r="N163" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O163" t="inlineStr">
@@ -9937,7 +9937,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>USEA.MI</t>
+          <t>USEE.AS</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -9980,7 +9980,7 @@
       </c>
       <c r="N164" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O164" t="inlineStr">
@@ -9995,7 +9995,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>USES.MI</t>
+          <t>SADU.PA</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -10038,7 +10038,7 @@
       </c>
       <c r="N165" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O165" t="inlineStr">
@@ -10048,8 +10048,8 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="5" t="n">
-        <v>3</v>
+      <c r="A166" s="1" t="n">
+        <v>2</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
@@ -10089,14 +10089,14 @@
       <c r="L166" t="n">
         <v>-0.3903</v>
       </c>
-      <c r="M166" s="6" t="inlineStr">
-        <is>
-          <t>L3</t>
+      <c r="M166" s="4" t="inlineStr">
+        <is>
+          <t>L2 WATCH</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O166" t="inlineStr">
@@ -10154,7 +10154,7 @@
       </c>
       <c r="N167" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O167" t="inlineStr">
@@ -10212,7 +10212,7 @@
       </c>
       <c r="N168" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O168" t="inlineStr">
@@ -10270,7 +10270,7 @@
       </c>
       <c r="N169" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O169" t="inlineStr">
@@ -10328,7 +10328,7 @@
       </c>
       <c r="N170" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O170" t="inlineStr">
@@ -10386,7 +10386,7 @@
       </c>
       <c r="N171" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O171" t="inlineStr">
@@ -10444,7 +10444,7 @@
       </c>
       <c r="N172" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O172" t="inlineStr">
@@ -10478,22 +10478,22 @@
         </is>
       </c>
       <c r="G173" t="n">
-        <v>15.39</v>
+        <v>15.878</v>
       </c>
       <c r="H173" t="n">
-        <v>15.0577</v>
+        <v>15.2079</v>
       </c>
       <c r="I173" t="n">
-        <v>15.0326</v>
+        <v>14.3084</v>
       </c>
       <c r="J173" t="n">
-        <v>64.40000000000001</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="K173" t="n">
-        <v>19.6</v>
+        <v>19.3</v>
       </c>
       <c r="L173" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.0323</v>
       </c>
       <c r="M173" s="4" t="inlineStr">
         <is>
@@ -10502,7 +10502,7 @@
       </c>
       <c r="N173" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O173" t="inlineStr">
@@ -10560,7 +10560,7 @@
       </c>
       <c r="N174" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O174" t="inlineStr">
@@ -10618,7 +10618,7 @@
       </c>
       <c r="N175" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O175" t="inlineStr">
@@ -10676,7 +10676,7 @@
       </c>
       <c r="N176" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O176" t="inlineStr">
@@ -10734,7 +10734,7 @@
       </c>
       <c r="N177" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O177" t="inlineStr">
@@ -10749,7 +10749,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>MILS.MI</t>
+          <t>GENY.L</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -10792,7 +10792,7 @@
       </c>
       <c r="N178" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O178" t="inlineStr">
@@ -10807,7 +10807,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>ROAI.MI</t>
+          <t>GOAI.PA</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -10850,7 +10850,7 @@
       </c>
       <c r="N179" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O179" t="inlineStr">
@@ -10908,7 +10908,7 @@
       </c>
       <c r="N180" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O180" t="inlineStr">
@@ -10966,7 +10966,7 @@
       </c>
       <c r="N181" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O181" t="inlineStr">
@@ -11000,22 +11000,22 @@
         </is>
       </c>
       <c r="G182" t="n">
-        <v>16.16</v>
+        <v>22.6</v>
       </c>
       <c r="H182" t="n">
-        <v>15.7244</v>
+        <v>21.7023</v>
       </c>
       <c r="I182" t="n">
-        <v>15.6592</v>
+        <v>19.3749</v>
       </c>
       <c r="J182" t="n">
-        <v>65.7</v>
+        <v>64</v>
       </c>
       <c r="K182" t="n">
-        <v>20.4</v>
+        <v>25.9</v>
       </c>
       <c r="L182" t="n">
-        <v>0.08790000000000001</v>
+        <v>-0.09569999999999999</v>
       </c>
       <c r="M182" s="4" t="inlineStr">
         <is>
@@ -11024,7 +11024,7 @@
       </c>
       <c r="N182" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O182" t="inlineStr">
@@ -11082,7 +11082,7 @@
       </c>
       <c r="N183" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O183" t="inlineStr">
@@ -11145,7 +11145,7 @@
       </c>
       <c r="N184" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O184" t="inlineStr">
@@ -11208,7 +11208,7 @@
       </c>
       <c r="N185" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O185" t="inlineStr">
@@ -11271,7 +11271,7 @@
       </c>
       <c r="N186" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O186" t="inlineStr">
@@ -11282,7 +11282,7 @@
     </row>
     <row r="187">
       <c r="A187" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -11310,31 +11310,31 @@
         </is>
       </c>
       <c r="G187" t="n">
-        <v>646.38</v>
+        <v>795.67</v>
       </c>
       <c r="H187" t="n">
-        <v>625.5232</v>
+        <v>781.3156</v>
       </c>
       <c r="I187" t="n">
-        <v>619.323</v>
+        <v>728.8896</v>
       </c>
       <c r="J187" t="n">
-        <v>77.2</v>
+        <v>59.7</v>
       </c>
       <c r="K187" t="n">
-        <v>27.4</v>
+        <v>20.5</v>
       </c>
       <c r="L187" t="n">
-        <v>3.4834</v>
-      </c>
-      <c r="M187" s="4" t="inlineStr">
-        <is>
-          <t>L2 WATCH</t>
+        <v>-2.8646</v>
+      </c>
+      <c r="M187" s="1" t="inlineStr">
+        <is>
+          <t>L1 BUY (5/5)</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O187" t="inlineStr">
@@ -11397,7 +11397,7 @@
       </c>
       <c r="N188" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O188" t="inlineStr">
@@ -11460,7 +11460,7 @@
       </c>
       <c r="N189" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O189" t="inlineStr">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="N190" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O190" t="inlineStr">
@@ -11533,8 +11533,8 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="1" t="n">
-        <v>2</v>
+      <c r="A191" s="5" t="n">
+        <v>3</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
@@ -11562,31 +11562,31 @@
         </is>
       </c>
       <c r="G191" t="n">
-        <v>164.86</v>
+        <v>42.125</v>
       </c>
       <c r="H191" t="n">
-        <v>154.0188</v>
+        <v>43.5879</v>
       </c>
       <c r="I191" t="n">
-        <v>151.6332</v>
+        <v>59.4245</v>
       </c>
       <c r="J191" t="n">
-        <v>79.7</v>
+        <v>47.5</v>
       </c>
       <c r="K191" t="n">
-        <v>26.8</v>
+        <v>7.3</v>
       </c>
       <c r="L191" t="n">
-        <v>1.7035</v>
-      </c>
-      <c r="M191" s="4" t="inlineStr">
-        <is>
-          <t>L2 WATCH</t>
+        <v>1.5795</v>
+      </c>
+      <c r="M191" s="6" t="inlineStr">
+        <is>
+          <t>L3</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O191" t="inlineStr">
@@ -11649,7 +11649,7 @@
       </c>
       <c r="N192" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O192" t="inlineStr">
@@ -11712,7 +11712,7 @@
       </c>
       <c r="N193" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O193" t="inlineStr">
@@ -11775,7 +11775,7 @@
       </c>
       <c r="N194" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O194" t="inlineStr">
@@ -11814,22 +11814,22 @@
         </is>
       </c>
       <c r="G195" t="n">
-        <v>121.96</v>
+        <v>4.4735</v>
       </c>
       <c r="H195" t="n">
-        <v>123.0848</v>
+        <v>7.7948</v>
       </c>
       <c r="I195" t="n">
-        <v>123.7056</v>
+        <v>26.0084</v>
       </c>
       <c r="J195" t="n">
-        <v>35.6</v>
+        <v>45.4</v>
       </c>
       <c r="K195" t="n">
-        <v>19.2</v>
+        <v>9.6</v>
       </c>
       <c r="L195" t="n">
-        <v>-0.1891</v>
+        <v>1.5434</v>
       </c>
       <c r="M195" s="6" t="inlineStr">
         <is>
@@ -11838,7 +11838,7 @@
       </c>
       <c r="N195" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O195" t="inlineStr">
@@ -11901,7 +11901,7 @@
       </c>
       <c r="N196" t="inlineStr">
         <is>
-          <t>2026-05-21 21:03</t>
+          <t>2026-05-21 22:20</t>
         </is>
       </c>
       <c r="O196" t="inlineStr">

</xml_diff>

<commit_message>
Aggiunge 19 nuovi ETF a etf_monitoraggio.xlsx (da L3)
Copertura ampliata con ETF mancanti per categoria:
- Asia/Emergenti: CNYA.L, NDIA.L, CSKR.L, LTAM.L, EMVL.L, CI2.PA
- Globale/Factor: WSML.L, VHYL.L, GGRP.L, IWMO.L, IWQU.L, MVOL.L
- Settoriale Salute: HEAL.L, HLTH.DE
- Settoriale Tecnologia: EQQQ.L, WTEC.L
- Obbligazionari: IGIL.L, AGGG.L, IBTS.L
Totale ETF: 195 → 214. ISIN da completare manualmente.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ETF" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ETF" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O196"/>
+  <dimension ref="A1:O215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11910,6 +11910,747 @@
         </is>
       </c>
     </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>3</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>CNYA.L</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>iShares MSCI China A UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Asia - Emergente</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Londra</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G197" t="n">
+        <v>6.2525</v>
+      </c>
+      <c r="N197" t="inlineStr">
+        <is>
+          <t>2026-05-22 01:10</t>
+        </is>
+      </c>
+      <c r="O197" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>3</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>NDIA.L</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>iShares MSCI India UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Asia - Emergente</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Londra</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G198" t="n">
+        <v>8.555</v>
+      </c>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>2026-05-22 01:10</t>
+        </is>
+      </c>
+      <c r="O198" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>3</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>WSML.L</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>iShares MSCI World Small Cap UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Globale / All-World</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Londra</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G199" t="n">
+        <v>10.042</v>
+      </c>
+      <c r="N199" t="inlineStr">
+        <is>
+          <t>2026-05-22 01:10</t>
+        </is>
+      </c>
+      <c r="O199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>3</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>VHYL.L</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Vanguard FTSE All-World High Div Yield UCITS ETF</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Globale / All-World</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Londra</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="G200" t="n">
+        <v>66.56999999999999</v>
+      </c>
+      <c r="N200" t="inlineStr">
+        <is>
+          <t>2026-05-22 01:10</t>
+        </is>
+      </c>
+      <c r="O200" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>3</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>GGRP.L</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>WisdomTree Global Quality Dividend Growth UCITS ETF</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Globale / All-World</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Londra</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="G201" t="n">
+        <v>2990</v>
+      </c>
+      <c r="N201" t="inlineStr">
+        <is>
+          <t>2026-05-22 01:10</t>
+        </is>
+      </c>
+      <c r="O201" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>3</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>HEAL.L</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>iShares Healthcare Innovation UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Settoriale - Salute</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Londra</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G202" t="n">
+        <v>8.625</v>
+      </c>
+      <c r="N202" t="inlineStr">
+        <is>
+          <t>2026-05-22 01:10</t>
+        </is>
+      </c>
+      <c r="O202" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>3</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>HLTH.DE</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Amundi MSCI World Health Care UCITS ETF EUR (Acc)</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Settoriale - Salute</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Francoforte</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G203" t="n">
+        <v>223.4</v>
+      </c>
+      <c r="N203" t="inlineStr">
+        <is>
+          <t>2026-05-22 01:10</t>
+        </is>
+      </c>
+      <c r="O203" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>3</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>EQQQ.L</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Invesco EQQQ NASDAQ-100 UCITS ETF</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Settoriale - Tecnologia</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Londra</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="G204" t="n">
+        <v>53152</v>
+      </c>
+      <c r="N204" t="inlineStr">
+        <is>
+          <t>2026-05-22 01:10</t>
+        </is>
+      </c>
+      <c r="O204" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>3</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>WTEC.L</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>SPDR MSCI World Technology UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Settoriale - Tecnologia</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Londra</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G205" t="n">
+        <v>256.86</v>
+      </c>
+      <c r="N205" t="inlineStr">
+        <is>
+          <t>2026-05-22 01:10</t>
+        </is>
+      </c>
+      <c r="O205" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>3</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>IWMO.L</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>iShares Edge MSCI World Momentum Factor UCITS ETF</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Globale / All-World</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Londra</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G206" t="n">
+        <v>112.91</v>
+      </c>
+      <c r="N206" t="inlineStr">
+        <is>
+          <t>2026-05-22 01:10</t>
+        </is>
+      </c>
+      <c r="O206" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>3</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>IWQU.L</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>iShares Edge MSCI World Quality Factor UCITS ETF</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Globale / All-World</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Londra</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G207" t="n">
+        <v>85.61</v>
+      </c>
+      <c r="N207" t="inlineStr">
+        <is>
+          <t>2026-05-22 01:10</t>
+        </is>
+      </c>
+      <c r="O207" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>3</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>MVOL.L</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>iShares Edge MSCI World Minimum Volatility UCITS ETF</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Globale / All-World</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Londra</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G208" t="n">
+        <v>74.64</v>
+      </c>
+      <c r="N208" t="inlineStr">
+        <is>
+          <t>2026-05-22 01:10</t>
+        </is>
+      </c>
+      <c r="O208" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>3</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>IGIL.L</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>iShares Global Inflation Linked Govt Bond UCITS ETF</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Obbligazionari - Inflation Linked</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Londra</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G209" t="n">
+        <v>165.99</v>
+      </c>
+      <c r="N209" t="inlineStr">
+        <is>
+          <t>2026-05-22 01:10</t>
+        </is>
+      </c>
+      <c r="O209" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>3</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>LTAM.L</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>iShares MSCI EM Latin America UCITS ETF USD (Dist)</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>America Latina e Centrale</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Londra</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="G210" t="n">
+        <v>1588.5</v>
+      </c>
+      <c r="N210" t="inlineStr">
+        <is>
+          <t>2026-05-22 01:10</t>
+        </is>
+      </c>
+      <c r="O210" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>3</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>CSKR.L</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>iShares MSCI Korea UCITS ETF USD (Dist)</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Asia - Emergente</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Londra</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G211" t="n">
+        <v>497.45</v>
+      </c>
+      <c r="N211" t="inlineStr">
+        <is>
+          <t>2026-05-22 01:10</t>
+        </is>
+      </c>
+      <c r="O211" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>3</v>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>AGGG.L</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>iShares Core Global Aggregate Bond UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Obbligazionari - Globali</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Londra</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G212" t="n">
+        <v>4.375</v>
+      </c>
+      <c r="N212" t="inlineStr">
+        <is>
+          <t>2026-05-22 01:10</t>
+        </is>
+      </c>
+      <c r="O212" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>3</v>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>IBTS.L</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>iShares $ Treasury Bond 1-3yr UCITS ETF USD (Dist)</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Obbligazionari - Governativi USD</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Londra</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="G213" t="n">
+        <v>94.58</v>
+      </c>
+      <c r="N213" t="inlineStr">
+        <is>
+          <t>2026-05-22 01:10</t>
+        </is>
+      </c>
+      <c r="O213" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>3</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>EMVL.L</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>iShares Edge MSCI EM Min Vol Factor UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Asia - Emergente</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Londra</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G214" t="n">
+        <v>94.97</v>
+      </c>
+      <c r="N214" t="inlineStr">
+        <is>
+          <t>2026-05-22 01:10</t>
+        </is>
+      </c>
+      <c r="O214" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" t="n">
+        <v>3</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>CI2.PA</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Amundi MSCI India UCITS ETF Swap EUR (Acc)</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Asia - Emergente</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Parigi</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G215" t="n">
+        <v>776.274</v>
+      </c>
+      <c r="N215" t="inlineStr">
+        <is>
+          <t>2026-05-22 01:10</t>
+        </is>
+      </c>
+      <c r="O215" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix MACD: pendenza sempre obbligatoria, rimosso bypass near_ema
La condizione 6 (MACD momentum) ora richiede sempre macd_h > 0 AND
macd_h > macd_h_prev. Rimosso il ramo OR (dist_ema20 < 2%) che
permetteva ingressi con MACD in calo se il prezzo era vicino all'EMA20
— causava falsi ingressi su ETF obbligazionari con prezzo in discesa.
Rimosso AFRN.PA da L1 (falso ingresso).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -593,7 +593,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -782,7 +782,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1349,7 +1349,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -1412,7 +1412,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -1538,7 +1538,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -1601,7 +1601,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -1727,7 +1727,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -1790,7 +1790,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -1916,7 +1916,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -2042,7 +2042,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -2168,7 +2168,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
@@ -2231,7 +2231,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
@@ -2294,7 +2294,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
@@ -2357,7 +2357,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -2609,7 +2609,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
@@ -2735,7 +2735,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
@@ -2798,7 +2798,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
@@ -2861,7 +2861,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
@@ -2924,7 +2924,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
@@ -2987,7 +2987,7 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
@@ -3176,7 +3176,7 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
@@ -3239,7 +3239,7 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
@@ -3302,7 +3302,7 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
@@ -3365,7 +3365,7 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
@@ -3428,7 +3428,7 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
@@ -3491,7 +3491,7 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
@@ -3554,7 +3554,7 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
@@ -3617,7 +3617,7 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
@@ -3680,7 +3680,7 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
@@ -3806,7 +3806,7 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
@@ -3932,7 +3932,7 @@
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
@@ -3995,7 +3995,7 @@
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
@@ -4058,7 +4058,7 @@
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O57" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O58" t="inlineStr">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
@@ -4247,7 +4247,7 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O60" t="inlineStr">
@@ -4310,7 +4310,7 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
@@ -4373,7 +4373,7 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O62" t="inlineStr">
@@ -4436,7 +4436,7 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O63" t="inlineStr">
@@ -4499,7 +4499,7 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
@@ -4625,7 +4625,7 @@
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O66" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O67" t="inlineStr">
@@ -4751,7 +4751,7 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O68" t="inlineStr">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
@@ -4877,7 +4877,7 @@
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O70" t="inlineStr">
@@ -4940,7 +4940,7 @@
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O71" t="inlineStr">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O72" t="inlineStr">
@@ -5066,7 +5066,7 @@
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O73" t="inlineStr">
@@ -5129,7 +5129,7 @@
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O74" t="inlineStr">
@@ -5192,7 +5192,7 @@
       </c>
       <c r="N75" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O75" t="inlineStr">
@@ -5255,7 +5255,7 @@
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O76" t="inlineStr">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
@@ -5381,7 +5381,7 @@
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O78" t="inlineStr">
@@ -5444,7 +5444,7 @@
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O79" t="inlineStr">
@@ -5507,7 +5507,7 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
@@ -5570,7 +5570,7 @@
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O81" t="inlineStr">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O82" t="inlineStr">
@@ -5696,7 +5696,7 @@
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O83" t="inlineStr">
@@ -5759,7 +5759,7 @@
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O84" t="inlineStr">
@@ -5822,7 +5822,7 @@
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O85" t="inlineStr">
@@ -5885,7 +5885,7 @@
       </c>
       <c r="N86" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O86" t="inlineStr">
@@ -5948,7 +5948,7 @@
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O87" t="inlineStr">
@@ -6011,7 +6011,7 @@
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O88" t="inlineStr">
@@ -6074,7 +6074,7 @@
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O89" t="inlineStr">
@@ -6137,7 +6137,7 @@
       </c>
       <c r="N90" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O90" t="inlineStr">
@@ -6200,7 +6200,7 @@
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O91" t="inlineStr">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="N92" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O92" t="inlineStr">
@@ -6326,7 +6326,7 @@
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O93" t="inlineStr">
@@ -6389,7 +6389,7 @@
       </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O94" t="inlineStr">
@@ -6452,7 +6452,7 @@
       </c>
       <c r="N95" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O95" t="inlineStr">
@@ -6515,7 +6515,7 @@
       </c>
       <c r="N96" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O96" t="inlineStr">
@@ -6578,7 +6578,7 @@
       </c>
       <c r="N97" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O97" t="inlineStr">
@@ -6641,7 +6641,7 @@
       </c>
       <c r="N98" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O98" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="N99" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O99" t="inlineStr">
@@ -6767,7 +6767,7 @@
       </c>
       <c r="N100" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O100" t="inlineStr">
@@ -6830,7 +6830,7 @@
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O101" t="inlineStr">
@@ -6893,7 +6893,7 @@
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O102" t="inlineStr">
@@ -6956,7 +6956,7 @@
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O103" t="inlineStr">
@@ -7019,7 +7019,7 @@
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O104" t="inlineStr">
@@ -7082,7 +7082,7 @@
       </c>
       <c r="N105" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O105" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="N106" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O106" t="inlineStr">
@@ -7208,7 +7208,7 @@
       </c>
       <c r="N107" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O107" t="inlineStr">
@@ -7219,7 +7219,7 @@
     </row>
     <row r="108">
       <c r="A108" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
@@ -7264,14 +7264,14 @@
       <c r="L108" t="n">
         <v>0.0013</v>
       </c>
-      <c r="M108" s="1" t="inlineStr">
-        <is>
-          <t>L1 BUY (6/6)</t>
+      <c r="M108" s="7" t="inlineStr">
+        <is>
+          <t>L3</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 13:06</t>
         </is>
       </c>
       <c r="O108" t="inlineStr">
@@ -7334,7 +7334,7 @@
       </c>
       <c r="N109" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O109" t="inlineStr">
@@ -7397,7 +7397,7 @@
       </c>
       <c r="N110" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O110" t="inlineStr">
@@ -7460,7 +7460,7 @@
       </c>
       <c r="N111" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O111" t="inlineStr">
@@ -7523,7 +7523,7 @@
       </c>
       <c r="N112" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O112" t="inlineStr">
@@ -7586,7 +7586,7 @@
       </c>
       <c r="N113" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O113" t="inlineStr">
@@ -7649,7 +7649,7 @@
       </c>
       <c r="N114" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O114" t="inlineStr">
@@ -7712,7 +7712,7 @@
       </c>
       <c r="N115" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O115" t="inlineStr">
@@ -7775,7 +7775,7 @@
       </c>
       <c r="N116" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O116" t="inlineStr">
@@ -7838,7 +7838,7 @@
       </c>
       <c r="N117" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O117" t="inlineStr">
@@ -7901,7 +7901,7 @@
       </c>
       <c r="N118" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O118" t="inlineStr">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="N119" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O119" t="inlineStr">
@@ -8027,7 +8027,7 @@
       </c>
       <c r="N120" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O120" t="inlineStr">
@@ -8090,7 +8090,7 @@
       </c>
       <c r="N121" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O121" t="inlineStr">
@@ -8153,7 +8153,7 @@
       </c>
       <c r="N122" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O122" t="inlineStr">
@@ -8216,7 +8216,7 @@
       </c>
       <c r="N123" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O123" t="inlineStr">
@@ -8279,7 +8279,7 @@
       </c>
       <c r="N124" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O124" t="inlineStr">
@@ -8342,7 +8342,7 @@
       </c>
       <c r="N125" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O125" t="inlineStr">
@@ -8405,7 +8405,7 @@
       </c>
       <c r="N126" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O126" t="inlineStr">
@@ -8468,7 +8468,7 @@
       </c>
       <c r="N127" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O127" t="inlineStr">
@@ -8531,7 +8531,7 @@
       </c>
       <c r="N128" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O128" t="inlineStr">
@@ -8594,7 +8594,7 @@
       </c>
       <c r="N129" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O129" t="inlineStr">
@@ -8657,7 +8657,7 @@
       </c>
       <c r="N130" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O130" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="N131" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O131" t="inlineStr">
@@ -8783,7 +8783,7 @@
       </c>
       <c r="N132" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O132" t="inlineStr">
@@ -8846,7 +8846,7 @@
       </c>
       <c r="N133" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O133" t="inlineStr">
@@ -8909,7 +8909,7 @@
       </c>
       <c r="N134" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O134" t="inlineStr">
@@ -8972,7 +8972,7 @@
       </c>
       <c r="N135" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O135" t="inlineStr">
@@ -9035,7 +9035,7 @@
       </c>
       <c r="N136" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O136" t="inlineStr">
@@ -9098,7 +9098,7 @@
       </c>
       <c r="N137" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O137" t="inlineStr">
@@ -9161,7 +9161,7 @@
       </c>
       <c r="N138" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O138" t="inlineStr">
@@ -9224,7 +9224,7 @@
       </c>
       <c r="N139" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O139" t="inlineStr">
@@ -9287,7 +9287,7 @@
       </c>
       <c r="N140" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O140" t="inlineStr">
@@ -9350,7 +9350,7 @@
       </c>
       <c r="N141" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O141" t="inlineStr">
@@ -9413,7 +9413,7 @@
       </c>
       <c r="N142" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O142" t="inlineStr">
@@ -9476,7 +9476,7 @@
       </c>
       <c r="N143" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O143" t="inlineStr">
@@ -9539,7 +9539,7 @@
       </c>
       <c r="N144" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O144" t="inlineStr">
@@ -9602,7 +9602,7 @@
       </c>
       <c r="N145" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O145" t="inlineStr">
@@ -9665,7 +9665,7 @@
       </c>
       <c r="N146" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O146" t="inlineStr">
@@ -9728,7 +9728,7 @@
       </c>
       <c r="N147" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O147" t="inlineStr">
@@ -9791,7 +9791,7 @@
       </c>
       <c r="N148" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O148" t="inlineStr">
@@ -9854,7 +9854,7 @@
       </c>
       <c r="N149" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O149" t="inlineStr">
@@ -9917,7 +9917,7 @@
       </c>
       <c r="N150" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O150" t="inlineStr">
@@ -9980,7 +9980,7 @@
       </c>
       <c r="N151" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O151" t="inlineStr">
@@ -10043,7 +10043,7 @@
       </c>
       <c r="N152" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O152" t="inlineStr">
@@ -10106,7 +10106,7 @@
       </c>
       <c r="N153" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O153" t="inlineStr">
@@ -10169,7 +10169,7 @@
       </c>
       <c r="N154" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O154" t="inlineStr">
@@ -10232,7 +10232,7 @@
       </c>
       <c r="N155" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O155" t="inlineStr">
@@ -10295,7 +10295,7 @@
       </c>
       <c r="N156" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O156" t="inlineStr">
@@ -10358,7 +10358,7 @@
       </c>
       <c r="N157" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O157" t="inlineStr">
@@ -10421,7 +10421,7 @@
       </c>
       <c r="N158" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O158" t="inlineStr">
@@ -10484,7 +10484,7 @@
       </c>
       <c r="N159" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O159" t="inlineStr">
@@ -10547,7 +10547,7 @@
       </c>
       <c r="N160" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O160" t="inlineStr">
@@ -10610,7 +10610,7 @@
       </c>
       <c r="N161" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O161" t="inlineStr">
@@ -10673,7 +10673,7 @@
       </c>
       <c r="N162" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O162" t="inlineStr">
@@ -10736,7 +10736,7 @@
       </c>
       <c r="N163" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O163" t="inlineStr">
@@ -10799,7 +10799,7 @@
       </c>
       <c r="N164" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O164" t="inlineStr">
@@ -10862,7 +10862,7 @@
       </c>
       <c r="N165" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O165" t="inlineStr">
@@ -10925,7 +10925,7 @@
       </c>
       <c r="N166" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O166" t="inlineStr">
@@ -10988,7 +10988,7 @@
       </c>
       <c r="N167" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O167" t="inlineStr">
@@ -11051,7 +11051,7 @@
       </c>
       <c r="N168" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O168" t="inlineStr">
@@ -11114,7 +11114,7 @@
       </c>
       <c r="N169" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O169" t="inlineStr">
@@ -11177,7 +11177,7 @@
       </c>
       <c r="N170" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O170" t="inlineStr">
@@ -11240,7 +11240,7 @@
       </c>
       <c r="N171" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O171" t="inlineStr">
@@ -11303,7 +11303,7 @@
       </c>
       <c r="N172" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O172" t="inlineStr">
@@ -11366,7 +11366,7 @@
       </c>
       <c r="N173" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O173" t="inlineStr">
@@ -11429,7 +11429,7 @@
       </c>
       <c r="N174" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O174" t="inlineStr">
@@ -11492,7 +11492,7 @@
       </c>
       <c r="N175" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O175" t="inlineStr">
@@ -11555,7 +11555,7 @@
       </c>
       <c r="N176" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O176" t="inlineStr">
@@ -11618,7 +11618,7 @@
       </c>
       <c r="N177" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O177" t="inlineStr">
@@ -11681,7 +11681,7 @@
       </c>
       <c r="N178" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O178" t="inlineStr">
@@ -11744,7 +11744,7 @@
       </c>
       <c r="N179" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O179" t="inlineStr">
@@ -11783,22 +11783,22 @@
         </is>
       </c>
       <c r="G180" t="n">
-        <v>362.75</v>
+        <v>65.81999999999999</v>
       </c>
       <c r="H180" t="n">
-        <v>345.7242</v>
+        <v>62.6522</v>
       </c>
       <c r="I180" t="n">
-        <v>337.8794</v>
+        <v>58.2662</v>
       </c>
       <c r="J180" t="n">
-        <v>79</v>
+        <v>72.3</v>
       </c>
       <c r="K180" t="n">
-        <v>32.9</v>
+        <v>44.4</v>
       </c>
       <c r="L180" t="n">
-        <v>2.1498</v>
+        <v>0.0555</v>
       </c>
       <c r="M180" s="4" t="inlineStr">
         <is>
@@ -11807,7 +11807,7 @@
       </c>
       <c r="N180" t="inlineStr">
         <is>
-          <t>2026-05-22 12:24</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O180" t="inlineStr">
@@ -11870,7 +11870,7 @@
       </c>
       <c r="N181" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
     </row>
@@ -11928,7 +11928,7 @@
       </c>
       <c r="N182" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
     </row>
@@ -11986,7 +11986,7 @@
       </c>
       <c r="N183" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
     </row>
@@ -12044,7 +12044,7 @@
       </c>
       <c r="N184" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
     </row>
@@ -12102,7 +12102,7 @@
       </c>
       <c r="N185" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
     </row>
@@ -12160,7 +12160,7 @@
       </c>
       <c r="N186" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
     </row>
@@ -12218,7 +12218,7 @@
       </c>
       <c r="N187" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
     </row>
@@ -12276,7 +12276,7 @@
       </c>
       <c r="N188" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
     </row>
@@ -12334,7 +12334,7 @@
       </c>
       <c r="N189" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O189" t="inlineStr">
@@ -12397,7 +12397,7 @@
       </c>
       <c r="N190" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
     </row>
@@ -12455,7 +12455,7 @@
       </c>
       <c r="N191" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O191" t="inlineStr">
@@ -12518,7 +12518,7 @@
       </c>
       <c r="N192" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O192" t="inlineStr">
@@ -12581,7 +12581,7 @@
       </c>
       <c r="N193" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
     </row>
@@ -12639,7 +12639,7 @@
       </c>
       <c r="N194" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
     </row>
@@ -12697,7 +12697,7 @@
       </c>
       <c r="N195" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O195" t="inlineStr">
@@ -12760,7 +12760,7 @@
       </c>
       <c r="N196" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
     </row>
@@ -12818,7 +12818,7 @@
       </c>
       <c r="N197" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O197" t="inlineStr">
@@ -12881,7 +12881,7 @@
       </c>
       <c r="N198" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
     </row>
@@ -12927,7 +12927,7 @@
         <v>93.09999999999999</v>
       </c>
       <c r="K199" t="n">
-        <v>89.5</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="L199" t="n">
         <v>-0.002</v>
@@ -12939,7 +12939,7 @@
       </c>
       <c r="N199" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O199" t="inlineStr">
@@ -12949,8 +12949,8 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" t="n">
-        <v>3</v>
+      <c r="A200" s="1" t="n">
+        <v>2</v>
       </c>
       <c r="B200" t="inlineStr">
         <is>
@@ -12977,14 +12977,32 @@
           <t>EUR</t>
         </is>
       </c>
-      <c r="M200" s="6" t="inlineStr">
-        <is>
-          <t>L3</t>
+      <c r="G200" t="n">
+        <v>99.09</v>
+      </c>
+      <c r="H200" t="n">
+        <v>99.0094</v>
+      </c>
+      <c r="I200" t="n">
+        <v>98.87</v>
+      </c>
+      <c r="J200" t="n">
+        <v>65.40000000000001</v>
+      </c>
+      <c r="K200" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="L200" t="n">
+        <v>0.0049</v>
+      </c>
+      <c r="M200" s="4" t="inlineStr">
+        <is>
+          <t>L2 WATCH</t>
         </is>
       </c>
       <c r="N200" t="inlineStr">
         <is>
-          <t>2026-05-22 12:19</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O200" t="inlineStr">
@@ -13035,7 +13053,7 @@
         <v>66.40000000000001</v>
       </c>
       <c r="K201" t="n">
-        <v>36.4</v>
+        <v>36.5</v>
       </c>
       <c r="L201" t="n">
         <v>-0.2042</v>
@@ -13047,7 +13065,7 @@
       </c>
       <c r="N201" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O201" t="inlineStr">
@@ -13098,7 +13116,7 @@
         <v>65.40000000000001</v>
       </c>
       <c r="K202" t="n">
-        <v>29.9</v>
+        <v>31.4</v>
       </c>
       <c r="L202" t="n">
         <v>-0.094</v>
@@ -13110,7 +13128,7 @@
       </c>
       <c r="N202" t="inlineStr">
         <is>
-          <t>2026-05-22 12:13</t>
+          <t>2026-05-22 12:28</t>
         </is>
       </c>
       <c r="O202" t="inlineStr">

</xml_diff>

<commit_message>
Fix 170 ticker .MI → alternative .PA/.DE/.L/.AS funzionanti su Yahoo Finance
- etf_monitoraggio.xlsx: 170 ticker .MI sostituiti con equivalenti su Euronext Paris (.PA),
  XETRA (.DE), LSE (.L), Amsterdam (.AS), SIX Swiss (.SW)
- deploy.sh: backup/restore ora usa smart_restore.py (preserva solo Livello dal VPS,
  lascia passare i nuovi ticker da git — evita che il restore sovrascriva le correzioni)
- smart_restore.py: merge intelligente backup VPS → Excel git (match per ISIN/Ticker)
- fix_mi_tickers.py: script one-shot usato per il fix (documentazione processo)

Rimasti 10 ticker .MI: 7 confermati funzionanti, 3 senza alternativa (BTP10, BTP13, USRIH)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ETF" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ETF" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -545,7 +545,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>KOR.MI</t>
+          <t>KRW.PA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>TUR.MI</t>
+          <t>TUR.PA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BRES.MI</t>
+          <t>LBRE.DE</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -734,7 +734,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>GRC.MI</t>
+          <t>GRE.PA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BRA.MI</t>
+          <t>RIO.PA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BRES.MI</t>
+          <t>CHM.PA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ENRG.MI</t>
+          <t>CWE.PA</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -986,7 +986,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ENER.MI</t>
+          <t>NRJ.PA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CEC.MI</t>
+          <t>CEC.PA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>TELE.MI</t>
+          <t>TELE.PA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>EMXC.MI</t>
+          <t>EMXC.L</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>UTIL.MI</t>
+          <t>UTI.MI</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>TPXH.MI</t>
+          <t>JPN.PA</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TPXH.MI</t>
+          <t>TPXH.PA</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>LAFRI.MI</t>
+          <t>LGQM.DE</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>AEEM.MI</t>
+          <t>AEMD.DE</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>AEEM.MI</t>
+          <t>AEME.PA</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>TPXH.MI</t>
+          <t>TPXE.PA</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1805,7 +1805,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>BNK.MI</t>
+          <t>BNK.PA</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1931,7 +1931,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>AMEG.MI</t>
+          <t>AMEG.L</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CJ1.MI</t>
+          <t>CJ1.PA</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2057,7 +2057,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>AASI.MI</t>
+          <t>AEJ.PA</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CRB.MI</t>
+          <t>COMO.PA</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>AASI.MI</t>
+          <t>EMAD.L</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2309,7 +2309,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>VLUE.MI</t>
+          <t>CV9.PA</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>BNKE.MI</t>
+          <t>BNKE.PA</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2498,7 +2498,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>AASI.MI</t>
+          <t>APX.PA</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2624,7 +2624,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>WAT.MI</t>
+          <t>WAT.PA</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2687,7 +2687,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CI2.MI</t>
+          <t>LIGS.DE</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>FOOD.MI</t>
+          <t>LFOD.DE</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>EMSR.MI</t>
+          <t>EMSRI.PA</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2876,7 +2876,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>EMES.MI</t>
+          <t>SADM.DE</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>EPRE.MI</t>
+          <t>EPRE.PA</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CN1.MI</t>
+          <t>CN1.PA</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CEM.MI</t>
+          <t>MMS.PA</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CV9.MI</t>
+          <t>VAL.PA</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -3191,7 +3191,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CEU.MI</t>
+          <t>MEU.PA</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -3254,7 +3254,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CEU.MI</t>
+          <t>CEU2.PA</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -3317,7 +3317,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>FMI.MI</t>
+          <t>MIB.PA</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -3380,7 +3380,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>LWCE.MI</t>
+          <t>LWCE.PA</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>EUPA.MI</t>
+          <t>CEUG.DE</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>RS2K.MI</t>
+          <t>RS2K.PA</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3632,7 +3632,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>EUPA.MI</t>
+          <t>ESGH.PA</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -3695,7 +3695,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>EUPA.MI</t>
+          <t>ESGE.PA</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>HLT.MI</t>
+          <t>HLT.PA</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3821,7 +3821,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>MFDD.MI</t>
+          <t>MFDD.L</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -3884,7 +3884,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>QCEU.MI</t>
+          <t>QCEU.PA</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -3947,7 +3947,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>CHIP.MI</t>
+          <t>CHIP.SW</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -4010,7 +4010,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>FMI.MI</t>
+          <t>FMI.PA</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -4073,7 +4073,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>MSE.MI</t>
+          <t>MSE.PA</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -4199,7 +4199,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>CMU.MI</t>
+          <t>CMU.PA</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -4262,7 +4262,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>CD9.MI</t>
+          <t>DJE.PA</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -4325,7 +4325,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>WINC.MI</t>
+          <t>WINC.AS</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -4388,7 +4388,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>CG9.MI</t>
+          <t>LGWT.DE</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -4451,7 +4451,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>EUPA.MI</t>
+          <t>EUSRI.PA</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>EPRA.MI</t>
+          <t>MWO.PA</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -4577,7 +4577,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>CC1.MI</t>
+          <t>CNAL.L</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -4640,7 +4640,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>EUPA.MI</t>
+          <t>EDSRI.MI</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ACWE.MI</t>
+          <t>ACWI.PA</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>EMI.MI</t>
+          <t>EMI.DE</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -4892,7 +4892,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>UINC.MI</t>
+          <t>INCI.AS</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -5018,7 +5018,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>WOEE.MI</t>
+          <t>WOEE.AS</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -5081,7 +5081,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>WHEA.MI</t>
+          <t>HLTW.PA</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -5144,7 +5144,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>X15E.MI</t>
+          <t>MTE.PA</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -5207,7 +5207,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>IFLX.MI</t>
+          <t>IFLX.DE</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -5270,7 +5270,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>SWDA.MI</t>
+          <t>IWDA.L</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ECRP.MI</t>
+          <t>CC4.PA</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -5459,7 +5459,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>CW8.MI</t>
+          <t>WLDH.PA</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -5522,7 +5522,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>ECRP.MI</t>
+          <t>ECRP.PA</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -5585,7 +5585,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>CC1.MI</t>
+          <t>CC1.PA</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>X710.MI</t>
+          <t>MTDD.DE</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -5711,7 +5711,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>X1G.MI</t>
+          <t>X1G.PA</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -5774,7 +5774,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>ECRP.MI</t>
+          <t>CRPX.L</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -5837,7 +5837,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>EGRI.MI</t>
+          <t>EGRI.PA</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -5900,7 +5900,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>X57E.MI</t>
+          <t>X57E.DE</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>CW8.MI</t>
+          <t>CW8.PA</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -6026,7 +6026,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>CW8.MI</t>
+          <t>WLD.PA</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -6089,7 +6089,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>AHYE.MI</t>
+          <t>AHYE.PA</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -6152,7 +6152,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>GOVA.MI</t>
+          <t>10AL.DE</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -6215,7 +6215,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>GGOV.MI</t>
+          <t>EAH.DE</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>CW8.MI</t>
+          <t>WLDC.PA</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -6341,7 +6341,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>CB3.MI</t>
+          <t>CB3.PA</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -6404,7 +6404,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>GAGG.MI</t>
+          <t>CLIM.PA</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -6467,7 +6467,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>CORP.MI</t>
+          <t>EBBB.PA</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -6530,7 +6530,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>CBEF.MI</t>
+          <t>CNB.PA</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -6593,7 +6593,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>GHYA.MI</t>
+          <t>GHYU.L</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -6656,7 +6656,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>ELCR.MI</t>
+          <t>ELCR.PA</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -6719,7 +6719,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>500H.MI</t>
+          <t>S500.PA</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -6782,7 +6782,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>GOVA.MI</t>
+          <t>EGOV.PA</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -6845,7 +6845,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>X35E.MI</t>
+          <t>EGV5.DE</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -6971,7 +6971,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>X15E.MI</t>
+          <t>E15G.DE</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -7097,7 +7097,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>MA35.MI</t>
+          <t>MA35.PA</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -7160,7 +7160,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>AM3A.MI</t>
+          <t>AM3A.PA</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -7286,7 +7286,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>EFRN.MI</t>
+          <t>EFRN.DE</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -7349,7 +7349,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>USYH.MI</t>
+          <t>LYXE.DE</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -7412,7 +7412,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>X1G.MI</t>
+          <t>X13G.PA</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -7475,7 +7475,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>MWRD.MI</t>
+          <t>MGT.PA</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -7538,7 +7538,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>X13E.MI</t>
+          <t>MTA.PA</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -7601,7 +7601,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>MA13.MI</t>
+          <t>MA13.PA</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>STHY.MI</t>
+          <t>YIEL.L</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -7727,7 +7727,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>ECRP.MI</t>
+          <t>ECR3.DE</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -7790,7 +7790,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>USYH.MI</t>
+          <t>USHY.L</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -7853,7 +7853,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>FINSW.MI</t>
+          <t>FINSW.PA</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -7916,7 +7916,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>C40.MI</t>
+          <t>CACC.PA</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -7979,7 +7979,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>LWCR.MI</t>
+          <t>LWCR.DE</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -8042,7 +8042,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>AFLT.MI</t>
+          <t>AFLT.PA</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -8105,7 +8105,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>ERNA.MI</t>
+          <t>YCSH.DE</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -8168,7 +8168,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>C3M.MI</t>
+          <t>C3M.PA</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -8231,7 +8231,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>CSH.MI</t>
+          <t>CSH.PA</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -8357,7 +8357,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>AGGH.MI</t>
+          <t>GAGG.PA</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -8420,7 +8420,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>CORP.MI</t>
+          <t>UBBB.PA</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -8546,7 +8546,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>EPRE.MI</t>
+          <t>EPRE.L</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -8609,7 +8609,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>CRB.MI</t>
+          <t>COMH.MI</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -8672,7 +8672,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>USYH.MI</t>
+          <t>UHYC.L</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -8798,7 +8798,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>AGEB.MI</t>
+          <t>AGEB.PA</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -8987,7 +8987,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>500H.MI</t>
+          <t>500H.PA</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -9050,7 +9050,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>LEMB.MI</t>
+          <t>LEMB.L</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -9113,7 +9113,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>500H.MI</t>
+          <t>500.PA</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -9176,7 +9176,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>USIH.MI</t>
+          <t>USIH.PA</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -9239,7 +9239,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>PRAP.MI</t>
+          <t>PRAP.SW</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -9302,7 +9302,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>GGOV.MI</t>
+          <t>GOVH.PA</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -9365,7 +9365,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>USIG.MI</t>
+          <t>USIG.L</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -9428,7 +9428,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>GGOV.MI</t>
+          <t>GGOV.PA</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -9491,7 +9491,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>USIC.MI</t>
+          <t>USIC.L</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -9743,7 +9743,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>CC1.MI</t>
+          <t>LHKG.DE</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -9806,7 +9806,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>CC1.MI</t>
+          <t>ASI.PA</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -9932,7 +9932,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>USEE.MI</t>
+          <t>USEE.AS</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -9995,7 +9995,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>SADU.MI</t>
+          <t>SADU.PA</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -10058,7 +10058,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>CATH.MI</t>
+          <t>WLSC.PA</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -10121,7 +10121,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>INDI.MI</t>
+          <t>INR.PA</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -10184,7 +10184,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>INS.MI</t>
+          <t>LIRU.DE</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -10247,7 +10247,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>INDI.MI</t>
+          <t>CI2.PA</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>GLUX.MI</t>
+          <t>GLUX.PA</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -10373,7 +10373,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>UST.MI</t>
+          <t>NDXH.PA</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -10436,7 +10436,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>UST.MI</t>
+          <t>UST.PA</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -10499,7 +10499,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>DTEC.MI</t>
+          <t>UNIC.L</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -10562,7 +10562,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>UST.MI</t>
+          <t>UST.PA</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -10625,7 +10625,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>UST.MI</t>
+          <t>ANX.PA</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -10688,7 +10688,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>FOOD.MI</t>
+          <t>LTVL.DE</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -10751,7 +10751,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>GENY.MI</t>
+          <t>GENY.L</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -10814,7 +10814,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>GOAI.MI</t>
+          <t>GOAI.PA</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -10877,7 +10877,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>INDO.MI</t>
+          <t>INDO.PA</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -10940,7 +10940,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>WTEC.MI</t>
+          <t>TNOW.PA</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -11003,7 +11003,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>DIGE.MI</t>
+          <t>DIGE.L</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -11066,7 +11066,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>DFNS.MI</t>
+          <t>DEFS.PA</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -11129,7 +11129,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>PHAU.MI</t>
+          <t>PHAU.L</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -11192,7 +11192,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>PHAG.MI</t>
+          <t>PHAG.L</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -11255,7 +11255,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>VWCE.MI</t>
+          <t>VWRA.L</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -11318,7 +11318,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>IWDP.MI</t>
+          <t>IASP.SW</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -11381,7 +11381,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>IPRP.MI</t>
+          <t>IWDP.SW</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -11444,7 +11444,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>INRG.MI</t>
+          <t>INRG.SW</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -11570,7 +11570,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>CSCA.MI</t>
+          <t>SXR2.DE</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -11633,7 +11633,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>INFR.MI</t>
+          <t>IQQI.DE</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -11696,7 +11696,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>IBTM.MI</t>
+          <t>IBGX.AS</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -11880,7 +11880,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>VHYL.MI</t>
+          <t>VHYL.L</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -12170,7 +12170,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>LTAM.MI</t>
+          <t>LTAM.L</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -12228,7 +12228,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>EMVL.MI</t>
+          <t>EMVL.L</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -12349,7 +12349,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>EMID.MI</t>
+          <t>EMID.L</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -12407,7 +12407,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>AIGI.MI</t>
+          <t>AIGI.L</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -12470,7 +12470,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>COPA.MI</t>
+          <t>COPA.L</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -12533,7 +12533,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>ALUM.MI</t>
+          <t>ALUM.L</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -12591,7 +12591,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>ZINC.MI</t>
+          <t>ZINC.L</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -12649,7 +12649,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>MINE.MI</t>
+          <t>COPM.AS</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -12712,7 +12712,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>BATG.MI</t>
+          <t>BATG.L</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -12770,7 +12770,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>IPRV.MI</t>
+          <t>IDPE.L</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -12833,7 +12833,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>XLPE.MI</t>
+          <t>XLPE.L</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -12891,7 +12891,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>XEON.MI</t>
+          <t>XEON.DE</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -12954,7 +12954,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>IEGE.MI</t>
+          <t>DLTM.L</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -13017,7 +13017,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>IUSE.MI</t>
+          <t>IUSE.L</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -13080,7 +13080,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>IWDE.MI</t>
+          <t>IWDE.L</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">

</xml_diff>

<commit_message>
Fix: Add 16 missing ETF with ticker resolution + update EUEB.DE
Resolved ISIN-ticker mappings for 16 ETF that were in database but missing
from Excel (tracked via ticker fallback). Added proper ticket symbols:
- 4 on Singapore (.SG): LU2037748345, IE000LAP5Z18, LU2240851688, LU2109787635
- 3 on Frankfurt (.DE): IE000XL4IXU1, XMGA.DE, WOEE.DE
- 3 on Milan (.MI): WLDX.MI, LVO.MI, CSSPX.MI
- 2 on Tel Aviv (.IL): 0XCK.IL, 0E2B.IL
- 2 on Paris (.PA): MAA.PA, PLAN.PA
- 2 on Swiss (.SW): WATC.SW, CSBGU7.SW
- 1 on London (.L): IART.L

Also updated IE000BUIVY49 ticker from ECEA.DE to EUEB.DE (Yahoo Finance current).
Total ETF now: 242 (was 226). Monitor will auto-download missing prices.

Removed 2 delisting (LU1681048127, LU1681041523) from scope.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O227"/>
+  <dimension ref="A1:O243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4829,7 +4829,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ECEA.DE</t>
+          <t>EUEB.DE</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -14367,6 +14367,950 @@
       <c r="O227" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="n">
+        <v>0</v>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>0XCK.IL</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Multi Units France - Lyxor FTSE Italia Mid Cap PIR</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Azionari Italia</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>Tel Aviv</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G228" t="n">
+        <v>0</v>
+      </c>
+      <c r="H228" t="n">
+        <v>0</v>
+      </c>
+      <c r="I228" t="n">
+        <v>0</v>
+      </c>
+      <c r="J228" t="n">
+        <v>0</v>
+      </c>
+      <c r="K228" t="n">
+        <v>0</v>
+      </c>
+      <c r="L228" t="n">
+        <v>0</v>
+      </c>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N228" t="inlineStr"/>
+      <c r="O228" t="inlineStr">
+        <is>
+          <t>FR0011758085</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="n">
+        <v>0</v>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>WLDX.MI</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Amundi MSCI World Ex USA Screened UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Azionari Sviluppati</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>Milano</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G229" t="n">
+        <v>0</v>
+      </c>
+      <c r="H229" t="n">
+        <v>0</v>
+      </c>
+      <c r="I229" t="n">
+        <v>0</v>
+      </c>
+      <c r="J229" t="n">
+        <v>0</v>
+      </c>
+      <c r="K229" t="n">
+        <v>0</v>
+      </c>
+      <c r="L229" t="n">
+        <v>0</v>
+      </c>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N229" t="inlineStr"/>
+      <c r="O229" t="inlineStr">
+        <is>
+          <t>FR0013209921</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n">
+        <v>0</v>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>MAA.PA</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Amundi Euro Highest Rated Macro-Weighted Governmen</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Obbligazionari Governo</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Parigi</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G230" t="n">
+        <v>0</v>
+      </c>
+      <c r="H230" t="n">
+        <v>0</v>
+      </c>
+      <c r="I230" t="n">
+        <v>0</v>
+      </c>
+      <c r="J230" t="n">
+        <v>0</v>
+      </c>
+      <c r="K230" t="n">
+        <v>0</v>
+      </c>
+      <c r="L230" t="n">
+        <v>0</v>
+      </c>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N230" t="inlineStr"/>
+      <c r="O230" t="inlineStr">
+        <is>
+          <t>LU1287023342</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="n">
+        <v>0</v>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>LU2037748345.SG</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Amundi MSCI Smart Cities ESG Sc</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Azionari Tematici</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Singapur</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G231" t="n">
+        <v>0</v>
+      </c>
+      <c r="H231" t="n">
+        <v>0</v>
+      </c>
+      <c r="I231" t="n">
+        <v>0</v>
+      </c>
+      <c r="J231" t="n">
+        <v>0</v>
+      </c>
+      <c r="K231" t="n">
+        <v>0</v>
+      </c>
+      <c r="L231" t="n">
+        <v>0</v>
+      </c>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N231" t="inlineStr"/>
+      <c r="O231" t="inlineStr">
+        <is>
+          <t>LU2037748345</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>0</v>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>IE000LAP5Z18.SG</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P 500 Equal Weight ESG</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Azionari USA</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Singapur</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G232" t="n">
+        <v>0</v>
+      </c>
+      <c r="H232" t="n">
+        <v>0</v>
+      </c>
+      <c r="I232" t="n">
+        <v>0</v>
+      </c>
+      <c r="J232" t="n">
+        <v>0</v>
+      </c>
+      <c r="K232" t="n">
+        <v>0</v>
+      </c>
+      <c r="L232" t="n">
+        <v>0</v>
+      </c>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N232" t="inlineStr"/>
+      <c r="O232" t="inlineStr">
+        <is>
+          <t>IE000LAP5Z18</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>0</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>0E2B.IL</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>LYXOR Index Fund - Lyxor Smart Overnight Return</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Liquidità</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Tel Aviv</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G233" t="n">
+        <v>0</v>
+      </c>
+      <c r="H233" t="n">
+        <v>0</v>
+      </c>
+      <c r="I233" t="n">
+        <v>0</v>
+      </c>
+      <c r="J233" t="n">
+        <v>0</v>
+      </c>
+      <c r="K233" t="n">
+        <v>0</v>
+      </c>
+      <c r="L233" t="n">
+        <v>0</v>
+      </c>
+      <c r="M233" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N233" t="inlineStr"/>
+      <c r="O233" t="inlineStr">
+        <is>
+          <t>LU1190417599</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>0</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>XMGA.DE</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Amundi MSCI USA Ex Mega Cap UCITS ETF USD Accumula</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Azionari USA</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Francoforte</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G234" t="n">
+        <v>0</v>
+      </c>
+      <c r="H234" t="n">
+        <v>0</v>
+      </c>
+      <c r="I234" t="n">
+        <v>0</v>
+      </c>
+      <c r="J234" t="n">
+        <v>0</v>
+      </c>
+      <c r="K234" t="n">
+        <v>0</v>
+      </c>
+      <c r="L234" t="n">
+        <v>0</v>
+      </c>
+      <c r="M234" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N234" t="inlineStr"/>
+      <c r="O234" t="inlineStr">
+        <is>
+          <t>IE000XL4IXU1</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>0</v>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>PLAN.PA</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Multi Units Luxembourg - Lyxor Corporate Green Bon</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Obbligazionari Corporate</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Parigi</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G235" t="n">
+        <v>0</v>
+      </c>
+      <c r="H235" t="n">
+        <v>0</v>
+      </c>
+      <c r="I235" t="n">
+        <v>0</v>
+      </c>
+      <c r="J235" t="n">
+        <v>0</v>
+      </c>
+      <c r="K235" t="n">
+        <v>0</v>
+      </c>
+      <c r="L235" t="n">
+        <v>0</v>
+      </c>
+      <c r="M235" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N235" t="inlineStr"/>
+      <c r="O235" t="inlineStr">
+        <is>
+          <t>LU2370241684</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>0</v>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>IART.L</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>iShares AI Innovation Active UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Azionari Tematici</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Londra</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G236" t="n">
+        <v>0</v>
+      </c>
+      <c r="H236" t="n">
+        <v>0</v>
+      </c>
+      <c r="I236" t="n">
+        <v>0</v>
+      </c>
+      <c r="J236" t="n">
+        <v>0</v>
+      </c>
+      <c r="K236" t="n">
+        <v>0</v>
+      </c>
+      <c r="L236" t="n">
+        <v>0</v>
+      </c>
+      <c r="M236" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N236" t="inlineStr"/>
+      <c r="O236" t="inlineStr">
+        <is>
+          <t>IE000G0E83X3</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>0</v>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>LU2240851688.SG</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Amundi DAX 50 ESG UCITS ETF - E</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Azionari Europa</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>Singapur</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G237" t="n">
+        <v>0</v>
+      </c>
+      <c r="H237" t="n">
+        <v>0</v>
+      </c>
+      <c r="I237" t="n">
+        <v>0</v>
+      </c>
+      <c r="J237" t="n">
+        <v>0</v>
+      </c>
+      <c r="K237" t="n">
+        <v>0</v>
+      </c>
+      <c r="L237" t="n">
+        <v>0</v>
+      </c>
+      <c r="M237" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N237" t="inlineStr"/>
+      <c r="O237" t="inlineStr">
+        <is>
+          <t>LU2240851688</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>0</v>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>LU2109787635.SG</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Amundi Index MSCI EMU SRI PBA U</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Azionari Europa</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>Singapur</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G238" t="n">
+        <v>0</v>
+      </c>
+      <c r="H238" t="n">
+        <v>0</v>
+      </c>
+      <c r="I238" t="n">
+        <v>0</v>
+      </c>
+      <c r="J238" t="n">
+        <v>0</v>
+      </c>
+      <c r="K238" t="n">
+        <v>0</v>
+      </c>
+      <c r="L238" t="n">
+        <v>0</v>
+      </c>
+      <c r="M238" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N238" t="inlineStr"/>
+      <c r="O238" t="inlineStr">
+        <is>
+          <t>LU2109787635</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>0</v>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>WATC.SW</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Amundi MSCI Water UCITS ETF Acc</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Azionari Tematici</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>Svizzera</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G239" t="n">
+        <v>0</v>
+      </c>
+      <c r="H239" t="n">
+        <v>0</v>
+      </c>
+      <c r="I239" t="n">
+        <v>0</v>
+      </c>
+      <c r="J239" t="n">
+        <v>0</v>
+      </c>
+      <c r="K239" t="n">
+        <v>0</v>
+      </c>
+      <c r="L239" t="n">
+        <v>0</v>
+      </c>
+      <c r="M239" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N239" t="inlineStr"/>
+      <c r="O239" t="inlineStr">
+        <is>
+          <t>FR0014002CH1</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>0</v>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>CSBGU7.SW</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>iShares VII PLC - iShares VII PLC - iShares $ Trea</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Obbligazionari Governo</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Svizzera</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G240" t="n">
+        <v>0</v>
+      </c>
+      <c r="H240" t="n">
+        <v>0</v>
+      </c>
+      <c r="I240" t="n">
+        <v>0</v>
+      </c>
+      <c r="J240" t="n">
+        <v>0</v>
+      </c>
+      <c r="K240" t="n">
+        <v>0</v>
+      </c>
+      <c r="L240" t="n">
+        <v>0</v>
+      </c>
+      <c r="M240" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N240" t="inlineStr"/>
+      <c r="O240" t="inlineStr">
+        <is>
+          <t>IE00B3VWN393</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>0</v>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>LVO.MI</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Amundi S&amp;P 500 VIX Futures Enhanced Roll UCITS ETF</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Azionari Alternativi</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>Milano</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G241" t="n">
+        <v>0</v>
+      </c>
+      <c r="H241" t="n">
+        <v>0</v>
+      </c>
+      <c r="I241" t="n">
+        <v>0</v>
+      </c>
+      <c r="J241" t="n">
+        <v>0</v>
+      </c>
+      <c r="K241" t="n">
+        <v>0</v>
+      </c>
+      <c r="L241" t="n">
+        <v>0</v>
+      </c>
+      <c r="M241" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N241" t="inlineStr"/>
+      <c r="O241" t="inlineStr">
+        <is>
+          <t>LU0832435464</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>0</v>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>CSSPX.MI</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Azionari USA</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>Milano</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G242" t="n">
+        <v>0</v>
+      </c>
+      <c r="H242" t="n">
+        <v>0</v>
+      </c>
+      <c r="I242" t="n">
+        <v>0</v>
+      </c>
+      <c r="J242" t="n">
+        <v>0</v>
+      </c>
+      <c r="K242" t="n">
+        <v>0</v>
+      </c>
+      <c r="L242" t="n">
+        <v>0</v>
+      </c>
+      <c r="M242" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N242" t="inlineStr"/>
+      <c r="O242" t="inlineStr">
+        <is>
+          <t>IE00B5BMR087</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>0</v>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>WOEE.DE</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>iShares World Equity Enhanced Active UCITS ETF USD</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Azionari Sviluppati</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>Francoforte</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G243" t="n">
+        <v>0</v>
+      </c>
+      <c r="H243" t="n">
+        <v>0</v>
+      </c>
+      <c r="I243" t="n">
+        <v>0</v>
+      </c>
+      <c r="J243" t="n">
+        <v>0</v>
+      </c>
+      <c r="K243" t="n">
+        <v>0</v>
+      </c>
+      <c r="L243" t="n">
+        <v>0</v>
+      </c>
+      <c r="M243" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="N243" t="inlineStr"/>
+      <c r="O243" t="inlineStr">
+        <is>
+          <t>IE000D8XC064</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: Resolve Singapur ETF ticker issues + remove irrisolti
Ticker resolution for Singapore-listed ETF:
- LU2240851688 (Amundi DAX 50 ESG): .SG → EXS1.DE (Frankfurt) ✓
- LU2109787635 (Amundi MSCI EMU SRI): .SG → MSEU.L (London) ✓

Removed 2 irrisolti (no alternative ticker found):
- LU2037748345 (Amundi MSCI Smart Cities ESG) - only .SG available
- IE000LAP5Z18 (Amundi S&P 500 Equal Weight ESG) - only .SG available

Total ETF now: 240 (was 242). Monitor will auto-update next run with resolved tickers.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O243"/>
+  <dimension ref="A1:O241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -667,7 +667,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -982,7 +982,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1045,7 +1045,7 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1108,7 +1108,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1171,7 +1171,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1297,7 +1297,7 @@
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1360,7 +1360,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1486,7 +1486,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1738,7 +1738,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1927,7 +1927,7 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1990,7 +1990,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2116,7 +2116,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2305,7 +2305,7 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2431,7 +2431,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2620,7 +2620,7 @@
     </row>
     <row r="35">
       <c r="A35" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2809,7 +2809,7 @@
     </row>
     <row r="38">
       <c r="A38" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -2872,7 +2872,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -2935,7 +2935,7 @@
     </row>
     <row r="40">
       <c r="A40" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3313,7 +3313,7 @@
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -3502,7 +3502,7 @@
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -3754,7 +3754,7 @@
     </row>
     <row r="53">
       <c r="A53" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -4006,7 +4006,7 @@
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -4132,7 +4132,7 @@
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -4447,7 +4447,7 @@
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
     </row>
     <row r="66">
       <c r="A66" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -4762,7 +4762,7 @@
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -4951,7 +4951,7 @@
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -5077,7 +5077,7 @@
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -5518,7 +5518,7 @@
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -5581,7 +5581,7 @@
     </row>
     <row r="82">
       <c r="A82" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -5707,7 +5707,7 @@
     </row>
     <row r="84">
       <c r="A84" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -5833,7 +5833,7 @@
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
@@ -6085,7 +6085,7 @@
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
@@ -6337,7 +6337,7 @@
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -6526,7 +6526,7 @@
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -6778,7 +6778,7 @@
     </row>
     <row r="101">
       <c r="A101" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -6904,7 +6904,7 @@
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -8353,7 +8353,7 @@
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -9487,7 +9487,7 @@
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
@@ -9550,7 +9550,7 @@
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
@@ -10369,7 +10369,7 @@
     </row>
     <row r="158">
       <c r="A158" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -10621,7 +10621,7 @@
     </row>
     <row r="162">
       <c r="A162" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
@@ -10810,7 +10810,7 @@
     </row>
     <row r="165">
       <c r="A165" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
@@ -10999,7 +10999,7 @@
     </row>
     <row r="168">
       <c r="A168" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -11188,7 +11188,7 @@
     </row>
     <row r="171">
       <c r="A171" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
@@ -11629,7 +11629,7 @@
     </row>
     <row r="178">
       <c r="A178" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
@@ -12161,7 +12161,7 @@
     </row>
     <row r="187">
       <c r="A187" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -12403,7 +12403,7 @@
     </row>
     <row r="191">
       <c r="A191" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
@@ -12703,7 +12703,7 @@
     </row>
     <row r="196">
       <c r="A196" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
@@ -12887,7 +12887,7 @@
     </row>
     <row r="199">
       <c r="A199" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B199" t="inlineStr">
         <is>
@@ -12950,7 +12950,7 @@
     </row>
     <row r="200">
       <c r="A200" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B200" t="inlineStr">
         <is>
@@ -13202,7 +13202,7 @@
     </row>
     <row r="204">
       <c r="A204" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
@@ -14422,7 +14422,6 @@
           <t>WATCH</t>
         </is>
       </c>
-      <c r="N228" t="inlineStr"/>
       <c r="O228" t="inlineStr">
         <is>
           <t>FR0011758085</t>
@@ -14481,7 +14480,6 @@
           <t>WATCH</t>
         </is>
       </c>
-      <c r="N229" t="inlineStr"/>
       <c r="O229" t="inlineStr">
         <is>
           <t>FR0013209921</t>
@@ -14540,7 +14538,6 @@
           <t>WATCH</t>
         </is>
       </c>
-      <c r="N230" t="inlineStr"/>
       <c r="O230" t="inlineStr">
         <is>
           <t>LU1287023342</t>
@@ -14553,27 +14550,27 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>LU2037748345.SG</t>
+          <t>0E2B.IL</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Amundi MSCI Smart Cities ESG Sc</t>
+          <t>LYXOR Index Fund - Lyxor Smart Overnight Return</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>Azionari Tematici</t>
+          <t>Liquidità</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Singapur</t>
+          <t>Tel Aviv</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="G231" t="n">
@@ -14599,10 +14596,9 @@
           <t>WATCH</t>
         </is>
       </c>
-      <c r="N231" t="inlineStr"/>
       <c r="O231" t="inlineStr">
         <is>
-          <t>LU2037748345</t>
+          <t>LU1190417599</t>
         </is>
       </c>
     </row>
@@ -14612,12 +14608,12 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>IE000LAP5Z18.SG</t>
+          <t>XMGA.DE</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P 500 Equal Weight ESG</t>
+          <t>Amundi MSCI USA Ex Mega Cap UCITS ETF USD Accumula</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
@@ -14627,7 +14623,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Singapur</t>
+          <t>Francoforte</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
@@ -14658,10 +14654,9 @@
           <t>WATCH</t>
         </is>
       </c>
-      <c r="N232" t="inlineStr"/>
       <c r="O232" t="inlineStr">
         <is>
-          <t>IE000LAP5Z18</t>
+          <t>IE000XL4IXU1</t>
         </is>
       </c>
     </row>
@@ -14671,22 +14666,22 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>0E2B.IL</t>
+          <t>PLAN.PA</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>LYXOR Index Fund - Lyxor Smart Overnight Return</t>
+          <t>Multi Units Luxembourg - Lyxor Corporate Green Bon</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>Liquidità</t>
+          <t>Obbligazionari Corporate</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>Tel Aviv</t>
+          <t>Parigi</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
@@ -14717,10 +14712,9 @@
           <t>WATCH</t>
         </is>
       </c>
-      <c r="N233" t="inlineStr"/>
       <c r="O233" t="inlineStr">
         <is>
-          <t>LU1190417599</t>
+          <t>LU2370241684</t>
         </is>
       </c>
     </row>
@@ -14730,22 +14724,22 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>XMGA.DE</t>
+          <t>IART.L</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Amundi MSCI USA Ex Mega Cap UCITS ETF USD Accumula</t>
+          <t>iShares AI Innovation Active UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>Azionari USA</t>
+          <t>Azionari Tematici</t>
         </is>
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>Francoforte</t>
+          <t>Londra</t>
         </is>
       </c>
       <c r="F234" t="inlineStr">
@@ -14776,10 +14770,9 @@
           <t>WATCH</t>
         </is>
       </c>
-      <c r="N234" t="inlineStr"/>
       <c r="O234" t="inlineStr">
         <is>
-          <t>IE000XL4IXU1</t>
+          <t>IE000G0E83X3</t>
         </is>
       </c>
     </row>
@@ -14789,22 +14782,22 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>PLAN.PA</t>
+          <t>EXS1.DE</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Multi Units Luxembourg - Lyxor Corporate Green Bon</t>
+          <t>Amundi DAX 50 ESG UCITS ETF - E</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>Obbligazionari Corporate</t>
+          <t>Azionari Europa</t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Parigi</t>
+          <t>Singapur</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
@@ -14835,10 +14828,9 @@
           <t>WATCH</t>
         </is>
       </c>
-      <c r="N235" t="inlineStr"/>
       <c r="O235" t="inlineStr">
         <is>
-          <t>LU2370241684</t>
+          <t>LU2240851688</t>
         </is>
       </c>
     </row>
@@ -14848,27 +14840,27 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>IART.L</t>
+          <t>MSEU.L</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>iShares AI Innovation Active UCITS ETF USD (Acc)</t>
+          <t>Amundi Index MSCI EMU SRI PBA U</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>Azionari Tematici</t>
+          <t>Azionari Europa</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Londra</t>
+          <t>Singapur</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="G236" t="n">
@@ -14894,10 +14886,9 @@
           <t>WATCH</t>
         </is>
       </c>
-      <c r="N236" t="inlineStr"/>
       <c r="O236" t="inlineStr">
         <is>
-          <t>IE000G0E83X3</t>
+          <t>LU2109787635</t>
         </is>
       </c>
     </row>
@@ -14907,22 +14898,22 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>LU2240851688.SG</t>
+          <t>WATC.SW</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>Amundi DAX 50 ESG UCITS ETF - E</t>
+          <t>Amundi MSCI Water UCITS ETF Acc</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>Azionari Europa</t>
+          <t>Azionari Tematici</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Singapur</t>
+          <t>Svizzera</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
@@ -14953,10 +14944,9 @@
           <t>WATCH</t>
         </is>
       </c>
-      <c r="N237" t="inlineStr"/>
       <c r="O237" t="inlineStr">
         <is>
-          <t>LU2240851688</t>
+          <t>FR0014002CH1</t>
         </is>
       </c>
     </row>
@@ -14966,27 +14956,27 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>LU2109787635.SG</t>
+          <t>CSBGU7.SW</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Amundi Index MSCI EMU SRI PBA U</t>
+          <t>iShares VII PLC - iShares VII PLC - iShares $ Trea</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>Azionari Europa</t>
+          <t>Obbligazionari Governo</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Singapur</t>
+          <t>Svizzera</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G238" t="n">
@@ -15012,10 +15002,9 @@
           <t>WATCH</t>
         </is>
       </c>
-      <c r="N238" t="inlineStr"/>
       <c r="O238" t="inlineStr">
         <is>
-          <t>LU2109787635</t>
+          <t>IE00B3VWN393</t>
         </is>
       </c>
     </row>
@@ -15025,22 +15014,22 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>WATC.SW</t>
+          <t>LVO.MI</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Amundi MSCI Water UCITS ETF Acc</t>
+          <t>Amundi S&amp;P 500 VIX Futures Enhanced Roll UCITS ETF</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Azionari Tematici</t>
+          <t>Azionari Alternativi</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>Svizzera</t>
+          <t>Milano</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
@@ -15071,10 +15060,9 @@
           <t>WATCH</t>
         </is>
       </c>
-      <c r="N239" t="inlineStr"/>
       <c r="O239" t="inlineStr">
         <is>
-          <t>FR0014002CH1</t>
+          <t>LU0832435464</t>
         </is>
       </c>
     </row>
@@ -15084,22 +15072,22 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>CSBGU7.SW</t>
+          <t>CSSPX.MI</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>iShares VII PLC - iShares VII PLC - iShares $ Trea</t>
+          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>Obbligazionari Governo</t>
+          <t>Azionari USA</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>Svizzera</t>
+          <t>Milano</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
@@ -15130,10 +15118,9 @@
           <t>WATCH</t>
         </is>
       </c>
-      <c r="N240" t="inlineStr"/>
       <c r="O240" t="inlineStr">
         <is>
-          <t>IE00B3VWN393</t>
+          <t>IE00B5BMR087</t>
         </is>
       </c>
     </row>
@@ -15143,27 +15130,27 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>LVO.MI</t>
+          <t>WOEE.DE</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Amundi S&amp;P 500 VIX Futures Enhanced Roll UCITS ETF</t>
+          <t>iShares World Equity Enhanced Active UCITS ETF USD</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>Azionari Alternativi</t>
+          <t>Azionari Sviluppati</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>Milano</t>
+          <t>Francoforte</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G241" t="n">
@@ -15189,126 +15176,7 @@
           <t>WATCH</t>
         </is>
       </c>
-      <c r="N241" t="inlineStr"/>
       <c r="O241" t="inlineStr">
-        <is>
-          <t>LU0832435464</t>
-        </is>
-      </c>
-    </row>
-    <row r="242">
-      <c r="A242" t="n">
-        <v>0</v>
-      </c>
-      <c r="B242" t="inlineStr">
-        <is>
-          <t>CSSPX.MI</t>
-        </is>
-      </c>
-      <c r="C242" t="inlineStr">
-        <is>
-          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
-        </is>
-      </c>
-      <c r="D242" t="inlineStr">
-        <is>
-          <t>Azionari USA</t>
-        </is>
-      </c>
-      <c r="E242" t="inlineStr">
-        <is>
-          <t>Milano</t>
-        </is>
-      </c>
-      <c r="F242" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G242" t="n">
-        <v>0</v>
-      </c>
-      <c r="H242" t="n">
-        <v>0</v>
-      </c>
-      <c r="I242" t="n">
-        <v>0</v>
-      </c>
-      <c r="J242" t="n">
-        <v>0</v>
-      </c>
-      <c r="K242" t="n">
-        <v>0</v>
-      </c>
-      <c r="L242" t="n">
-        <v>0</v>
-      </c>
-      <c r="M242" t="inlineStr">
-        <is>
-          <t>WATCH</t>
-        </is>
-      </c>
-      <c r="N242" t="inlineStr"/>
-      <c r="O242" t="inlineStr">
-        <is>
-          <t>IE00B5BMR087</t>
-        </is>
-      </c>
-    </row>
-    <row r="243">
-      <c r="A243" t="n">
-        <v>0</v>
-      </c>
-      <c r="B243" t="inlineStr">
-        <is>
-          <t>WOEE.DE</t>
-        </is>
-      </c>
-      <c r="C243" t="inlineStr">
-        <is>
-          <t>iShares World Equity Enhanced Active UCITS ETF USD</t>
-        </is>
-      </c>
-      <c r="D243" t="inlineStr">
-        <is>
-          <t>Azionari Sviluppati</t>
-        </is>
-      </c>
-      <c r="E243" t="inlineStr">
-        <is>
-          <t>Francoforte</t>
-        </is>
-      </c>
-      <c r="F243" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G243" t="n">
-        <v>0</v>
-      </c>
-      <c r="H243" t="n">
-        <v>0</v>
-      </c>
-      <c r="I243" t="n">
-        <v>0</v>
-      </c>
-      <c r="J243" t="n">
-        <v>0</v>
-      </c>
-      <c r="K243" t="n">
-        <v>0</v>
-      </c>
-      <c r="L243" t="n">
-        <v>0</v>
-      </c>
-      <c r="M243" t="inlineStr">
-        <is>
-          <t>WATCH</t>
-        </is>
-      </c>
-      <c r="N243" t="inlineStr"/>
-      <c r="O243" t="inlineStr">
         <is>
           <t>IE000D8XC064</t>
         </is>

</xml_diff>

<commit_message>
Cleanup: Remove obsolete Directa and Config Refactor Excel files
ETF_Monitor_Directa_Completo_2026.xlsx was a reference file with 144 ISIN,
all of which are already in etf_monitoraggio.xlsx. Our monitoring file is
now more complete (152 ISIN vs 144 in Directa) and uses correct ticker
resolution. Removed both this and the Config Refactor file as obsolete.

Keeping etf_monitoraggio.xlsx as single source of truth.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ETF" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ETF" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1927,7 +1927,7 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2809,7 +2809,7 @@
     </row>
     <row r="38">
       <c r="A38" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
     </row>
     <row r="66">
       <c r="A66" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -4888,7 +4888,7 @@
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -5707,7 +5707,7 @@
     </row>
     <row r="84">
       <c r="A84" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -10180,7 +10180,7 @@
     </row>
     <row r="155">
       <c r="A155" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
@@ -13877,7 +13877,7 @@
     </row>
     <row r="217">
       <c r="A217" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B217" t="inlineStr">
         <is>
@@ -13922,7 +13922,7 @@
     </row>
     <row r="218">
       <c r="A218" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B218" t="inlineStr">
         <is>
@@ -13967,7 +13967,7 @@
     </row>
     <row r="219">
       <c r="A219" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B219" t="inlineStr">
         <is>
@@ -14012,7 +14012,7 @@
     </row>
     <row r="220">
       <c r="A220" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B220" t="inlineStr">
         <is>
@@ -14057,7 +14057,7 @@
     </row>
     <row r="221">
       <c r="A221" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B221" t="inlineStr">
         <is>
@@ -14102,7 +14102,7 @@
     </row>
     <row r="222">
       <c r="A222" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B222" t="inlineStr">
         <is>
@@ -14147,7 +14147,7 @@
     </row>
     <row r="223">
       <c r="A223" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B223" t="inlineStr">
         <is>
@@ -14192,7 +14192,7 @@
     </row>
     <row r="224">
       <c r="A224" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B224" t="inlineStr">
         <is>
@@ -14237,7 +14237,7 @@
     </row>
     <row r="225">
       <c r="A225" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B225" t="inlineStr">
         <is>
@@ -14282,7 +14282,7 @@
     </row>
     <row r="226">
       <c r="A226" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B226" t="inlineStr">
         <is>
@@ -14327,7 +14327,7 @@
     </row>
     <row r="227">
       <c r="A227" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B227" t="inlineStr">
         <is>
@@ -14372,7 +14372,7 @@
     </row>
     <row r="228">
       <c r="A228" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B228" t="inlineStr">
         <is>
@@ -14430,7 +14430,7 @@
     </row>
     <row r="229">
       <c r="A229" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B229" t="inlineStr">
         <is>
@@ -14488,7 +14488,7 @@
     </row>
     <row r="230">
       <c r="A230" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B230" t="inlineStr">
         <is>
@@ -14546,7 +14546,7 @@
     </row>
     <row r="231">
       <c r="A231" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B231" t="inlineStr">
         <is>
@@ -14604,7 +14604,7 @@
     </row>
     <row r="232">
       <c r="A232" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B232" t="inlineStr">
         <is>
@@ -14662,7 +14662,7 @@
     </row>
     <row r="233">
       <c r="A233" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B233" t="inlineStr">
         <is>
@@ -14720,7 +14720,7 @@
     </row>
     <row r="234">
       <c r="A234" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B234" t="inlineStr">
         <is>
@@ -14778,7 +14778,7 @@
     </row>
     <row r="235">
       <c r="A235" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B235" t="inlineStr">
         <is>
@@ -14836,7 +14836,7 @@
     </row>
     <row r="236">
       <c r="A236" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B236" t="inlineStr">
         <is>
@@ -14894,7 +14894,7 @@
     </row>
     <row r="237">
       <c r="A237" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B237" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix: Strato 3 Filtri — Applica TUTTI i 5/6 (non solo == 5)
PROBLEMA: Il filtro ADX+dist si applicava solo quando buy_count == 5 esattamente.
Asset con 5/6 passavano perché potevano avere buy_count=5.0 (float).

SOLUZIONE: Riscrivere il filtro per applicarsi a TUTTI i buy_count < 6:
- Controlla buy_count < 6 (applica a 5/6, 4/6, ecc.)
- Se ADX < adx_entry OU dist > max → L2 (Watchlist)
- Se passa ADX+dist → valuta EMA slope
- Se EMA slope OK → L1
- Altrimenti → L2

Risultato atteso: 15 ETF L1 → ~3-5 ETF L1 veri

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -856,7 +856,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1927,7 +1927,7 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2305,7 +2305,7 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2809,7 +2809,7 @@
     </row>
     <row r="38">
       <c r="A38" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3187,7 +3187,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3250,7 +3250,7 @@
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -3439,7 +3439,7 @@
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -3565,7 +3565,7 @@
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -3628,7 +3628,7 @@
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -3691,7 +3691,7 @@
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -4258,7 +4258,7 @@
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -4384,7 +4384,7 @@
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
     </row>
     <row r="66">
       <c r="A66" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -4888,7 +4888,7 @@
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -5203,7 +5203,7 @@
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
@@ -10684,7 +10684,7 @@
     </row>
     <row r="163">
       <c r="A163" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
@@ -11566,7 +11566,7 @@
     </row>
     <row r="177">
       <c r="A177" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
@@ -12259,7 +12259,7 @@
     </row>
     <row r="188">
       <c r="A188" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
@@ -12322,7 +12322,7 @@
     </row>
     <row r="189">
       <c r="A189" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
@@ -12826,7 +12826,7 @@
     </row>
     <row r="197">
       <c r="A197" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
@@ -13942,7 +13942,7 @@
     </row>
     <row r="217">
       <c r="A217" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B217" t="inlineStr">
         <is>
@@ -13987,7 +13987,7 @@
     </row>
     <row r="218">
       <c r="A218" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B218" t="inlineStr">
         <is>
@@ -14032,7 +14032,7 @@
     </row>
     <row r="219">
       <c r="A219" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B219" t="inlineStr">
         <is>
@@ -14077,7 +14077,7 @@
     </row>
     <row r="220">
       <c r="A220" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B220" t="inlineStr">
         <is>
@@ -14122,7 +14122,7 @@
     </row>
     <row r="221">
       <c r="A221" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B221" t="inlineStr">
         <is>
@@ -14167,7 +14167,7 @@
     </row>
     <row r="222">
       <c r="A222" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B222" t="inlineStr">
         <is>
@@ -14212,7 +14212,7 @@
     </row>
     <row r="223">
       <c r="A223" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B223" t="inlineStr">
         <is>
@@ -14257,7 +14257,7 @@
     </row>
     <row r="224">
       <c r="A224" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B224" t="inlineStr">
         <is>
@@ -14302,7 +14302,7 @@
     </row>
     <row r="225">
       <c r="A225" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B225" t="inlineStr">
         <is>
@@ -14347,7 +14347,7 @@
     </row>
     <row r="226">
       <c r="A226" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B226" t="inlineStr">
         <is>
@@ -14392,7 +14392,7 @@
     </row>
     <row r="227">
       <c r="A227" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B227" t="inlineStr">
         <is>
@@ -15133,7 +15133,7 @@
     </row>
     <row r="240">
       <c r="A240" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B240" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix: Portfolio SL data stale — add ISIN filtering and clear fields during fetch
Backend: /api/portfolio-sl now supports ?isin= query param to filter at database level
Frontend: Clear SL input fields BEFORE fetching new data to prevent stale data visibility

This fixes the bug where switching between portfolio ETFs showed stale data until hard refresh.
Process: When clicking ETF A → clear fields → fetch new data → show ETF A's values

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ETF" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ETF" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -541,7 +541,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -982,7 +982,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1045,7 +1045,7 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1234,7 +1234,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1486,7 +1486,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1549,7 +1549,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1612,7 +1612,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1675,7 +1675,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1864,7 +1864,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2053,7 +2053,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2116,7 +2116,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2179,7 +2179,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2242,7 +2242,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2494,7 +2494,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2557,7 +2557,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2806,7 +2806,7 @@
     </row>
     <row r="38">
       <c r="A38" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -2869,7 +2869,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3058,7 +3058,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3121,7 +3121,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3940,7 +3940,7 @@
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -4255,7 +4255,7 @@
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -4570,7 +4570,7 @@
     </row>
     <row r="66">
       <c r="A66" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -5704,7 +5704,7 @@
     </row>
     <row r="84">
       <c r="A84" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -5893,7 +5893,7 @@
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
@@ -5956,7 +5956,7 @@
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -6586,7 +6586,7 @@
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -6901,7 +6901,7 @@
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -7783,7 +7783,7 @@
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -8350,7 +8350,7 @@
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -8539,7 +8539,7 @@
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -9610,7 +9610,7 @@
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
@@ -9673,7 +9673,7 @@
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
@@ -9736,7 +9736,7 @@
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
@@ -10303,7 +10303,7 @@
     </row>
     <row r="157">
       <c r="A157" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
@@ -10870,7 +10870,7 @@
     </row>
     <row r="166">
       <c r="A166" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
@@ -11437,7 +11437,7 @@
     </row>
     <row r="175">
       <c r="A175" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
@@ -11563,7 +11563,7 @@
     </row>
     <row r="177">
       <c r="A177" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
@@ -11689,7 +11689,7 @@
     </row>
     <row r="179">
       <c r="A179" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -12823,7 +12823,7 @@
     </row>
     <row r="197">
       <c r="A197" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
@@ -13201,7 +13201,7 @@
     </row>
     <row r="203">
       <c r="A203" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
@@ -13264,7 +13264,7 @@
     </row>
     <row r="204">
       <c r="A204" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
@@ -13327,7 +13327,7 @@
     </row>
     <row r="205">
       <c r="A205" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B205" t="inlineStr">
         <is>
@@ -13390,7 +13390,7 @@
     </row>
     <row r="206">
       <c r="A206" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B206" t="inlineStr">
         <is>
@@ -13453,7 +13453,7 @@
     </row>
     <row r="207">
       <c r="A207" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B207" t="inlineStr">
         <is>
@@ -14492,7 +14492,7 @@
     </row>
     <row r="229">
       <c r="A229" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B229" t="inlineStr">
         <is>
@@ -14666,7 +14666,7 @@
     </row>
     <row r="232">
       <c r="A232" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B232" t="inlineStr">
         <is>
@@ -14782,7 +14782,7 @@
     </row>
     <row r="234">
       <c r="A234" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B234" t="inlineStr">
         <is>
@@ -15072,7 +15072,7 @@
     </row>
     <row r="239">
       <c r="A239" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B239" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
FIX: PRIORITÀ 1 — Aggiungere high/low a suggest_level_0() signature
Errore: suggest_level_0() usava 'high' e 'low' senza riceverli come parametri.
Fix: Aggiungere parametri high e low alla firma della funzione.
Passare high/low da analyze_etf() con fallback a close se assenti.

Monitor error risolto: NameError: name 'high' is not defined
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -982,7 +982,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1990,7 +1990,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2680,7 +2680,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -4192,7 +4192,7 @@
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -4381,7 +4381,7 @@
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -4822,7 +4822,7 @@
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -5263,7 +5263,7 @@
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -5452,7 +5452,7 @@
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -5704,7 +5704,7 @@
     </row>
     <row r="84">
       <c r="A84" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -6397,7 +6397,7 @@
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -6460,7 +6460,7 @@
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
@@ -6523,7 +6523,7 @@
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -6586,7 +6586,7 @@
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -6964,7 +6964,7 @@
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -7027,7 +7027,7 @@
     </row>
     <row r="105">
       <c r="A105" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
@@ -7342,7 +7342,7 @@
     </row>
     <row r="110">
       <c r="A110" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -7468,7 +7468,7 @@
     </row>
     <row r="112">
       <c r="A112" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
@@ -7846,7 +7846,7 @@
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -8287,7 +8287,7 @@
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -8665,7 +8665,7 @@
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
@@ -8728,7 +8728,7 @@
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -9169,7 +9169,7 @@
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
@@ -9295,7 +9295,7 @@
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
@@ -9358,7 +9358,7 @@
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
@@ -9421,7 +9421,7 @@
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
@@ -9484,7 +9484,7 @@
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
@@ -9925,7 +9925,7 @@
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -10240,7 +10240,7 @@
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
@@ -10618,7 +10618,7 @@
     </row>
     <row r="162">
       <c r="A162" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
@@ -11122,7 +11122,7 @@
     </row>
     <row r="170">
       <c r="A170" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
@@ -12508,7 +12508,7 @@
     </row>
     <row r="192">
       <c r="A192" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
@@ -12697,7 +12697,7 @@
     </row>
     <row r="195">
       <c r="A195" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
@@ -12823,7 +12823,7 @@
     </row>
     <row r="197">
       <c r="A197" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
@@ -12949,7 +12949,7 @@
     </row>
     <row r="199">
       <c r="A199" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B199" t="inlineStr">
         <is>
@@ -13138,7 +13138,7 @@
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
@@ -13453,7 +13453,7 @@
     </row>
     <row r="207">
       <c r="A207" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B207" t="inlineStr">
         <is>
@@ -13669,7 +13669,7 @@
     </row>
     <row r="211">
       <c r="A211" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B211" t="inlineStr">
         <is>
@@ -14434,7 +14434,7 @@
     </row>
     <row r="228">
       <c r="A228" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B228" t="inlineStr">
         <is>
@@ -14724,7 +14724,7 @@
     </row>
     <row r="233">
       <c r="A233" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B233" t="inlineStr">
         <is>
@@ -14782,7 +14782,7 @@
     </row>
     <row r="234">
       <c r="A234" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B234" t="inlineStr">
         <is>
@@ -15014,7 +15014,7 @@
     </row>
     <row r="238">
       <c r="A238" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B238" t="inlineStr">
         <is>
@@ -15072,7 +15072,7 @@
     </row>
     <row r="239">
       <c r="A239" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B239" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
PRIORITÀ 2 FIX: Rimuovere filtro EMA20 slope — non è nella specifica STEP 3 v4.0
Il vecchio filtro EMA20 slope (>= 0.2% in 10gg) bloccava TUTTI gli ETF a L2.
Questo filtro NON è nella specifica STEP 3 v4.0.

Secondo la specifica, il SOLO filtro dovrebbe essere la 7ª condizione (spazio residuo).

Fix:
- Rimosso il blocco EMA20 slope dalle linee 1311-1323
- Mantiene SOLO la 7ª condizione (a OR b OR squeeze override)
- Codice ora conforme alla specifica

Risultato atteso: L1 dovrebbe ora accettare ETF con 6/6 + 7ª OK.
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -982,7 +982,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -6586,7 +6586,7 @@
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -12697,7 +12697,7 @@
     </row>
     <row r="195">
       <c r="A195" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
@@ -14782,7 +14782,7 @@
     </row>
     <row r="234">
       <c r="A234" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B234" t="inlineStr">
         <is>
@@ -15072,7 +15072,7 @@
     </row>
     <row r="239">
       <c r="A239" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B239" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
DEBUG: Stampa quale condizione L1 fallisce (5/6 case)
Aggiungi debug che stampa esattamente quale tra le 6 condizioni fallisce
quando buy_count < 6. Aiuta a diagnosticare perché L1 rimane vuoto.
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -604,7 +604,7 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -667,7 +667,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -982,7 +982,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1171,7 +1171,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1486,7 +1486,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1927,7 +1927,7 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2116,7 +2116,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2806,7 +2806,7 @@
     </row>
     <row r="38">
       <c r="A38" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -4570,7 +4570,7 @@
     </row>
     <row r="66">
       <c r="A66" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -4885,7 +4885,7 @@
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -5515,7 +5515,7 @@
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -5578,7 +5578,7 @@
     </row>
     <row r="82">
       <c r="A82" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -5704,7 +5704,7 @@
     </row>
     <row r="84">
       <c r="A84" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -6586,7 +6586,7 @@
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -6775,7 +6775,7 @@
     </row>
     <row r="101">
       <c r="A101" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -6901,7 +6901,7 @@
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -8224,7 +8224,7 @@
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -8539,7 +8539,7 @@
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -9673,7 +9673,7 @@
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
@@ -9736,7 +9736,7 @@
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
@@ -10807,7 +10807,7 @@
     </row>
     <row r="165">
       <c r="A165" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
@@ -10996,7 +10996,7 @@
     </row>
     <row r="168">
       <c r="A168" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -11059,7 +11059,7 @@
     </row>
     <row r="169">
       <c r="A169" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
@@ -11122,7 +11122,7 @@
     </row>
     <row r="170">
       <c r="A170" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
@@ -11374,7 +11374,7 @@
     </row>
     <row r="174">
       <c r="A174" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -11689,7 +11689,7 @@
     </row>
     <row r="179">
       <c r="A179" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -11878,7 +11878,7 @@
     </row>
     <row r="182">
       <c r="A182" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
@@ -12130,7 +12130,7 @@
     </row>
     <row r="186">
       <c r="A186" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -12382,7 +12382,7 @@
     </row>
     <row r="190">
       <c r="A190" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -12508,7 +12508,7 @@
     </row>
     <row r="192">
       <c r="A192" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
@@ -12634,7 +12634,7 @@
     </row>
     <row r="194">
       <c r="A194" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -12697,7 +12697,7 @@
     </row>
     <row r="195">
       <c r="A195" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
@@ -12760,7 +12760,7 @@
     </row>
     <row r="196">
       <c r="A196" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
@@ -13138,7 +13138,7 @@
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
@@ -13201,7 +13201,7 @@
     </row>
     <row r="203">
       <c r="A203" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
@@ -13264,7 +13264,7 @@
     </row>
     <row r="204">
       <c r="A204" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
@@ -13516,7 +13516,7 @@
     </row>
     <row r="208">
       <c r="A208" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B208" t="inlineStr">
         <is>
@@ -13669,7 +13669,7 @@
     </row>
     <row r="211">
       <c r="A211" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B211" t="inlineStr">
         <is>
@@ -13939,7 +13939,7 @@
     </row>
     <row r="217">
       <c r="A217" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B217" t="inlineStr">
         <is>
@@ -13984,7 +13984,7 @@
     </row>
     <row r="218">
       <c r="A218" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B218" t="inlineStr">
         <is>
@@ -14029,7 +14029,7 @@
     </row>
     <row r="219">
       <c r="A219" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B219" t="inlineStr">
         <is>
@@ -14074,7 +14074,7 @@
     </row>
     <row r="220">
       <c r="A220" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B220" t="inlineStr">
         <is>
@@ -14119,7 +14119,7 @@
     </row>
     <row r="221">
       <c r="A221" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B221" t="inlineStr">
         <is>
@@ -14164,7 +14164,7 @@
     </row>
     <row r="222">
       <c r="A222" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B222" t="inlineStr">
         <is>
@@ -14209,7 +14209,7 @@
     </row>
     <row r="223">
       <c r="A223" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B223" t="inlineStr">
         <is>
@@ -14254,7 +14254,7 @@
     </row>
     <row r="224">
       <c r="A224" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B224" t="inlineStr">
         <is>
@@ -14299,7 +14299,7 @@
     </row>
     <row r="225">
       <c r="A225" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B225" t="inlineStr">
         <is>
@@ -14344,7 +14344,7 @@
     </row>
     <row r="226">
       <c r="A226" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B226" t="inlineStr">
         <is>
@@ -14389,7 +14389,7 @@
     </row>
     <row r="227">
       <c r="A227" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B227" t="inlineStr">
         <is>
@@ -14782,7 +14782,7 @@
     </row>
     <row r="234">
       <c r="A234" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B234" t="inlineStr">
         <is>
@@ -15072,7 +15072,7 @@
     </row>
     <row r="239">
       <c r="A239" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B239" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
FIX: L0 State Persistence — UPDATE existing L0 entries se confirmation_mode NULL
Bug: set_l0_entry() era saltato per L0 entries existenti (if isin not in existing_l0).
Risultato: L0 entries vecchi rimettevano con confirmation_mode = NULL.

Fix:
- Estrai confirmation_mode + trigger_low_price per TUTTI gli L0
- Se entry è NEW: set_l0_entry() con i nuovi campi
- Se entry è EXISTING + confirmation_mode è NULL: update_l0_state()
- Log: differenziato tra NUOVO L0 e UPDATE L0
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -604,7 +604,7 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -667,7 +667,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -982,7 +982,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1171,7 +1171,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1486,7 +1486,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1927,7 +1927,7 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2116,7 +2116,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2806,7 +2806,7 @@
     </row>
     <row r="38">
       <c r="A38" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -4570,7 +4570,7 @@
     </row>
     <row r="66">
       <c r="A66" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -4885,7 +4885,7 @@
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -5515,7 +5515,7 @@
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -5578,7 +5578,7 @@
     </row>
     <row r="82">
       <c r="A82" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -5704,7 +5704,7 @@
     </row>
     <row r="84">
       <c r="A84" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -6586,7 +6586,7 @@
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -6775,7 +6775,7 @@
     </row>
     <row r="101">
       <c r="A101" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -6901,7 +6901,7 @@
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -8224,7 +8224,7 @@
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -8539,7 +8539,7 @@
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -9673,7 +9673,7 @@
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
@@ -9736,7 +9736,7 @@
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
@@ -10807,7 +10807,7 @@
     </row>
     <row r="165">
       <c r="A165" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
@@ -10996,7 +10996,7 @@
     </row>
     <row r="168">
       <c r="A168" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -11059,7 +11059,7 @@
     </row>
     <row r="169">
       <c r="A169" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
@@ -11122,7 +11122,7 @@
     </row>
     <row r="170">
       <c r="A170" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
@@ -11374,7 +11374,7 @@
     </row>
     <row r="174">
       <c r="A174" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -11689,7 +11689,7 @@
     </row>
     <row r="179">
       <c r="A179" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -11878,7 +11878,7 @@
     </row>
     <row r="182">
       <c r="A182" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
@@ -12130,7 +12130,7 @@
     </row>
     <row r="186">
       <c r="A186" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -12382,7 +12382,7 @@
     </row>
     <row r="190">
       <c r="A190" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -12508,7 +12508,7 @@
     </row>
     <row r="192">
       <c r="A192" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
@@ -12634,7 +12634,7 @@
     </row>
     <row r="194">
       <c r="A194" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -12697,7 +12697,7 @@
     </row>
     <row r="195">
       <c r="A195" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
@@ -12760,7 +12760,7 @@
     </row>
     <row r="196">
       <c r="A196" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
@@ -13138,7 +13138,7 @@
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
@@ -13201,7 +13201,7 @@
     </row>
     <row r="203">
       <c r="A203" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
@@ -13264,7 +13264,7 @@
     </row>
     <row r="204">
       <c r="A204" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
@@ -13516,7 +13516,7 @@
     </row>
     <row r="208">
       <c r="A208" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B208" t="inlineStr">
         <is>
@@ -13669,7 +13669,7 @@
     </row>
     <row r="211">
       <c r="A211" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B211" t="inlineStr">
         <is>
@@ -13939,7 +13939,7 @@
     </row>
     <row r="217">
       <c r="A217" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B217" t="inlineStr">
         <is>
@@ -13984,7 +13984,7 @@
     </row>
     <row r="218">
       <c r="A218" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B218" t="inlineStr">
         <is>
@@ -14029,7 +14029,7 @@
     </row>
     <row r="219">
       <c r="A219" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B219" t="inlineStr">
         <is>
@@ -14074,7 +14074,7 @@
     </row>
     <row r="220">
       <c r="A220" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B220" t="inlineStr">
         <is>
@@ -14119,7 +14119,7 @@
     </row>
     <row r="221">
       <c r="A221" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B221" t="inlineStr">
         <is>
@@ -14164,7 +14164,7 @@
     </row>
     <row r="222">
       <c r="A222" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B222" t="inlineStr">
         <is>
@@ -14209,7 +14209,7 @@
     </row>
     <row r="223">
       <c r="A223" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B223" t="inlineStr">
         <is>
@@ -14254,7 +14254,7 @@
     </row>
     <row r="224">
       <c r="A224" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B224" t="inlineStr">
         <is>
@@ -14299,7 +14299,7 @@
     </row>
     <row r="225">
       <c r="A225" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B225" t="inlineStr">
         <is>
@@ -14344,7 +14344,7 @@
     </row>
     <row r="226">
       <c r="A226" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B226" t="inlineStr">
         <is>
@@ -14389,7 +14389,7 @@
     </row>
     <row r="227">
       <c r="A227" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B227" t="inlineStr">
         <is>
@@ -14782,7 +14782,7 @@
     </row>
     <row r="234">
       <c r="A234" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B234" t="inlineStr">
         <is>
@@ -15072,7 +15072,7 @@
     </row>
     <row r="239">
       <c r="A239" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B239" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix: remove undefined l1_tiered reference in portfolio SL update — simplify to STEP 3 v4.0 logic
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -604,7 +604,7 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -667,7 +667,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -982,7 +982,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1171,7 +1171,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1486,7 +1486,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1927,7 +1927,7 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2116,7 +2116,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2806,7 +2806,7 @@
     </row>
     <row r="38">
       <c r="A38" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -4570,7 +4570,7 @@
     </row>
     <row r="66">
       <c r="A66" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -4885,7 +4885,7 @@
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -5515,7 +5515,7 @@
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -5578,7 +5578,7 @@
     </row>
     <row r="82">
       <c r="A82" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -5704,7 +5704,7 @@
     </row>
     <row r="84">
       <c r="A84" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -6586,7 +6586,7 @@
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -6775,7 +6775,7 @@
     </row>
     <row r="101">
       <c r="A101" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -6901,7 +6901,7 @@
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -8224,7 +8224,7 @@
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -8539,7 +8539,7 @@
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -9673,7 +9673,7 @@
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
@@ -9736,7 +9736,7 @@
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
@@ -10807,7 +10807,7 @@
     </row>
     <row r="165">
       <c r="A165" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
@@ -10996,7 +10996,7 @@
     </row>
     <row r="168">
       <c r="A168" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -11059,7 +11059,7 @@
     </row>
     <row r="169">
       <c r="A169" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
@@ -11122,7 +11122,7 @@
     </row>
     <row r="170">
       <c r="A170" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
@@ -11374,7 +11374,7 @@
     </row>
     <row r="174">
       <c r="A174" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -11689,7 +11689,7 @@
     </row>
     <row r="179">
       <c r="A179" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -11878,7 +11878,7 @@
     </row>
     <row r="182">
       <c r="A182" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
@@ -12130,7 +12130,7 @@
     </row>
     <row r="186">
       <c r="A186" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -12382,7 +12382,7 @@
     </row>
     <row r="190">
       <c r="A190" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -12508,7 +12508,7 @@
     </row>
     <row r="192">
       <c r="A192" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
@@ -12634,7 +12634,7 @@
     </row>
     <row r="194">
       <c r="A194" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -12697,7 +12697,7 @@
     </row>
     <row r="195">
       <c r="A195" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
@@ -12760,7 +12760,7 @@
     </row>
     <row r="196">
       <c r="A196" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
@@ -13138,7 +13138,7 @@
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
@@ -13201,7 +13201,7 @@
     </row>
     <row r="203">
       <c r="A203" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
@@ -13264,7 +13264,7 @@
     </row>
     <row r="204">
       <c r="A204" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
@@ -13516,7 +13516,7 @@
     </row>
     <row r="208">
       <c r="A208" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B208" t="inlineStr">
         <is>
@@ -13669,7 +13669,7 @@
     </row>
     <row r="211">
       <c r="A211" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B211" t="inlineStr">
         <is>
@@ -13939,7 +13939,7 @@
     </row>
     <row r="217">
       <c r="A217" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B217" t="inlineStr">
         <is>
@@ -13984,7 +13984,7 @@
     </row>
     <row r="218">
       <c r="A218" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B218" t="inlineStr">
         <is>
@@ -14029,7 +14029,7 @@
     </row>
     <row r="219">
       <c r="A219" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B219" t="inlineStr">
         <is>
@@ -14074,7 +14074,7 @@
     </row>
     <row r="220">
       <c r="A220" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B220" t="inlineStr">
         <is>
@@ -14119,7 +14119,7 @@
     </row>
     <row r="221">
       <c r="A221" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B221" t="inlineStr">
         <is>
@@ -14164,7 +14164,7 @@
     </row>
     <row r="222">
       <c r="A222" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B222" t="inlineStr">
         <is>
@@ -14209,7 +14209,7 @@
     </row>
     <row r="223">
       <c r="A223" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B223" t="inlineStr">
         <is>
@@ -14254,7 +14254,7 @@
     </row>
     <row r="224">
       <c r="A224" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B224" t="inlineStr">
         <is>
@@ -14299,7 +14299,7 @@
     </row>
     <row r="225">
       <c r="A225" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B225" t="inlineStr">
         <is>
@@ -14344,7 +14344,7 @@
     </row>
     <row r="226">
       <c r="A226" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B226" t="inlineStr">
         <is>
@@ -14389,7 +14389,7 @@
     </row>
     <row r="227">
       <c r="A227" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B227" t="inlineStr">
         <is>
@@ -14782,7 +14782,7 @@
     </row>
     <row r="234">
       <c r="A234" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B234" t="inlineStr">
         <is>
@@ -15072,7 +15072,7 @@
     </row>
     <row r="239">
       <c r="A239" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B239" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
FIX: Dashboard & CLAUDE.md — Update to 7 mandatory conditions for L1 (STEP 3 v4.0)
- dashboard.html: Aggiorna schema da '6 Condizioni' a '7 Condizioni TUTTE Obbligatorie'
- Aggiunge 7a condizione: Spazio Residuo
- Min Buy Count: da 5/6 o 6/6 → 7/7 per tutte le famiglie
- CLAUDE.md: Aggiorna versione a STEP 3 v4.0

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -604,7 +604,7 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -667,7 +667,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -982,7 +982,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1927,7 +1927,7 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1990,7 +1990,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2116,7 +2116,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2305,7 +2305,7 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2680,7 +2680,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -2743,7 +2743,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -2806,7 +2806,7 @@
     </row>
     <row r="38">
       <c r="A38" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3058,7 +3058,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3940,7 +3940,7 @@
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -4192,7 +4192,7 @@
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -4381,7 +4381,7 @@
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -4570,7 +4570,7 @@
     </row>
     <row r="66">
       <c r="A66" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -4822,7 +4822,7 @@
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -4885,7 +4885,7 @@
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -5263,7 +5263,7 @@
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -5578,7 +5578,7 @@
     </row>
     <row r="82">
       <c r="A82" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -5704,7 +5704,7 @@
     </row>
     <row r="84">
       <c r="A84" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -6397,7 +6397,7 @@
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -6523,7 +6523,7 @@
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -6586,7 +6586,7 @@
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -6775,7 +6775,7 @@
     </row>
     <row r="101">
       <c r="A101" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -6964,7 +6964,7 @@
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -7027,7 +7027,7 @@
     </row>
     <row r="105">
       <c r="A105" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
@@ -7342,7 +7342,7 @@
     </row>
     <row r="110">
       <c r="A110" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -7468,7 +7468,7 @@
     </row>
     <row r="112">
       <c r="A112" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
@@ -7846,7 +7846,7 @@
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -8287,7 +8287,7 @@
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -8476,7 +8476,7 @@
     </row>
     <row r="128">
       <c r="A128" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
@@ -8539,7 +8539,7 @@
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -8665,7 +8665,7 @@
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
@@ -8728,7 +8728,7 @@
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -9106,7 +9106,7 @@
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
@@ -9169,7 +9169,7 @@
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
@@ -9295,7 +9295,7 @@
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
@@ -9358,7 +9358,7 @@
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
@@ -9421,7 +9421,7 @@
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
@@ -9484,7 +9484,7 @@
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
@@ -9925,7 +9925,7 @@
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -10051,7 +10051,7 @@
     </row>
     <row r="153">
       <c r="A153" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
@@ -10177,7 +10177,7 @@
     </row>
     <row r="155">
       <c r="A155" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
@@ -10240,7 +10240,7 @@
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
@@ -10618,7 +10618,7 @@
     </row>
     <row r="162">
       <c r="A162" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
@@ -11311,7 +11311,7 @@
     </row>
     <row r="173">
       <c r="A173" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
@@ -11374,7 +11374,7 @@
     </row>
     <row r="174">
       <c r="A174" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -11689,7 +11689,7 @@
     </row>
     <row r="179">
       <c r="A179" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -11878,7 +11878,7 @@
     </row>
     <row r="182">
       <c r="A182" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
@@ -12130,7 +12130,7 @@
     </row>
     <row r="186">
       <c r="A186" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -12382,7 +12382,7 @@
     </row>
     <row r="190">
       <c r="A190" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -12508,7 +12508,7 @@
     </row>
     <row r="192">
       <c r="A192" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
@@ -12634,7 +12634,7 @@
     </row>
     <row r="194">
       <c r="A194" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -12697,7 +12697,7 @@
     </row>
     <row r="195">
       <c r="A195" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
@@ -12823,7 +12823,7 @@
     </row>
     <row r="197">
       <c r="A197" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
@@ -12949,7 +12949,7 @@
     </row>
     <row r="199">
       <c r="A199" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B199" t="inlineStr">
         <is>
@@ -13264,7 +13264,7 @@
     </row>
     <row r="204">
       <c r="A204" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
@@ -13516,7 +13516,7 @@
     </row>
     <row r="208">
       <c r="A208" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B208" t="inlineStr">
         <is>
@@ -14434,7 +14434,7 @@
     </row>
     <row r="228">
       <c r="A228" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B228" t="inlineStr">
         <is>
@@ -14724,7 +14724,7 @@
     </row>
     <row r="233">
       <c r="A233" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B233" t="inlineStr">
         <is>
@@ -14782,7 +14782,7 @@
     </row>
     <row r="234">
       <c r="A234" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B234" t="inlineStr">
         <is>
@@ -15014,7 +15014,7 @@
     </row>
     <row r="238">
       <c r="A238" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B238" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Sync etf_monitoraggio.xlsx da VPS post-deploy
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -604,7 +604,7 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -667,7 +667,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1171,7 +1171,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1486,7 +1486,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1927,7 +1927,7 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2116,7 +2116,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -4885,7 +4885,7 @@
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -5515,7 +5515,7 @@
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -5578,7 +5578,7 @@
     </row>
     <row r="82">
       <c r="A82" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -6775,7 +6775,7 @@
     </row>
     <row r="101">
       <c r="A101" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -6901,7 +6901,7 @@
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -7594,7 +7594,7 @@
     </row>
     <row r="114">
       <c r="A114" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
@@ -8224,7 +8224,7 @@
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -8539,7 +8539,7 @@
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -8665,7 +8665,7 @@
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
@@ -9106,7 +9106,7 @@
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
@@ -9673,7 +9673,7 @@
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
@@ -9736,7 +9736,7 @@
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
@@ -10051,7 +10051,7 @@
     </row>
     <row r="153">
       <c r="A153" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
@@ -10177,7 +10177,7 @@
     </row>
     <row r="155">
       <c r="A155" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
@@ -10240,7 +10240,7 @@
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
@@ -10807,7 +10807,7 @@
     </row>
     <row r="165">
       <c r="A165" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
@@ -10996,7 +10996,7 @@
     </row>
     <row r="168">
       <c r="A168" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -11059,7 +11059,7 @@
     </row>
     <row r="169">
       <c r="A169" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
@@ -11122,7 +11122,7 @@
     </row>
     <row r="170">
       <c r="A170" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
@@ -11248,7 +11248,7 @@
     </row>
     <row r="172">
       <c r="A172" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
@@ -11311,7 +11311,7 @@
     </row>
     <row r="173">
       <c r="A173" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
@@ -11689,7 +11689,7 @@
     </row>
     <row r="179">
       <c r="A179" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -11878,7 +11878,7 @@
     </row>
     <row r="182">
       <c r="A182" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
@@ -12130,7 +12130,7 @@
     </row>
     <row r="186">
       <c r="A186" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -12382,7 +12382,7 @@
     </row>
     <row r="190">
       <c r="A190" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -12508,7 +12508,7 @@
     </row>
     <row r="192">
       <c r="A192" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
@@ -12634,7 +12634,7 @@
     </row>
     <row r="194">
       <c r="A194" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -12760,7 +12760,7 @@
     </row>
     <row r="196">
       <c r="A196" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
@@ -13138,7 +13138,7 @@
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
@@ -13201,7 +13201,7 @@
     </row>
     <row r="203">
       <c r="A203" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
@@ -13264,7 +13264,7 @@
     </row>
     <row r="204">
       <c r="A204" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
@@ -13669,7 +13669,7 @@
     </row>
     <row r="211">
       <c r="A211" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B211" t="inlineStr">
         <is>
@@ -13939,7 +13939,7 @@
     </row>
     <row r="217">
       <c r="A217" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B217" t="inlineStr">
         <is>
@@ -13984,7 +13984,7 @@
     </row>
     <row r="218">
       <c r="A218" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B218" t="inlineStr">
         <is>
@@ -14029,7 +14029,7 @@
     </row>
     <row r="219">
       <c r="A219" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B219" t="inlineStr">
         <is>
@@ -14074,7 +14074,7 @@
     </row>
     <row r="220">
       <c r="A220" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B220" t="inlineStr">
         <is>
@@ -14119,7 +14119,7 @@
     </row>
     <row r="221">
       <c r="A221" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B221" t="inlineStr">
         <is>
@@ -14164,7 +14164,7 @@
     </row>
     <row r="222">
       <c r="A222" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B222" t="inlineStr">
         <is>
@@ -14209,7 +14209,7 @@
     </row>
     <row r="223">
       <c r="A223" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B223" t="inlineStr">
         <is>
@@ -14254,7 +14254,7 @@
     </row>
     <row r="224">
       <c r="A224" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B224" t="inlineStr">
         <is>
@@ -14299,7 +14299,7 @@
     </row>
     <row r="225">
       <c r="A225" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B225" t="inlineStr">
         <is>
@@ -14344,7 +14344,7 @@
     </row>
     <row r="226">
       <c r="A226" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B226" t="inlineStr">
         <is>
@@ -14389,7 +14389,7 @@
     </row>
     <row r="227">
       <c r="A227" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B227" t="inlineStr">
         <is>
@@ -14608,7 +14608,7 @@
     </row>
     <row r="231">
       <c r="A231" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B231" t="inlineStr">
         <is>
@@ -15072,7 +15072,7 @@
     </row>
     <row r="239">
       <c r="A239" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B239" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: allinea etf_monitoraggio.xlsx (sync fine sessione)
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -667,7 +667,7 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -2116,7 +2116,7 @@
     </row>
     <row r="27">
       <c r="A27" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -8227,7 +8227,7 @@
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -8542,7 +8542,7 @@
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -9676,7 +9676,7 @@
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
@@ -9739,7 +9739,7 @@
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
@@ -10810,7 +10810,7 @@
     </row>
     <row r="165">
       <c r="A165" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
@@ -11062,7 +11062,7 @@
     </row>
     <row r="169">
       <c r="A169" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
@@ -12133,7 +12133,7 @@
     </row>
     <row r="186">
       <c r="A186" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -12385,7 +12385,7 @@
     </row>
     <row r="190">
       <c r="A190" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -12637,7 +12637,7 @@
     </row>
     <row r="194">
       <c r="A194" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -13204,7 +13204,7 @@
     </row>
     <row r="203">
       <c r="A203" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
@@ -13267,7 +13267,7 @@
     </row>
     <row r="204">
       <c r="A204" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
@@ -13645,7 +13645,7 @@
     </row>
     <row r="210">
       <c r="A210" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B210" t="inlineStr">
         <is>
@@ -13771,7 +13771,7 @@
     </row>
     <row r="212">
       <c r="A212" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B212" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Revert ticker LU1954152853 fix: LU1954152853.SG non fetchabile da yfinance, torna a UST.PA (problema noto, non risolto)
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -593,7 +593,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -782,7 +782,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1349,7 +1349,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -1412,7 +1412,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -1538,7 +1538,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -1601,7 +1601,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -1727,7 +1727,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -1790,7 +1790,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -1916,7 +1916,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -2042,7 +2042,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -2168,7 +2168,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
@@ -2231,7 +2231,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
@@ -2294,7 +2294,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
@@ -2357,7 +2357,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -2609,7 +2609,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
@@ -2735,7 +2735,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
@@ -2798,7 +2798,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
@@ -2861,7 +2861,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
@@ -2924,7 +2924,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
@@ -2987,7 +2987,7 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
@@ -3176,7 +3176,7 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
@@ -3239,7 +3239,7 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
@@ -3302,7 +3302,7 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
@@ -3365,7 +3365,7 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
@@ -3428,7 +3428,7 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
@@ -3491,7 +3491,7 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
@@ -3554,7 +3554,7 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
@@ -3617,7 +3617,7 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
@@ -3680,7 +3680,7 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
@@ -3806,7 +3806,7 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
@@ -3932,7 +3932,7 @@
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
@@ -3995,7 +3995,7 @@
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
@@ -4058,7 +4058,7 @@
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O57" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O58" t="inlineStr">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
@@ -4247,7 +4247,7 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O60" t="inlineStr">
@@ -4310,7 +4310,7 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
@@ -4373,7 +4373,7 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O62" t="inlineStr">
@@ -4436,7 +4436,7 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O63" t="inlineStr">
@@ -4499,7 +4499,7 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
@@ -4625,7 +4625,7 @@
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O66" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O67" t="inlineStr">
@@ -4751,7 +4751,7 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O68" t="inlineStr">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
@@ -4877,7 +4877,7 @@
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O70" t="inlineStr">
@@ -4940,7 +4940,7 @@
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O71" t="inlineStr">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O72" t="inlineStr">
@@ -5066,7 +5066,7 @@
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O73" t="inlineStr">
@@ -5129,7 +5129,7 @@
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O74" t="inlineStr">
@@ -5192,7 +5192,7 @@
       </c>
       <c r="N75" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O75" t="inlineStr">
@@ -5255,7 +5255,7 @@
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O76" t="inlineStr">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
@@ -5381,7 +5381,7 @@
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O78" t="inlineStr">
@@ -5444,7 +5444,7 @@
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O79" t="inlineStr">
@@ -5507,7 +5507,7 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
@@ -5570,7 +5570,7 @@
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O81" t="inlineStr">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O82" t="inlineStr">
@@ -5696,7 +5696,7 @@
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O83" t="inlineStr">
@@ -5759,7 +5759,7 @@
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O84" t="inlineStr">
@@ -5822,7 +5822,7 @@
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O85" t="inlineStr">
@@ -5885,7 +5885,7 @@
       </c>
       <c r="N86" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O86" t="inlineStr">
@@ -5948,7 +5948,7 @@
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O87" t="inlineStr">
@@ -6011,7 +6011,7 @@
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O88" t="inlineStr">
@@ -6074,7 +6074,7 @@
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O89" t="inlineStr">
@@ -6137,7 +6137,7 @@
       </c>
       <c r="N90" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O90" t="inlineStr">
@@ -6200,7 +6200,7 @@
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O91" t="inlineStr">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="N92" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O92" t="inlineStr">
@@ -6326,7 +6326,7 @@
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O93" t="inlineStr">
@@ -6389,7 +6389,7 @@
       </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O94" t="inlineStr">
@@ -6452,7 +6452,7 @@
       </c>
       <c r="N95" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O95" t="inlineStr">
@@ -6515,7 +6515,7 @@
       </c>
       <c r="N96" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O96" t="inlineStr">
@@ -6578,7 +6578,7 @@
       </c>
       <c r="N97" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O97" t="inlineStr">
@@ -6641,7 +6641,7 @@
       </c>
       <c r="N98" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O98" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="N99" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O99" t="inlineStr">
@@ -6767,7 +6767,7 @@
       </c>
       <c r="N100" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O100" t="inlineStr">
@@ -6830,7 +6830,7 @@
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O101" t="inlineStr">
@@ -6893,7 +6893,7 @@
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O102" t="inlineStr">
@@ -6956,7 +6956,7 @@
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O103" t="inlineStr">
@@ -7019,7 +7019,7 @@
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O104" t="inlineStr">
@@ -7082,7 +7082,7 @@
       </c>
       <c r="N105" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O105" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="N106" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O106" t="inlineStr">
@@ -7208,7 +7208,7 @@
       </c>
       <c r="N107" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O107" t="inlineStr">
@@ -7271,7 +7271,7 @@
       </c>
       <c r="N108" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O108" t="inlineStr">
@@ -7334,7 +7334,7 @@
       </c>
       <c r="N109" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O109" t="inlineStr">
@@ -7397,7 +7397,7 @@
       </c>
       <c r="N110" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O110" t="inlineStr">
@@ -7460,7 +7460,7 @@
       </c>
       <c r="N111" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O111" t="inlineStr">
@@ -7523,7 +7523,7 @@
       </c>
       <c r="N112" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O112" t="inlineStr">
@@ -7586,7 +7586,7 @@
       </c>
       <c r="N113" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O113" t="inlineStr">
@@ -7649,7 +7649,7 @@
       </c>
       <c r="N114" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O114" t="inlineStr">
@@ -7712,7 +7712,7 @@
       </c>
       <c r="N115" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O115" t="inlineStr">
@@ -7775,7 +7775,7 @@
       </c>
       <c r="N116" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O116" t="inlineStr">
@@ -7838,7 +7838,7 @@
       </c>
       <c r="N117" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O117" t="inlineStr">
@@ -7901,7 +7901,7 @@
       </c>
       <c r="N118" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O118" t="inlineStr">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="N119" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O119" t="inlineStr">
@@ -8027,7 +8027,7 @@
       </c>
       <c r="N120" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O120" t="inlineStr">
@@ -8090,7 +8090,7 @@
       </c>
       <c r="N121" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O121" t="inlineStr">
@@ -8153,7 +8153,7 @@
       </c>
       <c r="N122" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O122" t="inlineStr">
@@ -8216,7 +8216,7 @@
       </c>
       <c r="N123" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O123" t="inlineStr">
@@ -8279,7 +8279,7 @@
       </c>
       <c r="N124" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O124" t="inlineStr">
@@ -8342,7 +8342,7 @@
       </c>
       <c r="N125" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O125" t="inlineStr">
@@ -8405,7 +8405,7 @@
       </c>
       <c r="N126" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O126" t="inlineStr">
@@ -8468,7 +8468,7 @@
       </c>
       <c r="N127" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O127" t="inlineStr">
@@ -8531,7 +8531,7 @@
       </c>
       <c r="N128" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O128" t="inlineStr">
@@ -8594,7 +8594,7 @@
       </c>
       <c r="N129" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O129" t="inlineStr">
@@ -8657,7 +8657,7 @@
       </c>
       <c r="N130" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O130" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="N131" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O131" t="inlineStr">
@@ -8783,7 +8783,7 @@
       </c>
       <c r="N132" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O132" t="inlineStr">
@@ -8846,7 +8846,7 @@
       </c>
       <c r="N133" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O133" t="inlineStr">
@@ -8909,7 +8909,7 @@
       </c>
       <c r="N134" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O134" t="inlineStr">
@@ -8972,7 +8972,7 @@
       </c>
       <c r="N135" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O135" t="inlineStr">
@@ -9035,7 +9035,7 @@
       </c>
       <c r="N136" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O136" t="inlineStr">
@@ -9098,7 +9098,7 @@
       </c>
       <c r="N137" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O137" t="inlineStr">
@@ -9161,7 +9161,7 @@
       </c>
       <c r="N138" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O138" t="inlineStr">
@@ -9224,7 +9224,7 @@
       </c>
       <c r="N139" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O139" t="inlineStr">
@@ -9287,7 +9287,7 @@
       </c>
       <c r="N140" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O140" t="inlineStr">
@@ -9350,7 +9350,7 @@
       </c>
       <c r="N141" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O141" t="inlineStr">
@@ -9413,7 +9413,7 @@
       </c>
       <c r="N142" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O142" t="inlineStr">
@@ -9476,7 +9476,7 @@
       </c>
       <c r="N143" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O143" t="inlineStr">
@@ -9539,7 +9539,7 @@
       </c>
       <c r="N144" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O144" t="inlineStr">
@@ -9602,7 +9602,7 @@
       </c>
       <c r="N145" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O145" t="inlineStr">
@@ -9641,22 +9641,22 @@
         </is>
       </c>
       <c r="G146" t="n">
-        <v>118.54</v>
+        <v>118.36</v>
       </c>
       <c r="H146" t="n">
-        <v>118.15</v>
+        <v>118.17</v>
       </c>
       <c r="I146" t="n">
-        <v>117.4704</v>
+        <v>117.3876</v>
       </c>
       <c r="J146" t="n">
-        <v>52.7</v>
+        <v>52.1</v>
       </c>
       <c r="K146" t="n">
-        <v>23.4</v>
+        <v>23.1</v>
       </c>
       <c r="L146" t="n">
-        <v>-0.0343</v>
+        <v>-0.1144</v>
       </c>
       <c r="M146" s="6" t="inlineStr">
         <is>
@@ -9665,7 +9665,7 @@
       </c>
       <c r="N146" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O146" t="inlineStr">
@@ -9728,7 +9728,7 @@
       </c>
       <c r="N147" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O147" t="inlineStr">
@@ -9791,7 +9791,7 @@
       </c>
       <c r="N148" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O148" t="inlineStr">
@@ -9854,7 +9854,7 @@
       </c>
       <c r="N149" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O149" t="inlineStr">
@@ -9917,7 +9917,7 @@
       </c>
       <c r="N150" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O150" t="inlineStr">
@@ -9980,7 +9980,7 @@
       </c>
       <c r="N151" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O151" t="inlineStr">
@@ -10043,7 +10043,7 @@
       </c>
       <c r="N152" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O152" t="inlineStr">
@@ -10106,7 +10106,7 @@
       </c>
       <c r="N153" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O153" t="inlineStr">
@@ -10169,7 +10169,7 @@
       </c>
       <c r="N154" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O154" t="inlineStr">
@@ -10232,7 +10232,7 @@
       </c>
       <c r="N155" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O155" t="inlineStr">
@@ -10295,7 +10295,7 @@
       </c>
       <c r="N156" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O156" t="inlineStr">
@@ -10358,7 +10358,7 @@
       </c>
       <c r="N157" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O157" t="inlineStr">
@@ -10373,7 +10373,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>LU1954152853.SG</t>
+          <t>UST.PA</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -10388,7 +10388,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Stoccarda</t>
+          <t>Milano</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -10421,7 +10421,7 @@
       </c>
       <c r="N158" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O158" t="inlineStr">
@@ -10484,7 +10484,7 @@
       </c>
       <c r="N159" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O159" t="inlineStr">
@@ -10547,7 +10547,7 @@
       </c>
       <c r="N160" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O160" t="inlineStr">
@@ -10610,7 +10610,7 @@
       </c>
       <c r="N161" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O161" t="inlineStr">
@@ -10673,7 +10673,7 @@
       </c>
       <c r="N162" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O162" t="inlineStr">
@@ -10736,7 +10736,7 @@
       </c>
       <c r="N163" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O163" t="inlineStr">
@@ -10799,7 +10799,7 @@
       </c>
       <c r="N164" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O164" t="inlineStr">
@@ -10862,7 +10862,7 @@
       </c>
       <c r="N165" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O165" t="inlineStr">
@@ -10925,7 +10925,7 @@
       </c>
       <c r="N166" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O166" t="inlineStr">
@@ -10988,7 +10988,7 @@
       </c>
       <c r="N167" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O167" t="inlineStr">
@@ -11051,7 +11051,7 @@
       </c>
       <c r="N168" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O168" t="inlineStr">
@@ -11114,7 +11114,7 @@
       </c>
       <c r="N169" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O169" t="inlineStr">
@@ -11177,7 +11177,7 @@
       </c>
       <c r="N170" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O170" t="inlineStr">
@@ -11240,7 +11240,7 @@
       </c>
       <c r="N171" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O171" t="inlineStr">
@@ -11303,7 +11303,7 @@
       </c>
       <c r="N172" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O172" t="inlineStr">
@@ -11366,7 +11366,7 @@
       </c>
       <c r="N173" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O173" t="inlineStr">
@@ -11429,7 +11429,7 @@
       </c>
       <c r="N174" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O174" t="inlineStr">
@@ -11492,7 +11492,7 @@
       </c>
       <c r="N175" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O175" t="inlineStr">
@@ -11555,7 +11555,7 @@
       </c>
       <c r="N176" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O176" t="inlineStr">
@@ -11618,7 +11618,7 @@
       </c>
       <c r="N177" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O177" t="inlineStr">
@@ -11681,7 +11681,7 @@
       </c>
       <c r="N178" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O178" t="inlineStr">
@@ -11744,7 +11744,7 @@
       </c>
       <c r="N179" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O179" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="N180" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O180" t="inlineStr">
@@ -11870,7 +11870,7 @@
       </c>
       <c r="N181" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O181" t="inlineStr">
@@ -11933,7 +11933,7 @@
       </c>
       <c r="N182" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O182" t="inlineStr">
@@ -11996,7 +11996,7 @@
       </c>
       <c r="N183" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O183" t="inlineStr">
@@ -12059,7 +12059,7 @@
       </c>
       <c r="N184" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O184" t="inlineStr">
@@ -12122,7 +12122,7 @@
       </c>
       <c r="N185" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O185" t="inlineStr">
@@ -12185,7 +12185,7 @@
       </c>
       <c r="N186" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O186" t="inlineStr">
@@ -12248,7 +12248,7 @@
       </c>
       <c r="N187" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O187" t="inlineStr">
@@ -12311,7 +12311,7 @@
       </c>
       <c r="N188" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O188" t="inlineStr">
@@ -12374,7 +12374,7 @@
       </c>
       <c r="N189" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O189" t="inlineStr">
@@ -12437,7 +12437,7 @@
       </c>
       <c r="N190" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O190" t="inlineStr">
@@ -12500,7 +12500,7 @@
       </c>
       <c r="N191" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O191" t="inlineStr">
@@ -12563,7 +12563,7 @@
       </c>
       <c r="N192" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O192" t="inlineStr">
@@ -12626,7 +12626,7 @@
       </c>
       <c r="N193" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O193" t="inlineStr">
@@ -12689,7 +12689,7 @@
       </c>
       <c r="N194" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O194" t="inlineStr">
@@ -12752,7 +12752,7 @@
       </c>
       <c r="N195" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O195" t="inlineStr">
@@ -12815,7 +12815,7 @@
       </c>
       <c r="N196" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O196" t="inlineStr">
@@ -12878,7 +12878,7 @@
       </c>
       <c r="N197" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O197" t="inlineStr">
@@ -12941,7 +12941,7 @@
       </c>
       <c r="N198" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O198" t="inlineStr">
@@ -13004,7 +13004,7 @@
       </c>
       <c r="N199" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O199" t="inlineStr">
@@ -13067,7 +13067,7 @@
       </c>
       <c r="N200" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O200" t="inlineStr">
@@ -13130,7 +13130,7 @@
       </c>
       <c r="N201" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O201" t="inlineStr">
@@ -13193,7 +13193,7 @@
       </c>
       <c r="N202" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O202" t="inlineStr">
@@ -13256,7 +13256,7 @@
       </c>
       <c r="N203" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O203" t="inlineStr">
@@ -13319,7 +13319,7 @@
       </c>
       <c r="N204" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O204" t="inlineStr">
@@ -13382,7 +13382,7 @@
       </c>
       <c r="N205" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O205" t="inlineStr">
@@ -13445,7 +13445,7 @@
       </c>
       <c r="N206" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O206" t="inlineStr">
@@ -13508,7 +13508,7 @@
       </c>
       <c r="N207" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O207" t="inlineStr">
@@ -13571,7 +13571,7 @@
       </c>
       <c r="N208" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O208" t="inlineStr">
@@ -13634,7 +13634,7 @@
       </c>
       <c r="N209" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O209" t="inlineStr">
@@ -13697,7 +13697,7 @@
       </c>
       <c r="N210" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O210" t="inlineStr">
@@ -13760,7 +13760,7 @@
       </c>
       <c r="N211" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O211" t="inlineStr">
@@ -13823,7 +13823,7 @@
       </c>
       <c r="N212" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O212" t="inlineStr">
@@ -13883,7 +13883,7 @@
       </c>
       <c r="N213" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O213" t="inlineStr">
@@ -13946,7 +13946,7 @@
       </c>
       <c r="N214" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O214" t="inlineStr">
@@ -14009,7 +14009,7 @@
       </c>
       <c r="N215" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O215" t="inlineStr">
@@ -14072,7 +14072,7 @@
       </c>
       <c r="N216" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O216" t="inlineStr">
@@ -14135,7 +14135,7 @@
       </c>
       <c r="N217" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O217" t="inlineStr">
@@ -14198,7 +14198,7 @@
       </c>
       <c r="N218" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O218" t="inlineStr">
@@ -14261,7 +14261,7 @@
       </c>
       <c r="N219" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O219" t="inlineStr">
@@ -14324,7 +14324,7 @@
       </c>
       <c r="N220" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O220" t="inlineStr">
@@ -14387,7 +14387,7 @@
       </c>
       <c r="N221" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O221" t="inlineStr">
@@ -14450,7 +14450,7 @@
       </c>
       <c r="N222" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O222" t="inlineStr">
@@ -14513,7 +14513,7 @@
       </c>
       <c r="N223" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O223" t="inlineStr">
@@ -14576,7 +14576,7 @@
       </c>
       <c r="N224" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O224" t="inlineStr">
@@ -14639,7 +14639,7 @@
       </c>
       <c r="N225" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O225" t="inlineStr">
@@ -14702,7 +14702,7 @@
       </c>
       <c r="N226" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O226" t="inlineStr">
@@ -14765,7 +14765,7 @@
       </c>
       <c r="N227" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O227" t="inlineStr">
@@ -14828,7 +14828,7 @@
       </c>
       <c r="N228" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O228" t="inlineStr">
@@ -14891,7 +14891,7 @@
       </c>
       <c r="N229" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O229" t="inlineStr">
@@ -14954,7 +14954,7 @@
       </c>
       <c r="N230" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O230" t="inlineStr">
@@ -15017,7 +15017,7 @@
       </c>
       <c r="N231" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O231" t="inlineStr">
@@ -15080,7 +15080,7 @@
       </c>
       <c r="N232" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O232" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="N233" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O233" t="inlineStr">
@@ -15206,7 +15206,7 @@
       </c>
       <c r="N234" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O234" t="inlineStr">
@@ -15269,7 +15269,7 @@
       </c>
       <c r="N235" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O235" t="inlineStr">
@@ -15332,7 +15332,7 @@
       </c>
       <c r="N236" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O236" t="inlineStr">
@@ -15395,7 +15395,7 @@
       </c>
       <c r="N237" t="inlineStr">
         <is>
-          <t>2026-08-25 12:55</t>
+          <t>2026-08-25 14:28</t>
         </is>
       </c>
       <c r="O237" t="inlineStr">

</xml_diff>

<commit_message>
Fix ticker WATC e INRG: allineati al listino Directa (EUR)
- WATC.SW -> WATC.PA (FR0014002CH1): il ticker svizzero restituiva CHF ma
  l'Excel diceva EUR -> prezzo mostrato ~6.55 in realta' CHF. WATC.PA e' il
  listino Euronext Paris in EUR (~7.00), quello negoziato su Directa.
- INRG.SW -> INRG.MI (IE00B1XNHC34): il ticker svizzero restituiva USD
  (~10.23) mostrato come EUR; l'Excel gia' diceva Milano/EUR. INRG.MI e'
  vivo su Yahoo, EUR ~8.74 (Directa Milano) — corregge anche un errore di
  prezzo del ~16%.

Principio: il monitor deve sempre seguire lo stesso listino/valuta che
negozia Directa (i nostri ETF sono quelli di Directa).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HPsTcHPHNyTy55bZuN9KB6
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1903" uniqueCount="785">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1903" uniqueCount="784">
   <si>
     <t>Livello</t>
   </si>
@@ -1748,7 +1748,7 @@
     <t>IE00B1FZS350</t>
   </si>
   <si>
-    <t>INRG.SW</t>
+    <t>INRG.MI</t>
   </si>
   <si>
     <t>iShares Global Clean Energy UCITS ETF USD Dist</t>
@@ -2078,9 +2078,6 @@
     <t>IE000V0H6AD4</t>
   </si>
   <si>
-    <t>INRG.MI</t>
-  </si>
-  <si>
     <t>iShares Global Clean Energy Transition UCITS ETF</t>
   </si>
   <si>
@@ -2333,22 +2330,22 @@
     <t>FR0012399806</t>
   </si>
   <si>
-    <t>WATC.SW</t>
+    <t>WATC.PA</t>
   </si>
   <si>
     <t>Amundi MSCI Water UCITS ETF Acc</t>
   </si>
   <si>
+    <t>FR0014002CH1</t>
+  </si>
+  <si>
+    <t>CSBGU7.SW</t>
+  </si>
+  <si>
+    <t>iShares VII PLC - iShares VII PLC - iShares $ Trea</t>
+  </si>
+  <si>
     <t>Svizzera</t>
-  </si>
-  <si>
-    <t>FR0014002CH1</t>
-  </si>
-  <si>
-    <t>CSBGU7.SW</t>
-  </si>
-  <si>
-    <t>iShares VII PLC - iShares VII PLC - iShares $ Trea</t>
   </si>
   <si>
     <t>IE00B3VWN393</t>
@@ -3440,7 +3437,7 @@
     </row>
     <row r="2" spans="1:15">
       <c r="A2" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B2" t="s">
         <v>15</v>
@@ -3816,7 +3813,7 @@
     </row>
     <row r="10" spans="1:15">
       <c r="A10" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B10" t="s">
         <v>52</v>
@@ -4803,7 +4800,7 @@
     </row>
     <row r="31" spans="1:15">
       <c r="A31" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B31" t="s">
         <v>122</v>
@@ -5132,7 +5129,7 @@
     </row>
     <row r="38" spans="1:15">
       <c r="A38" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B38" t="s">
         <v>145</v>
@@ -5179,7 +5176,7 @@
     </row>
     <row r="39" spans="1:15">
       <c r="A39" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B39" t="s">
         <v>148</v>
@@ -5414,7 +5411,7 @@
     </row>
     <row r="44" spans="1:15">
       <c r="A44" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B44" t="s">
         <v>163</v>
@@ -5837,7 +5834,7 @@
     </row>
     <row r="53" spans="1:15">
       <c r="A53" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B53" t="s">
         <v>191</v>
@@ -5931,7 +5928,7 @@
     </row>
     <row r="55" spans="1:15">
       <c r="A55" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B55" t="s">
         <v>197</v>
@@ -6307,7 +6304,7 @@
     </row>
     <row r="63" spans="1:15">
       <c r="A63" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B63" t="s">
         <v>222</v>
@@ -8422,7 +8419,7 @@
     </row>
     <row r="108" spans="1:15">
       <c r="A108" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B108" t="s">
         <v>367</v>
@@ -8704,7 +8701,7 @@
     </row>
     <row r="114" spans="1:15">
       <c r="A114" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B114" t="s">
         <v>385</v>
@@ -8751,7 +8748,7 @@
     </row>
     <row r="115" spans="1:15">
       <c r="A115" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B115" t="s">
         <v>388</v>
@@ -12088,7 +12085,7 @@
     </row>
     <row r="186" spans="1:15">
       <c r="A186" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B186" t="s">
         <v>613</v>
@@ -13125,10 +13122,10 @@
         <v>3</v>
       </c>
       <c r="B208" t="s">
+        <v>573</v>
+      </c>
+      <c r="C208" t="s">
         <v>683</v>
-      </c>
-      <c r="C208" t="s">
-        <v>684</v>
       </c>
       <c r="D208" t="s">
         <v>46</v>
@@ -13164,7 +13161,7 @@
         <v>21</v>
       </c>
       <c r="O208" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="209" spans="1:15">
@@ -13172,10 +13169,10 @@
         <v>3</v>
       </c>
       <c r="B209" t="s">
+        <v>685</v>
+      </c>
+      <c r="C209" t="s">
         <v>686</v>
-      </c>
-      <c r="C209" t="s">
-        <v>687</v>
       </c>
       <c r="D209" t="s">
         <v>555</v>
@@ -13211,7 +13208,7 @@
         <v>21</v>
       </c>
       <c r="O209" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
     </row>
     <row r="210" spans="1:15">
@@ -13219,13 +13216,13 @@
         <v>3</v>
       </c>
       <c r="B210" t="s">
+        <v>688</v>
+      </c>
+      <c r="C210" t="s">
         <v>689</v>
       </c>
-      <c r="C210" t="s">
+      <c r="D210" t="s">
         <v>690</v>
-      </c>
-      <c r="D210" t="s">
-        <v>691</v>
       </c>
       <c r="E210" t="s">
         <v>18</v>
@@ -13258,7 +13255,7 @@
         <v>21</v>
       </c>
       <c r="O210" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="211" spans="1:15">
@@ -13266,19 +13263,19 @@
         <v>3</v>
       </c>
       <c r="B211" t="s">
+        <v>692</v>
+      </c>
+      <c r="C211" t="s">
         <v>693</v>
       </c>
-      <c r="C211" t="s">
+      <c r="D211" t="s">
         <v>694</v>
       </c>
-      <c r="D211" t="s">
+      <c r="E211" t="s">
         <v>695</v>
       </c>
-      <c r="E211" t="s">
+      <c r="F211" t="s">
         <v>696</v>
-      </c>
-      <c r="F211" t="s">
-        <v>697</v>
       </c>
       <c r="G211">
         <v>61.09</v>
@@ -13305,7 +13302,7 @@
         <v>21</v>
       </c>
       <c r="O211" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
     </row>
     <row r="212" spans="1:15">
@@ -13313,19 +13310,19 @@
         <v>3</v>
       </c>
       <c r="B212" t="s">
+        <v>698</v>
+      </c>
+      <c r="C212" t="s">
         <v>699</v>
       </c>
-      <c r="C212" t="s">
-        <v>700</v>
-      </c>
       <c r="D212" t="s">
+        <v>694</v>
+      </c>
+      <c r="E212" t="s">
         <v>695</v>
       </c>
-      <c r="E212" t="s">
+      <c r="F212" t="s">
         <v>696</v>
-      </c>
-      <c r="F212" t="s">
-        <v>697</v>
       </c>
       <c r="G212">
         <v>61.08</v>
@@ -13352,7 +13349,7 @@
         <v>21</v>
       </c>
       <c r="O212" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
     </row>
     <row r="213" spans="1:15">
@@ -13360,19 +13357,19 @@
         <v>2</v>
       </c>
       <c r="B213" t="s">
+        <v>701</v>
+      </c>
+      <c r="C213" t="s">
         <v>702</v>
       </c>
-      <c r="C213" t="s">
-        <v>703</v>
-      </c>
       <c r="D213" t="s">
+        <v>694</v>
+      </c>
+      <c r="E213" t="s">
         <v>695</v>
       </c>
-      <c r="E213" t="s">
+      <c r="F213" t="s">
         <v>696</v>
-      </c>
-      <c r="F213" t="s">
-        <v>697</v>
       </c>
       <c r="G213">
         <v>9.262</v>
@@ -13396,7 +13393,7 @@
         <v>21</v>
       </c>
       <c r="O213" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="214" spans="1:15">
@@ -13404,16 +13401,16 @@
         <v>3</v>
       </c>
       <c r="B214" t="s">
+        <v>704</v>
+      </c>
+      <c r="C214" t="s">
         <v>705</v>
       </c>
-      <c r="C214" t="s">
+      <c r="D214" t="s">
+        <v>694</v>
+      </c>
+      <c r="E214" t="s">
         <v>706</v>
-      </c>
-      <c r="D214" t="s">
-        <v>695</v>
-      </c>
-      <c r="E214" t="s">
-        <v>707</v>
       </c>
       <c r="F214" t="s">
         <v>19</v>
@@ -13443,7 +13440,7 @@
         <v>21</v>
       </c>
       <c r="O214" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="215" spans="1:15">
@@ -13451,16 +13448,16 @@
         <v>3</v>
       </c>
       <c r="B215" t="s">
+        <v>708</v>
+      </c>
+      <c r="C215" t="s">
         <v>709</v>
       </c>
-      <c r="C215" t="s">
-        <v>710</v>
-      </c>
       <c r="D215" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E215" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="F215" t="s">
         <v>557</v>
@@ -13490,7 +13487,7 @@
         <v>21</v>
       </c>
       <c r="O215" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
     </row>
     <row r="216" spans="1:15">
@@ -13498,13 +13495,13 @@
         <v>3</v>
       </c>
       <c r="B216" t="s">
+        <v>711</v>
+      </c>
+      <c r="C216" t="s">
         <v>712</v>
       </c>
-      <c r="C216" t="s">
+      <c r="D216" t="s">
         <v>713</v>
-      </c>
-      <c r="D216" t="s">
-        <v>714</v>
       </c>
       <c r="E216" t="s">
         <v>18</v>
@@ -13537,7 +13534,7 @@
         <v>21</v>
       </c>
       <c r="O216" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
     </row>
     <row r="217" spans="1:15">
@@ -13545,13 +13542,13 @@
         <v>3</v>
       </c>
       <c r="B217" t="s">
+        <v>715</v>
+      </c>
+      <c r="C217" t="s">
         <v>716</v>
       </c>
-      <c r="C217" t="s">
-        <v>717</v>
-      </c>
       <c r="D217" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="E217" t="s">
         <v>18</v>
@@ -13584,7 +13581,7 @@
         <v>21</v>
       </c>
       <c r="O217" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
     </row>
     <row r="218" spans="1:15">
@@ -13592,13 +13589,13 @@
         <v>3</v>
       </c>
       <c r="B218" t="s">
+        <v>717</v>
+      </c>
+      <c r="C218" t="s">
         <v>718</v>
       </c>
-      <c r="C218" t="s">
-        <v>719</v>
-      </c>
       <c r="D218" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="E218" t="s">
         <v>18</v>
@@ -13631,7 +13628,7 @@
         <v>21</v>
       </c>
       <c r="O218" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
     </row>
     <row r="219" spans="1:15">
@@ -13639,13 +13636,13 @@
         <v>3</v>
       </c>
       <c r="B219" t="s">
+        <v>719</v>
+      </c>
+      <c r="C219" t="s">
         <v>720</v>
       </c>
-      <c r="C219" t="s">
-        <v>721</v>
-      </c>
       <c r="D219" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="E219" t="s">
         <v>556</v>
@@ -13678,7 +13675,7 @@
         <v>21</v>
       </c>
       <c r="O219" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
     </row>
     <row r="220" spans="1:15">
@@ -13686,13 +13683,13 @@
         <v>3</v>
       </c>
       <c r="B220" t="s">
+        <v>721</v>
+      </c>
+      <c r="C220" t="s">
         <v>722</v>
       </c>
-      <c r="C220" t="s">
-        <v>723</v>
-      </c>
       <c r="D220" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="E220" t="s">
         <v>18</v>
@@ -13725,7 +13722,7 @@
         <v>21</v>
       </c>
       <c r="O220" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
     </row>
     <row r="221" spans="1:15">
@@ -13733,13 +13730,13 @@
         <v>3</v>
       </c>
       <c r="B221" t="s">
+        <v>723</v>
+      </c>
+      <c r="C221" t="s">
         <v>724</v>
       </c>
-      <c r="C221" t="s">
-        <v>725</v>
-      </c>
       <c r="D221" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="E221" t="s">
         <v>18</v>
@@ -13772,7 +13769,7 @@
         <v>21</v>
       </c>
       <c r="O221" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
     </row>
     <row r="222" spans="1:15">
@@ -13780,13 +13777,13 @@
         <v>3</v>
       </c>
       <c r="B222" t="s">
+        <v>725</v>
+      </c>
+      <c r="C222" t="s">
         <v>726</v>
       </c>
-      <c r="C222" t="s">
-        <v>727</v>
-      </c>
       <c r="D222" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="E222" t="s">
         <v>18</v>
@@ -13819,7 +13816,7 @@
         <v>21</v>
       </c>
       <c r="O222" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
     </row>
     <row r="223" spans="1:15">
@@ -13827,13 +13824,13 @@
         <v>3</v>
       </c>
       <c r="B223" t="s">
+        <v>727</v>
+      </c>
+      <c r="C223" t="s">
         <v>728</v>
       </c>
-      <c r="C223" t="s">
-        <v>729</v>
-      </c>
       <c r="D223" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="E223" t="s">
         <v>18</v>
@@ -13866,7 +13863,7 @@
         <v>21</v>
       </c>
       <c r="O223" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
     </row>
     <row r="224" spans="1:15">
@@ -13874,16 +13871,16 @@
         <v>3</v>
       </c>
       <c r="B224" t="s">
+        <v>729</v>
+      </c>
+      <c r="C224" t="s">
         <v>730</v>
       </c>
-      <c r="C224" t="s">
+      <c r="D224" t="s">
         <v>731</v>
       </c>
-      <c r="D224" t="s">
+      <c r="E224" t="s">
         <v>732</v>
-      </c>
-      <c r="E224" t="s">
-        <v>733</v>
       </c>
       <c r="F224" t="s">
         <v>19</v>
@@ -13913,7 +13910,7 @@
         <v>21</v>
       </c>
       <c r="O224" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
     </row>
     <row r="225" spans="1:15">
@@ -13921,13 +13918,13 @@
         <v>3</v>
       </c>
       <c r="B225" t="s">
+        <v>734</v>
+      </c>
+      <c r="C225" t="s">
         <v>735</v>
       </c>
-      <c r="C225" t="s">
+      <c r="D225" t="s">
         <v>736</v>
-      </c>
-      <c r="D225" t="s">
-        <v>737</v>
       </c>
       <c r="E225" t="s">
         <v>18</v>
@@ -13960,7 +13957,7 @@
         <v>21</v>
       </c>
       <c r="O225" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="226" spans="1:15">
@@ -13968,13 +13965,13 @@
         <v>3</v>
       </c>
       <c r="B226" t="s">
+        <v>738</v>
+      </c>
+      <c r="C226" t="s">
         <v>739</v>
       </c>
-      <c r="C226" t="s">
+      <c r="D226" t="s">
         <v>740</v>
-      </c>
-      <c r="D226" t="s">
-        <v>741</v>
       </c>
       <c r="E226" t="s">
         <v>165</v>
@@ -14007,7 +14004,7 @@
         <v>21</v>
       </c>
       <c r="O226" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="227" spans="1:15">
@@ -14015,16 +14012,16 @@
         <v>3</v>
       </c>
       <c r="B227" t="s">
+        <v>742</v>
+      </c>
+      <c r="C227" t="s">
         <v>743</v>
       </c>
-      <c r="C227" t="s">
+      <c r="D227" t="s">
         <v>744</v>
       </c>
-      <c r="D227" t="s">
-        <v>745</v>
-      </c>
       <c r="E227" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="F227" t="s">
         <v>19</v>
@@ -14054,7 +14051,7 @@
         <v>21</v>
       </c>
       <c r="O227" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
     </row>
     <row r="228" spans="1:15">
@@ -14062,13 +14059,13 @@
         <v>3</v>
       </c>
       <c r="B228" t="s">
+        <v>746</v>
+      </c>
+      <c r="C228" t="s">
         <v>747</v>
       </c>
-      <c r="C228" t="s">
+      <c r="D228" t="s">
         <v>748</v>
-      </c>
-      <c r="D228" t="s">
-        <v>749</v>
       </c>
       <c r="E228" t="s">
         <v>220</v>
@@ -14101,7 +14098,7 @@
         <v>21</v>
       </c>
       <c r="O228" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
     </row>
     <row r="229" spans="1:15">
@@ -14109,13 +14106,13 @@
         <v>3</v>
       </c>
       <c r="B229" t="s">
+        <v>750</v>
+      </c>
+      <c r="C229" t="s">
         <v>751</v>
       </c>
-      <c r="C229" t="s">
+      <c r="D229" t="s">
         <v>752</v>
-      </c>
-      <c r="D229" t="s">
-        <v>753</v>
       </c>
       <c r="E229" t="s">
         <v>165</v>
@@ -14148,7 +14145,7 @@
         <v>21</v>
       </c>
       <c r="O229" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
     </row>
     <row r="230" spans="1:15">
@@ -14156,16 +14153,16 @@
         <v>3</v>
       </c>
       <c r="B230" t="s">
+        <v>754</v>
+      </c>
+      <c r="C230" t="s">
         <v>755</v>
       </c>
-      <c r="C230" t="s">
+      <c r="D230" t="s">
         <v>756</v>
       </c>
-      <c r="D230" t="s">
+      <c r="E230" t="s">
         <v>757</v>
-      </c>
-      <c r="E230" t="s">
-        <v>758</v>
       </c>
       <c r="F230" t="s">
         <v>557</v>
@@ -14195,7 +14192,7 @@
         <v>21</v>
       </c>
       <c r="O230" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
     </row>
     <row r="231" spans="1:15">
@@ -14203,16 +14200,16 @@
         <v>3</v>
       </c>
       <c r="B231" t="s">
+        <v>759</v>
+      </c>
+      <c r="C231" t="s">
         <v>760</v>
       </c>
-      <c r="C231" t="s">
+      <c r="D231" t="s">
         <v>761</v>
       </c>
-      <c r="D231" t="s">
+      <c r="E231" t="s">
         <v>762</v>
-      </c>
-      <c r="E231" t="s">
-        <v>763</v>
       </c>
       <c r="F231" t="s">
         <v>19</v>
@@ -14242,7 +14239,7 @@
         <v>21</v>
       </c>
       <c r="O231" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
     </row>
     <row r="232" spans="1:15">
@@ -14250,16 +14247,16 @@
         <v>3</v>
       </c>
       <c r="B232" t="s">
+        <v>764</v>
+      </c>
+      <c r="C232" t="s">
         <v>765</v>
       </c>
-      <c r="C232" t="s">
-        <v>766</v>
-      </c>
       <c r="D232" t="s">
+        <v>761</v>
+      </c>
+      <c r="E232" t="s">
         <v>762</v>
-      </c>
-      <c r="E232" t="s">
-        <v>763</v>
       </c>
       <c r="F232" t="s">
         <v>19</v>
@@ -14289,7 +14286,7 @@
         <v>21</v>
       </c>
       <c r="O232" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
     </row>
     <row r="233" spans="1:15">
@@ -14297,16 +14294,16 @@
         <v>3</v>
       </c>
       <c r="B233" t="s">
+        <v>767</v>
+      </c>
+      <c r="C233" t="s">
         <v>768</v>
       </c>
-      <c r="C233" t="s">
-        <v>769</v>
-      </c>
       <c r="D233" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="E233" t="s">
-        <v>770</v>
+        <v>165</v>
       </c>
       <c r="F233" t="s">
         <v>19</v>
@@ -14336,7 +14333,7 @@
         <v>21</v>
       </c>
       <c r="O233" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
     </row>
     <row r="234" spans="1:15">
@@ -14344,16 +14341,16 @@
         <v>3</v>
       </c>
       <c r="B234" t="s">
+        <v>770</v>
+      </c>
+      <c r="C234" t="s">
+        <v>771</v>
+      </c>
+      <c r="D234" t="s">
+        <v>740</v>
+      </c>
+      <c r="E234" t="s">
         <v>772</v>
-      </c>
-      <c r="C234" t="s">
-        <v>773</v>
-      </c>
-      <c r="D234" t="s">
-        <v>741</v>
-      </c>
-      <c r="E234" t="s">
-        <v>770</v>
       </c>
       <c r="F234" t="s">
         <v>557</v>
@@ -14383,7 +14380,7 @@
         <v>21</v>
       </c>
       <c r="O234" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
     </row>
     <row r="235" spans="1:15">
@@ -14391,13 +14388,13 @@
         <v>3</v>
       </c>
       <c r="B235" t="s">
+        <v>774</v>
+      </c>
+      <c r="C235" t="s">
         <v>775</v>
       </c>
-      <c r="C235" t="s">
+      <c r="D235" t="s">
         <v>776</v>
-      </c>
-      <c r="D235" t="s">
-        <v>777</v>
       </c>
       <c r="E235" t="s">
         <v>18</v>
@@ -14430,7 +14427,7 @@
         <v>21</v>
       </c>
       <c r="O235" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
     </row>
     <row r="236" spans="1:15">
@@ -14438,13 +14435,13 @@
         <v>3</v>
       </c>
       <c r="B236" t="s">
+        <v>778</v>
+      </c>
+      <c r="C236" t="s">
         <v>779</v>
       </c>
-      <c r="C236" t="s">
-        <v>780</v>
-      </c>
       <c r="D236" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="E236" t="s">
         <v>18</v>
@@ -14477,7 +14474,7 @@
         <v>21</v>
       </c>
       <c r="O236" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
     </row>
     <row r="237" spans="1:15">
@@ -14485,13 +14482,13 @@
         <v>3</v>
       </c>
       <c r="B237" t="s">
+        <v>781</v>
+      </c>
+      <c r="C237" t="s">
         <v>782</v>
       </c>
-      <c r="C237" t="s">
-        <v>783</v>
-      </c>
       <c r="D237" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="E237" t="s">
         <v>220</v>
@@ -14524,7 +14521,7 @@
         <v>21</v>
       </c>
       <c r="O237" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert fix INRG (creava ticker duplicato); tieni solo WATC.PA
R174 (IE00B1XNHC34) era stata messa a INRG.MI, ma esiste gia' R208 con
ticker INRG.MI per un ISIN diverso (IE00B1W57M07 "Clean Energy Transition")
-> due righe stesso ticker = violazione idx_ticker. R174 torna a INRG.SW/USD
(coerente: e' la share class USD Dist). Da chiarire a parte quale listino EUR
corrisponde davvero a IE00B1XNHC34 e se R208 ha l'ISIN giusto.

WATC.SW -> WATC.PA (FR0014002CH1) resta: nessun conflitto, listino Parigi EUR
allineato a Directa.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HPsTcHPHNyTy55bZuN9KB6
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1903" uniqueCount="784">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1903" uniqueCount="785">
   <si>
     <t>Livello</t>
   </si>
@@ -1748,336 +1748,342 @@
     <t>IE00B1FZS350</t>
   </si>
   <si>
+    <t>INRG.SW</t>
+  </si>
+  <si>
+    <t>iShares Global Clean Energy UCITS ETF USD Dist</t>
+  </si>
+  <si>
+    <t>Svizzera</t>
+  </si>
+  <si>
+    <t>IE00B1XNHC34</t>
+  </si>
+  <si>
+    <t>XAIX.DE</t>
+  </si>
+  <si>
+    <t>Xtrackers Artificial Intelligence &amp; Big Data UCITS ETF</t>
+  </si>
+  <si>
+    <t>Settoriale - Tecnologia</t>
+  </si>
+  <si>
+    <t>IE00BGV5VN51</t>
+  </si>
+  <si>
+    <t>SXR2.DE</t>
+  </si>
+  <si>
+    <t>iShares MSCI Canada UCITS ETF USD Acc</t>
+  </si>
+  <si>
+    <t>Canada</t>
+  </si>
+  <si>
+    <t>IE00B52SF786</t>
+  </si>
+  <si>
+    <t>IQQI.DE</t>
+  </si>
+  <si>
+    <t>iShares Global Infrastructure UCITS ETF USD Dist</t>
+  </si>
+  <si>
+    <t>Infrastrutture</t>
+  </si>
+  <si>
+    <t>IE00B6QW5T61</t>
+  </si>
+  <si>
+    <t>IBGX.AS</t>
+  </si>
+  <si>
+    <t>iShares USD Treasury Bond 7-10yr UCITS ETF USD Dist</t>
+  </si>
+  <si>
+    <t>Obbligazionari - Governativi USD</t>
+  </si>
+  <si>
+    <t>IE00B1FZS681</t>
+  </si>
+  <si>
+    <t>IS3S.DE</t>
+  </si>
+  <si>
+    <t>iShares MSCI Europe Small Cap UCITS ETF EUR Acc</t>
+  </si>
+  <si>
+    <t>IE00B3VWMM18</t>
+  </si>
+  <si>
+    <t>WSML.L</t>
+  </si>
+  <si>
+    <t>iShares MSCI World Small Cap UCITS ETF USD (Acc)</t>
+  </si>
+  <si>
+    <t>IE00BDVWFV31</t>
+  </si>
+  <si>
+    <t>VHYL.MI</t>
+  </si>
+  <si>
+    <t>Vanguard FTSE All-World High Div Yield UCITS ETF</t>
+  </si>
+  <si>
+    <t>IE00B8GKDB10</t>
+  </si>
+  <si>
+    <t>HLTH.DE</t>
+  </si>
+  <si>
+    <t>SPDR MSCI Europe Health Care UCITS ETF</t>
+  </si>
+  <si>
+    <t>IE00BKWQ0H23</t>
+  </si>
+  <si>
+    <t>IWMO.L</t>
+  </si>
+  <si>
+    <t>iShares Edge MSCI World Momentum Factor UCITS ETF</t>
+  </si>
+  <si>
+    <t>IE00B0M63912</t>
+  </si>
+  <si>
+    <t>IWQU.L</t>
+  </si>
+  <si>
+    <t>iShares Edge MSCI World Quality Factor UCITS ETF</t>
+  </si>
+  <si>
+    <t>IE00B0M63961</t>
+  </si>
+  <si>
+    <t>MVOL.L</t>
+  </si>
+  <si>
+    <t>iShares Edge MSCI World Minimum Volatility UCITS ETF</t>
+  </si>
+  <si>
+    <t>IE00B0M63507</t>
+  </si>
+  <si>
+    <t>LTAM.MI</t>
+  </si>
+  <si>
+    <t>iShares MSCI EM Latin America UCITS ETF USD (Dist)</t>
+  </si>
+  <si>
+    <t>IE00B27YCK28</t>
+  </si>
+  <si>
+    <t>EMV.MI</t>
+  </si>
+  <si>
+    <t>iShares Edge MSCI EM Min Vol Factor UCITS ETF USD (Acc)</t>
+  </si>
+  <si>
+    <t>IE00B8KGV557</t>
+  </si>
+  <si>
+    <t>IS3T.DE</t>
+  </si>
+  <si>
+    <t>iShares MSCI World Mid-Cap Equal Weight UCITS ETF EUR</t>
+  </si>
+  <si>
+    <t>Azionario Mid Cap</t>
+  </si>
+  <si>
+    <t>IE00BP3QZD73</t>
+  </si>
+  <si>
+    <t>EMID.L</t>
+  </si>
+  <si>
+    <t>iShares MSCI Europe Mid Cap UCITS ETF EUR (Dist)</t>
+  </si>
+  <si>
+    <t>IE00BFXR5895</t>
+  </si>
+  <si>
+    <t>AIGI.MI</t>
+  </si>
+  <si>
+    <t>WisdomTree Industrial Metals ETC (Al+Cu+Zn+Ni+Pb)</t>
+  </si>
+  <si>
+    <t>Metalli Industriali</t>
+  </si>
+  <si>
+    <t>GB00B15KYG56</t>
+  </si>
+  <si>
+    <t>COPA.MI</t>
+  </si>
+  <si>
+    <t>WisdomTree Copper ETC</t>
+  </si>
+  <si>
+    <t>GB00B15KXQ89</t>
+  </si>
+  <si>
+    <t>ALUM.MI</t>
+  </si>
+  <si>
+    <t>WisdomTree Aluminium ETC</t>
+  </si>
+  <si>
+    <t>DE000A0Q4MJ7</t>
+  </si>
+  <si>
+    <t>ZINC.MI</t>
+  </si>
+  <si>
+    <t>WisdomTree Zinc ETC</t>
+  </si>
+  <si>
+    <t>DE000A0QLW44</t>
+  </si>
+  <si>
+    <t>COPM.MI</t>
+  </si>
+  <si>
+    <t>iShares Copper Miners UCITS ETF USD (Acc)</t>
+  </si>
+  <si>
+    <t>IE00063FT9K6</t>
+  </si>
+  <si>
+    <t>BATE.DE</t>
+  </si>
+  <si>
+    <t>L&amp;G Battery Value-Chain UCITS ETF</t>
+  </si>
+  <si>
+    <t>IE00BMDX3P59</t>
+  </si>
+  <si>
+    <t>IPRE.DE</t>
+  </si>
+  <si>
+    <t>iShares European Property Yield UCITS ETF EUR (Acc)</t>
+  </si>
+  <si>
+    <t>Private Equity</t>
+  </si>
+  <si>
+    <t>IE00BGDQ0L74</t>
+  </si>
+  <si>
+    <t>DX2G.DE</t>
+  </si>
+  <si>
+    <t>Xtrackers CAC 40 UCITS ETF 1D</t>
+  </si>
+  <si>
+    <t>LU0322250985</t>
+  </si>
+  <si>
+    <t>XEON.DE</t>
+  </si>
+  <si>
+    <t>Xtrackers II EUR Overnight Rate Swap UCITS ETF 1C</t>
+  </si>
+  <si>
+    <t>LU0290358497</t>
+  </si>
+  <si>
+    <t>IBGS.MI</t>
+  </si>
+  <si>
+    <t>iShares EUR Govt Bond 1-3yr UCITS ETF EUR (Dist)</t>
+  </si>
+  <si>
+    <t>Obbligazionari - Governativi EUR</t>
+  </si>
+  <si>
+    <t>IE00B14X4Q57</t>
+  </si>
+  <si>
+    <t>IUSE.L</t>
+  </si>
+  <si>
+    <t>iShares Core S&amp;P 500 UCITS ETF EUR Hedged (Acc)</t>
+  </si>
+  <si>
+    <t>IE00B3ZW0K18</t>
+  </si>
+  <si>
+    <t>IWDE.L</t>
+  </si>
+  <si>
+    <t>iShares MSCI World EUR Hedged UCITS ETF (Acc)</t>
+  </si>
+  <si>
+    <t>IE00B441G979</t>
+  </si>
+  <si>
+    <t>SGLD.MI</t>
+  </si>
+  <si>
+    <t>Invesco Physical Gold ETC</t>
+  </si>
+  <si>
+    <t>IE00B579F325</t>
+  </si>
+  <si>
+    <t>BTCN.AS</t>
+  </si>
+  <si>
+    <t>iShares Bitcoin ETP</t>
+  </si>
+  <si>
+    <t>XS2940466316</t>
+  </si>
+  <si>
+    <t>CMOD.MI</t>
+  </si>
+  <si>
+    <t>Invesco Bloomberg Commodity UCITS ETF</t>
+  </si>
+  <si>
+    <t>IE00BD6FVP32</t>
+  </si>
+  <si>
+    <t>XDWT.DE</t>
+  </si>
+  <si>
+    <t>Xtrackers MSCI World Information Technology UCITS ETF 1C</t>
+  </si>
+  <si>
+    <t>IE00BM67HT60</t>
+  </si>
+  <si>
+    <t>USPY.DE</t>
+  </si>
+  <si>
+    <t>L&amp;G Cyber Security UCITS ETF</t>
+  </si>
+  <si>
+    <t>IE00BYPLS672</t>
+  </si>
+  <si>
+    <t>AIFS.DE</t>
+  </si>
+  <si>
+    <t>iShares AI Infrastructure UCITS ETF</t>
+  </si>
+  <si>
+    <t>IE000V0H6AD4</t>
+  </si>
+  <si>
     <t>INRG.MI</t>
   </si>
   <si>
-    <t>iShares Global Clean Energy UCITS ETF USD Dist</t>
-  </si>
-  <si>
-    <t>IE00B1XNHC34</t>
-  </si>
-  <si>
-    <t>XAIX.DE</t>
-  </si>
-  <si>
-    <t>Xtrackers Artificial Intelligence &amp; Big Data UCITS ETF</t>
-  </si>
-  <si>
-    <t>Settoriale - Tecnologia</t>
-  </si>
-  <si>
-    <t>IE00BGV5VN51</t>
-  </si>
-  <si>
-    <t>SXR2.DE</t>
-  </si>
-  <si>
-    <t>iShares MSCI Canada UCITS ETF USD Acc</t>
-  </si>
-  <si>
-    <t>Canada</t>
-  </si>
-  <si>
-    <t>IE00B52SF786</t>
-  </si>
-  <si>
-    <t>IQQI.DE</t>
-  </si>
-  <si>
-    <t>iShares Global Infrastructure UCITS ETF USD Dist</t>
-  </si>
-  <si>
-    <t>Infrastrutture</t>
-  </si>
-  <si>
-    <t>IE00B6QW5T61</t>
-  </si>
-  <si>
-    <t>IBGX.AS</t>
-  </si>
-  <si>
-    <t>iShares USD Treasury Bond 7-10yr UCITS ETF USD Dist</t>
-  </si>
-  <si>
-    <t>Obbligazionari - Governativi USD</t>
-  </si>
-  <si>
-    <t>IE00B1FZS681</t>
-  </si>
-  <si>
-    <t>IS3S.DE</t>
-  </si>
-  <si>
-    <t>iShares MSCI Europe Small Cap UCITS ETF EUR Acc</t>
-  </si>
-  <si>
-    <t>IE00B3VWMM18</t>
-  </si>
-  <si>
-    <t>WSML.L</t>
-  </si>
-  <si>
-    <t>iShares MSCI World Small Cap UCITS ETF USD (Acc)</t>
-  </si>
-  <si>
-    <t>IE00BDVWFV31</t>
-  </si>
-  <si>
-    <t>VHYL.MI</t>
-  </si>
-  <si>
-    <t>Vanguard FTSE All-World High Div Yield UCITS ETF</t>
-  </si>
-  <si>
-    <t>IE00B8GKDB10</t>
-  </si>
-  <si>
-    <t>HLTH.DE</t>
-  </si>
-  <si>
-    <t>SPDR MSCI Europe Health Care UCITS ETF</t>
-  </si>
-  <si>
-    <t>IE00BKWQ0H23</t>
-  </si>
-  <si>
-    <t>IWMO.L</t>
-  </si>
-  <si>
-    <t>iShares Edge MSCI World Momentum Factor UCITS ETF</t>
-  </si>
-  <si>
-    <t>IE00B0M63912</t>
-  </si>
-  <si>
-    <t>IWQU.L</t>
-  </si>
-  <si>
-    <t>iShares Edge MSCI World Quality Factor UCITS ETF</t>
-  </si>
-  <si>
-    <t>IE00B0M63961</t>
-  </si>
-  <si>
-    <t>MVOL.L</t>
-  </si>
-  <si>
-    <t>iShares Edge MSCI World Minimum Volatility UCITS ETF</t>
-  </si>
-  <si>
-    <t>IE00B0M63507</t>
-  </si>
-  <si>
-    <t>LTAM.MI</t>
-  </si>
-  <si>
-    <t>iShares MSCI EM Latin America UCITS ETF USD (Dist)</t>
-  </si>
-  <si>
-    <t>IE00B27YCK28</t>
-  </si>
-  <si>
-    <t>EMV.MI</t>
-  </si>
-  <si>
-    <t>iShares Edge MSCI EM Min Vol Factor UCITS ETF USD (Acc)</t>
-  </si>
-  <si>
-    <t>IE00B8KGV557</t>
-  </si>
-  <si>
-    <t>IS3T.DE</t>
-  </si>
-  <si>
-    <t>iShares MSCI World Mid-Cap Equal Weight UCITS ETF EUR</t>
-  </si>
-  <si>
-    <t>Azionario Mid Cap</t>
-  </si>
-  <si>
-    <t>IE00BP3QZD73</t>
-  </si>
-  <si>
-    <t>EMID.L</t>
-  </si>
-  <si>
-    <t>iShares MSCI Europe Mid Cap UCITS ETF EUR (Dist)</t>
-  </si>
-  <si>
-    <t>IE00BFXR5895</t>
-  </si>
-  <si>
-    <t>AIGI.MI</t>
-  </si>
-  <si>
-    <t>WisdomTree Industrial Metals ETC (Al+Cu+Zn+Ni+Pb)</t>
-  </si>
-  <si>
-    <t>Metalli Industriali</t>
-  </si>
-  <si>
-    <t>GB00B15KYG56</t>
-  </si>
-  <si>
-    <t>COPA.MI</t>
-  </si>
-  <si>
-    <t>WisdomTree Copper ETC</t>
-  </si>
-  <si>
-    <t>GB00B15KXQ89</t>
-  </si>
-  <si>
-    <t>ALUM.MI</t>
-  </si>
-  <si>
-    <t>WisdomTree Aluminium ETC</t>
-  </si>
-  <si>
-    <t>DE000A0Q4MJ7</t>
-  </si>
-  <si>
-    <t>ZINC.MI</t>
-  </si>
-  <si>
-    <t>WisdomTree Zinc ETC</t>
-  </si>
-  <si>
-    <t>DE000A0QLW44</t>
-  </si>
-  <si>
-    <t>COPM.MI</t>
-  </si>
-  <si>
-    <t>iShares Copper Miners UCITS ETF USD (Acc)</t>
-  </si>
-  <si>
-    <t>IE00063FT9K6</t>
-  </si>
-  <si>
-    <t>BATE.DE</t>
-  </si>
-  <si>
-    <t>L&amp;G Battery Value-Chain UCITS ETF</t>
-  </si>
-  <si>
-    <t>IE00BMDX3P59</t>
-  </si>
-  <si>
-    <t>IPRE.DE</t>
-  </si>
-  <si>
-    <t>iShares European Property Yield UCITS ETF EUR (Acc)</t>
-  </si>
-  <si>
-    <t>Private Equity</t>
-  </si>
-  <si>
-    <t>IE00BGDQ0L74</t>
-  </si>
-  <si>
-    <t>DX2G.DE</t>
-  </si>
-  <si>
-    <t>Xtrackers CAC 40 UCITS ETF 1D</t>
-  </si>
-  <si>
-    <t>LU0322250985</t>
-  </si>
-  <si>
-    <t>XEON.DE</t>
-  </si>
-  <si>
-    <t>Xtrackers II EUR Overnight Rate Swap UCITS ETF 1C</t>
-  </si>
-  <si>
-    <t>LU0290358497</t>
-  </si>
-  <si>
-    <t>IBGS.MI</t>
-  </si>
-  <si>
-    <t>iShares EUR Govt Bond 1-3yr UCITS ETF EUR (Dist)</t>
-  </si>
-  <si>
-    <t>Obbligazionari - Governativi EUR</t>
-  </si>
-  <si>
-    <t>IE00B14X4Q57</t>
-  </si>
-  <si>
-    <t>IUSE.L</t>
-  </si>
-  <si>
-    <t>iShares Core S&amp;P 500 UCITS ETF EUR Hedged (Acc)</t>
-  </si>
-  <si>
-    <t>IE00B3ZW0K18</t>
-  </si>
-  <si>
-    <t>IWDE.L</t>
-  </si>
-  <si>
-    <t>iShares MSCI World EUR Hedged UCITS ETF (Acc)</t>
-  </si>
-  <si>
-    <t>IE00B441G979</t>
-  </si>
-  <si>
-    <t>SGLD.MI</t>
-  </si>
-  <si>
-    <t>Invesco Physical Gold ETC</t>
-  </si>
-  <si>
-    <t>IE00B579F325</t>
-  </si>
-  <si>
-    <t>BTCN.AS</t>
-  </si>
-  <si>
-    <t>iShares Bitcoin ETP</t>
-  </si>
-  <si>
-    <t>XS2940466316</t>
-  </si>
-  <si>
-    <t>CMOD.MI</t>
-  </si>
-  <si>
-    <t>Invesco Bloomberg Commodity UCITS ETF</t>
-  </si>
-  <si>
-    <t>IE00BD6FVP32</t>
-  </si>
-  <si>
-    <t>XDWT.DE</t>
-  </si>
-  <si>
-    <t>Xtrackers MSCI World Information Technology UCITS ETF 1C</t>
-  </si>
-  <si>
-    <t>IE00BM67HT60</t>
-  </si>
-  <si>
-    <t>USPY.DE</t>
-  </si>
-  <si>
-    <t>L&amp;G Cyber Security UCITS ETF</t>
-  </si>
-  <si>
-    <t>IE00BYPLS672</t>
-  </si>
-  <si>
-    <t>AIFS.DE</t>
-  </si>
-  <si>
-    <t>iShares AI Infrastructure UCITS ETF</t>
-  </si>
-  <si>
-    <t>IE000V0H6AD4</t>
-  </si>
-  <si>
     <t>iShares Global Clean Energy Transition UCITS ETF</t>
   </si>
   <si>
@@ -2343,9 +2349,6 @@
   </si>
   <si>
     <t>iShares VII PLC - iShares VII PLC - iShares $ Trea</t>
-  </si>
-  <si>
-    <t>Svizzera</t>
   </si>
   <si>
     <t>IE00B3VWN393</t>
@@ -11533,10 +11536,10 @@
         <v>46</v>
       </c>
       <c r="E174" t="s">
-        <v>18</v>
+        <v>575</v>
       </c>
       <c r="F174" t="s">
-        <v>19</v>
+        <v>557</v>
       </c>
       <c r="G174">
         <v>10.174</v>
@@ -11563,7 +11566,7 @@
         <v>21</v>
       </c>
       <c r="O174" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
     </row>
     <row r="175" spans="1:15">
@@ -11571,13 +11574,13 @@
         <v>3</v>
       </c>
       <c r="B175" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="C175" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="D175" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="E175" t="s">
         <v>220</v>
@@ -11610,7 +11613,7 @@
         <v>21</v>
       </c>
       <c r="O175" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
     </row>
     <row r="176" spans="1:15">
@@ -11618,13 +11621,13 @@
         <v>3</v>
       </c>
       <c r="B176" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C176" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="D176" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E176" t="s">
         <v>18</v>
@@ -11657,7 +11660,7 @@
         <v>21</v>
       </c>
       <c r="O176" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
     </row>
     <row r="177" spans="1:15">
@@ -11665,13 +11668,13 @@
         <v>3</v>
       </c>
       <c r="B177" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="C177" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D177" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="E177" t="s">
         <v>18</v>
@@ -11704,7 +11707,7 @@
         <v>21</v>
       </c>
       <c r="O177" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
     </row>
     <row r="178" spans="1:15">
@@ -11712,13 +11715,13 @@
         <v>3</v>
       </c>
       <c r="B178" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="C178" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="D178" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="E178" t="s">
         <v>18</v>
@@ -11751,7 +11754,7 @@
         <v>21</v>
       </c>
       <c r="O178" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
     </row>
     <row r="179" spans="1:15">
@@ -11759,10 +11762,10 @@
         <v>3</v>
       </c>
       <c r="B179" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="C179" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D179" t="s">
         <v>54</v>
@@ -11798,7 +11801,7 @@
         <v>21</v>
       </c>
       <c r="O179" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
     </row>
     <row r="180" spans="1:15">
@@ -11806,10 +11809,10 @@
         <v>3</v>
       </c>
       <c r="B180" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="C180" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="D180" t="s">
         <v>564</v>
@@ -11845,7 +11848,7 @@
         <v>21</v>
       </c>
       <c r="O180" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
     </row>
     <row r="181" spans="1:15">
@@ -11853,10 +11856,10 @@
         <v>3</v>
       </c>
       <c r="B181" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="C181" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="D181" t="s">
         <v>564</v>
@@ -11892,7 +11895,7 @@
         <v>21</v>
       </c>
       <c r="O181" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
     </row>
     <row r="182" spans="1:15">
@@ -11900,10 +11903,10 @@
         <v>3</v>
       </c>
       <c r="B182" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="C182" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="D182" t="s">
         <v>258</v>
@@ -11939,7 +11942,7 @@
         <v>21</v>
       </c>
       <c r="O182" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
     </row>
     <row r="183" spans="1:15">
@@ -11947,10 +11950,10 @@
         <v>3</v>
       </c>
       <c r="B183" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="C183" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="D183" t="s">
         <v>564</v>
@@ -11986,7 +11989,7 @@
         <v>21</v>
       </c>
       <c r="O183" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
     </row>
     <row r="184" spans="1:15">
@@ -11994,10 +11997,10 @@
         <v>3</v>
       </c>
       <c r="B184" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="C184" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="D184" t="s">
         <v>564</v>
@@ -12033,7 +12036,7 @@
         <v>21</v>
       </c>
       <c r="O184" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
     </row>
     <row r="185" spans="1:15">
@@ -12041,10 +12044,10 @@
         <v>3</v>
       </c>
       <c r="B185" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="C185" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="D185" t="s">
         <v>564</v>
@@ -12080,7 +12083,7 @@
         <v>21</v>
       </c>
       <c r="O185" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
     </row>
     <row r="186" spans="1:15">
@@ -12088,10 +12091,10 @@
         <v>2</v>
       </c>
       <c r="B186" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="C186" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="D186" t="s">
         <v>37</v>
@@ -12127,7 +12130,7 @@
         <v>21</v>
       </c>
       <c r="O186" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
     </row>
     <row r="187" spans="1:15">
@@ -12135,10 +12138,10 @@
         <v>3</v>
       </c>
       <c r="B187" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="C187" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="D187" t="s">
         <v>17</v>
@@ -12174,7 +12177,7 @@
         <v>21</v>
       </c>
       <c r="O187" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
     </row>
     <row r="188" spans="1:15">
@@ -12182,13 +12185,13 @@
         <v>3</v>
       </c>
       <c r="B188" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="C188" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="D188" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="E188" t="s">
         <v>220</v>
@@ -12221,7 +12224,7 @@
         <v>21</v>
       </c>
       <c r="O188" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
     </row>
     <row r="189" spans="1:15">
@@ -12229,13 +12232,13 @@
         <v>3</v>
       </c>
       <c r="B189" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="C189" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="D189" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="E189" t="s">
         <v>18</v>
@@ -12268,7 +12271,7 @@
         <v>21</v>
       </c>
       <c r="O189" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
     </row>
     <row r="190" spans="1:15">
@@ -12276,13 +12279,13 @@
         <v>3</v>
       </c>
       <c r="B190" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="C190" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D190" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="E190" t="s">
         <v>18</v>
@@ -12315,7 +12318,7 @@
         <v>21</v>
       </c>
       <c r="O190" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
     </row>
     <row r="191" spans="1:15">
@@ -12323,13 +12326,13 @@
         <v>3</v>
       </c>
       <c r="B191" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C191" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="D191" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="E191" t="s">
         <v>18</v>
@@ -12362,7 +12365,7 @@
         <v>21</v>
       </c>
       <c r="O191" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
     </row>
     <row r="192" spans="1:15">
@@ -12370,13 +12373,13 @@
         <v>3</v>
       </c>
       <c r="B192" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="C192" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="D192" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="E192" t="s">
         <v>18</v>
@@ -12409,7 +12412,7 @@
         <v>21</v>
       </c>
       <c r="O192" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
     </row>
     <row r="193" spans="1:15">
@@ -12417,13 +12420,13 @@
         <v>3</v>
       </c>
       <c r="B193" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="C193" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="D193" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="E193" t="s">
         <v>18</v>
@@ -12456,7 +12459,7 @@
         <v>21</v>
       </c>
       <c r="O193" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
     </row>
     <row r="194" spans="1:15">
@@ -12464,13 +12467,13 @@
         <v>3</v>
       </c>
       <c r="B194" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="C194" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D194" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="E194" t="s">
         <v>18</v>
@@ -12503,7 +12506,7 @@
         <v>21</v>
       </c>
       <c r="O194" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
     </row>
     <row r="195" spans="1:15">
@@ -12511,13 +12514,13 @@
         <v>3</v>
       </c>
       <c r="B195" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="C195" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="D195" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="E195" t="s">
         <v>220</v>
@@ -12550,7 +12553,7 @@
         <v>21</v>
       </c>
       <c r="O195" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
     </row>
     <row r="196" spans="1:15">
@@ -12558,13 +12561,13 @@
         <v>3</v>
       </c>
       <c r="B196" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="C196" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="D196" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="E196" t="s">
         <v>220</v>
@@ -12597,7 +12600,7 @@
         <v>21</v>
       </c>
       <c r="O196" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
     </row>
     <row r="197" spans="1:15">
@@ -12605,13 +12608,13 @@
         <v>3</v>
       </c>
       <c r="B197" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="C197" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="D197" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="E197" t="s">
         <v>220</v>
@@ -12644,7 +12647,7 @@
         <v>21</v>
       </c>
       <c r="O197" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
     </row>
     <row r="198" spans="1:15">
@@ -12652,10 +12655,10 @@
         <v>3</v>
       </c>
       <c r="B198" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="C198" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="D198" t="s">
         <v>409</v>
@@ -12691,7 +12694,7 @@
         <v>21</v>
       </c>
       <c r="O198" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
     </row>
     <row r="199" spans="1:15">
@@ -12699,13 +12702,13 @@
         <v>3</v>
       </c>
       <c r="B199" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C199" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="D199" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="E199" t="s">
         <v>18</v>
@@ -12738,7 +12741,7 @@
         <v>21</v>
       </c>
       <c r="O199" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
     </row>
     <row r="200" spans="1:15">
@@ -12746,10 +12749,10 @@
         <v>3</v>
       </c>
       <c r="B200" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="C200" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="D200" t="s">
         <v>50</v>
@@ -12785,7 +12788,7 @@
         <v>21</v>
       </c>
       <c r="O200" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="201" spans="1:15">
@@ -12793,10 +12796,10 @@
         <v>3</v>
       </c>
       <c r="B201" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="C201" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="D201" t="s">
         <v>564</v>
@@ -12832,7 +12835,7 @@
         <v>21</v>
       </c>
       <c r="O201" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
     </row>
     <row r="202" spans="1:15">
@@ -12840,10 +12843,10 @@
         <v>3</v>
       </c>
       <c r="B202" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="C202" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="D202" t="s">
         <v>555</v>
@@ -12879,7 +12882,7 @@
         <v>21</v>
       </c>
       <c r="O202" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
     </row>
     <row r="203" spans="1:15">
@@ -12887,13 +12890,13 @@
         <v>3</v>
       </c>
       <c r="B203" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="C203" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="D203" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="E203" t="s">
         <v>18</v>
@@ -12926,7 +12929,7 @@
         <v>21</v>
       </c>
       <c r="O203" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
     </row>
     <row r="204" spans="1:15">
@@ -12934,10 +12937,10 @@
         <v>3</v>
       </c>
       <c r="B204" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="C204" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="D204" t="s">
         <v>110</v>
@@ -12973,7 +12976,7 @@
         <v>21</v>
       </c>
       <c r="O204" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
     </row>
     <row r="205" spans="1:15">
@@ -12981,13 +12984,13 @@
         <v>3</v>
       </c>
       <c r="B205" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="C205" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="D205" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="E205" t="s">
         <v>220</v>
@@ -13020,7 +13023,7 @@
         <v>21</v>
       </c>
       <c r="O205" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
     </row>
     <row r="206" spans="1:15">
@@ -13028,13 +13031,13 @@
         <v>3</v>
       </c>
       <c r="B206" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="C206" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="D206" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="E206" t="s">
         <v>220</v>
@@ -13067,7 +13070,7 @@
         <v>21</v>
       </c>
       <c r="O206" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
     </row>
     <row r="207" spans="1:15">
@@ -13075,13 +13078,13 @@
         <v>3</v>
       </c>
       <c r="B207" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="C207" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="D207" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="E207" t="s">
         <v>220</v>
@@ -13114,7 +13117,7 @@
         <v>21</v>
       </c>
       <c r="O207" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
     </row>
     <row r="208" spans="1:15">
@@ -13122,10 +13125,10 @@
         <v>3</v>
       </c>
       <c r="B208" t="s">
-        <v>573</v>
+        <v>684</v>
       </c>
       <c r="C208" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="D208" t="s">
         <v>46</v>
@@ -13161,7 +13164,7 @@
         <v>21</v>
       </c>
       <c r="O208" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
     </row>
     <row r="209" spans="1:15">
@@ -13169,10 +13172,10 @@
         <v>3</v>
       </c>
       <c r="B209" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="C209" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="D209" t="s">
         <v>555</v>
@@ -13208,7 +13211,7 @@
         <v>21</v>
       </c>
       <c r="O209" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
     </row>
     <row r="210" spans="1:15">
@@ -13216,13 +13219,13 @@
         <v>3</v>
       </c>
       <c r="B210" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="C210" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="D210" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="E210" t="s">
         <v>18</v>
@@ -13255,7 +13258,7 @@
         <v>21</v>
       </c>
       <c r="O210" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
     </row>
     <row r="211" spans="1:15">
@@ -13263,19 +13266,19 @@
         <v>3</v>
       </c>
       <c r="B211" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="C211" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="D211" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="E211" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="F211" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="G211">
         <v>61.09</v>
@@ -13302,7 +13305,7 @@
         <v>21</v>
       </c>
       <c r="O211" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
     </row>
     <row r="212" spans="1:15">
@@ -13310,19 +13313,19 @@
         <v>3</v>
       </c>
       <c r="B212" t="s">
+        <v>700</v>
+      </c>
+      <c r="C212" t="s">
+        <v>701</v>
+      </c>
+      <c r="D212" t="s">
+        <v>696</v>
+      </c>
+      <c r="E212" t="s">
+        <v>697</v>
+      </c>
+      <c r="F212" t="s">
         <v>698</v>
-      </c>
-      <c r="C212" t="s">
-        <v>699</v>
-      </c>
-      <c r="D212" t="s">
-        <v>694</v>
-      </c>
-      <c r="E212" t="s">
-        <v>695</v>
-      </c>
-      <c r="F212" t="s">
-        <v>696</v>
       </c>
       <c r="G212">
         <v>61.08</v>
@@ -13349,7 +13352,7 @@
         <v>21</v>
       </c>
       <c r="O212" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
     </row>
     <row r="213" spans="1:15">
@@ -13357,19 +13360,19 @@
         <v>2</v>
       </c>
       <c r="B213" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="C213" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="D213" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="E213" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="F213" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="G213">
         <v>9.262</v>
@@ -13393,7 +13396,7 @@
         <v>21</v>
       </c>
       <c r="O213" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
     </row>
     <row r="214" spans="1:15">
@@ -13401,16 +13404,16 @@
         <v>3</v>
       </c>
       <c r="B214" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="C214" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="D214" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="E214" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="F214" t="s">
         <v>19</v>
@@ -13440,7 +13443,7 @@
         <v>21</v>
       </c>
       <c r="O214" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
     </row>
     <row r="215" spans="1:15">
@@ -13448,16 +13451,16 @@
         <v>3</v>
       </c>
       <c r="B215" t="s">
+        <v>710</v>
+      </c>
+      <c r="C215" t="s">
+        <v>711</v>
+      </c>
+      <c r="D215" t="s">
+        <v>696</v>
+      </c>
+      <c r="E215" t="s">
         <v>708</v>
-      </c>
-      <c r="C215" t="s">
-        <v>709</v>
-      </c>
-      <c r="D215" t="s">
-        <v>694</v>
-      </c>
-      <c r="E215" t="s">
-        <v>706</v>
       </c>
       <c r="F215" t="s">
         <v>557</v>
@@ -13487,7 +13490,7 @@
         <v>21</v>
       </c>
       <c r="O215" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
     </row>
     <row r="216" spans="1:15">
@@ -13495,13 +13498,13 @@
         <v>3</v>
       </c>
       <c r="B216" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="C216" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="D216" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="E216" t="s">
         <v>18</v>
@@ -13534,7 +13537,7 @@
         <v>21</v>
       </c>
       <c r="O216" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
     </row>
     <row r="217" spans="1:15">
@@ -13542,13 +13545,13 @@
         <v>3</v>
       </c>
       <c r="B217" t="s">
+        <v>717</v>
+      </c>
+      <c r="C217" t="s">
+        <v>718</v>
+      </c>
+      <c r="D217" t="s">
         <v>715</v>
-      </c>
-      <c r="C217" t="s">
-        <v>716</v>
-      </c>
-      <c r="D217" t="s">
-        <v>713</v>
       </c>
       <c r="E217" t="s">
         <v>18</v>
@@ -13581,7 +13584,7 @@
         <v>21</v>
       </c>
       <c r="O217" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
     </row>
     <row r="218" spans="1:15">
@@ -13589,13 +13592,13 @@
         <v>3</v>
       </c>
       <c r="B218" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="C218" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="D218" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="E218" t="s">
         <v>18</v>
@@ -13628,7 +13631,7 @@
         <v>21</v>
       </c>
       <c r="O218" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
     </row>
     <row r="219" spans="1:15">
@@ -13636,13 +13639,13 @@
         <v>3</v>
       </c>
       <c r="B219" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="C219" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="D219" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="E219" t="s">
         <v>556</v>
@@ -13675,7 +13678,7 @@
         <v>21</v>
       </c>
       <c r="O219" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
     </row>
     <row r="220" spans="1:15">
@@ -13683,13 +13686,13 @@
         <v>3</v>
       </c>
       <c r="B220" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="C220" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="D220" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="E220" t="s">
         <v>18</v>
@@ -13722,7 +13725,7 @@
         <v>21</v>
       </c>
       <c r="O220" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
     </row>
     <row r="221" spans="1:15">
@@ -13730,13 +13733,13 @@
         <v>3</v>
       </c>
       <c r="B221" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="C221" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="D221" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="E221" t="s">
         <v>18</v>
@@ -13769,7 +13772,7 @@
         <v>21</v>
       </c>
       <c r="O221" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
     </row>
     <row r="222" spans="1:15">
@@ -13777,13 +13780,13 @@
         <v>3</v>
       </c>
       <c r="B222" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="C222" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="D222" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="E222" t="s">
         <v>18</v>
@@ -13816,7 +13819,7 @@
         <v>21</v>
       </c>
       <c r="O222" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
     </row>
     <row r="223" spans="1:15">
@@ -13824,13 +13827,13 @@
         <v>3</v>
       </c>
       <c r="B223" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="C223" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="D223" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="E223" t="s">
         <v>18</v>
@@ -13863,7 +13866,7 @@
         <v>21</v>
       </c>
       <c r="O223" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
     </row>
     <row r="224" spans="1:15">
@@ -13871,16 +13874,16 @@
         <v>3</v>
       </c>
       <c r="B224" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="C224" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="D224" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="E224" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="F224" t="s">
         <v>19</v>
@@ -13910,7 +13913,7 @@
         <v>21</v>
       </c>
       <c r="O224" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
     </row>
     <row r="225" spans="1:15">
@@ -13918,13 +13921,13 @@
         <v>3</v>
       </c>
       <c r="B225" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="C225" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="D225" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="E225" t="s">
         <v>18</v>
@@ -13957,7 +13960,7 @@
         <v>21</v>
       </c>
       <c r="O225" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
     </row>
     <row r="226" spans="1:15">
@@ -13965,13 +13968,13 @@
         <v>3</v>
       </c>
       <c r="B226" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="C226" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="D226" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="E226" t="s">
         <v>165</v>
@@ -14004,7 +14007,7 @@
         <v>21</v>
       </c>
       <c r="O226" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
     </row>
     <row r="227" spans="1:15">
@@ -14012,16 +14015,16 @@
         <v>3</v>
       </c>
       <c r="B227" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="C227" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="D227" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="E227" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="F227" t="s">
         <v>19</v>
@@ -14051,7 +14054,7 @@
         <v>21</v>
       </c>
       <c r="O227" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
     </row>
     <row r="228" spans="1:15">
@@ -14059,13 +14062,13 @@
         <v>3</v>
       </c>
       <c r="B228" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="C228" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="D228" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="E228" t="s">
         <v>220</v>
@@ -14098,7 +14101,7 @@
         <v>21</v>
       </c>
       <c r="O228" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
     </row>
     <row r="229" spans="1:15">
@@ -14106,13 +14109,13 @@
         <v>3</v>
       </c>
       <c r="B229" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="C229" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="D229" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="E229" t="s">
         <v>165</v>
@@ -14145,7 +14148,7 @@
         <v>21</v>
       </c>
       <c r="O229" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
     </row>
     <row r="230" spans="1:15">
@@ -14153,16 +14156,16 @@
         <v>3</v>
       </c>
       <c r="B230" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="C230" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="D230" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="E230" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="F230" t="s">
         <v>557</v>
@@ -14192,7 +14195,7 @@
         <v>21</v>
       </c>
       <c r="O230" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
     </row>
     <row r="231" spans="1:15">
@@ -14200,16 +14203,16 @@
         <v>3</v>
       </c>
       <c r="B231" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="C231" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="D231" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
       <c r="E231" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="F231" t="s">
         <v>19</v>
@@ -14239,7 +14242,7 @@
         <v>21</v>
       </c>
       <c r="O231" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
     </row>
     <row r="232" spans="1:15">
@@ -14247,16 +14250,16 @@
         <v>3</v>
       </c>
       <c r="B232" t="s">
+        <v>766</v>
+      </c>
+      <c r="C232" t="s">
+        <v>767</v>
+      </c>
+      <c r="D232" t="s">
+        <v>763</v>
+      </c>
+      <c r="E232" t="s">
         <v>764</v>
-      </c>
-      <c r="C232" t="s">
-        <v>765</v>
-      </c>
-      <c r="D232" t="s">
-        <v>761</v>
-      </c>
-      <c r="E232" t="s">
-        <v>762</v>
       </c>
       <c r="F232" t="s">
         <v>19</v>
@@ -14286,7 +14289,7 @@
         <v>21</v>
       </c>
       <c r="O232" t="s">
-        <v>766</v>
+        <v>768</v>
       </c>
     </row>
     <row r="233" spans="1:15">
@@ -14294,13 +14297,13 @@
         <v>3</v>
       </c>
       <c r="B233" t="s">
-        <v>767</v>
+        <v>769</v>
       </c>
       <c r="C233" t="s">
-        <v>768</v>
+        <v>770</v>
       </c>
       <c r="D233" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="E233" t="s">
         <v>165</v>
@@ -14333,7 +14336,7 @@
         <v>21</v>
       </c>
       <c r="O233" t="s">
-        <v>769</v>
+        <v>771</v>
       </c>
     </row>
     <row r="234" spans="1:15">
@@ -14341,16 +14344,16 @@
         <v>3</v>
       </c>
       <c r="B234" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="C234" t="s">
-        <v>771</v>
+        <v>773</v>
       </c>
       <c r="D234" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="E234" t="s">
-        <v>772</v>
+        <v>575</v>
       </c>
       <c r="F234" t="s">
         <v>557</v>
@@ -14380,7 +14383,7 @@
         <v>21</v>
       </c>
       <c r="O234" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
     </row>
     <row r="235" spans="1:15">
@@ -14388,13 +14391,13 @@
         <v>3</v>
       </c>
       <c r="B235" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="C235" t="s">
-        <v>775</v>
+        <v>776</v>
       </c>
       <c r="D235" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="E235" t="s">
         <v>18</v>
@@ -14427,7 +14430,7 @@
         <v>21</v>
       </c>
       <c r="O235" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
     </row>
     <row r="236" spans="1:15">
@@ -14435,13 +14438,13 @@
         <v>3</v>
       </c>
       <c r="B236" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="C236" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="D236" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="E236" t="s">
         <v>18</v>
@@ -14474,7 +14477,7 @@
         <v>21</v>
       </c>
       <c r="O236" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
     </row>
     <row r="237" spans="1:15">
@@ -14482,13 +14485,13 @@
         <v>3</v>
       </c>
       <c r="B237" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="C237" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
       <c r="D237" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="E237" t="s">
         <v>220</v>
@@ -14521,7 +14524,7 @@
         <v>21</v>
       </c>
       <c r="O237" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
etf: 3MIB.MI (GraniteShares, delistato) -> 3ITL.MI (WisdomTree FTSE MIB 3x, rebrand post-acquisizione)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01WGAuRwCqWvHwxtYhtZkFxQ
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ETF" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ETF" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -15122,12 +15122,12 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>3MIB.MI</t>
+          <t>3ITL.MI</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>GraniteShares 3x Long FTSE MIB Daily ETP</t>
+          <t>WisdomTree FTSE MIB 3x Daily Leveraged</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">

</xml_diff>

<commit_message>
fix ticker+ISIN BATE.DE->BATT.MI, AIFS.DE->AINF.MI (verificati su Directa + Yahoo)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UWycesgje3BJc12FLmMZTJ
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -16271,7 +16271,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>BATE.DE</t>
+          <t>BATT.MI</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -16324,7 +16324,7 @@
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>IE00BMDX3P59</t>
+          <t>IE00BF0M2Z96</t>
         </is>
       </c>
       <c r="P195" t="inlineStr">
@@ -17207,7 +17207,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>AIFS.DE</t>
+          <t>AINF.MI</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -17260,7 +17260,7 @@
       </c>
       <c r="O207" t="inlineStr">
         <is>
-          <t>IE000V0H6AD4</t>
+          <t>IE000X59ZHE2</t>
         </is>
       </c>
       <c r="P207" t="inlineStr">

</xml_diff>

<commit_message>
PAC: fix plan start_dates (5 ETF started 08/09 not 01/09) + memory sync
- XMAE/DAPP/GBSE/HLT/GOAI start_date -> 2026-09-08 (only VWCE+GAGG ran on 01/09,
  old 2-ETF plan). Prevents _process_pac_plans inventing phantom 01/09 buys.
- Deleted 3 phantom auto rows. DB back to 9 real executions, 1217.94EUR.
- xlsx: monitor refresh incl. the 3 new PAC ETFs with live prices.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ETF" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ETF" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -19653,7 +19653,6 @@
           <t>L3</t>
         </is>
       </c>
-      <c r="N238" t="inlineStr"/>
       <c r="O238" t="inlineStr">
         <is>
           <t>IE00BMDKNW35</t>
@@ -19709,7 +19708,6 @@
           <t>L3</t>
         </is>
       </c>
-      <c r="N239" t="inlineStr"/>
       <c r="O239" t="inlineStr">
         <is>
           <t>IE000VXC51U5</t>
@@ -19765,7 +19763,6 @@
           <t>L3</t>
         </is>
       </c>
-      <c r="N240" t="inlineStr"/>
       <c r="O240" t="inlineStr">
         <is>
           <t>JE00B8DFY052</t>

</xml_diff>